<commit_message>
update E2E test plan: Status column now auto-calculates PASS/FAIL based on Actual vs Expected results
</commit_message>
<xml_diff>
--- a/docs/plans/Nutrio-Fuel-E2E-Test-Plan.xlsx
+++ b/docs/plans/Nutrio-Fuel-E2E-Test-Plan.xlsx
@@ -577,10 +577,7 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -625,10 +622,7 @@
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -665,7 +659,6 @@
           <t>Test Date</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -673,7 +666,6 @@
           <t>Tester Name</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -681,7 +673,6 @@
           <t>Browser</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -689,7 +680,6 @@
           <t>Device</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -697,7 +687,6 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -831,7 +820,10 @@
           <t>User logged in and redirected to dashboard</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr"/>
+      <c r="H2" s="5">
+        <f>IF(I2="","",IF(I2=G2,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I2" s="5" t="inlineStr"/>
       <c r="J2" s="5" t="inlineStr"/>
       <c r="K2" s="6" t="inlineStr">
@@ -880,7 +872,10 @@
           <t>Error message: Invalid credentials</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr"/>
+      <c r="H3" s="5">
+        <f>IF(I3="","",IF(I3=G3,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I3" s="5" t="inlineStr"/>
       <c r="J3" s="5" t="inlineStr"/>
       <c r="K3" s="6" t="inlineStr">
@@ -930,7 +925,10 @@
           <t>Account created successfully, verification email sent</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr"/>
+      <c r="H4" s="5">
+        <f>IF(I4="","",IF(I4=G4,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I4" s="5" t="inlineStr"/>
       <c r="J4" s="5" t="inlineStr"/>
       <c r="K4" s="6" t="inlineStr">
@@ -981,7 +979,10 @@
           <t>Password reset successful, can login with new password</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
+      <c r="H5" s="5">
+        <f>IF(I5="","",IF(I5=G5,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr">
@@ -1028,7 +1029,10 @@
           <t>User logged out, redirected to login page</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr"/>
+      <c r="H6" s="5">
+        <f>IF(I6="","",IF(I6=G6,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr"/>
       <c r="K6" s="6" t="inlineStr">
@@ -1075,7 +1079,10 @@
           <t>Dashboard loads with subscription info, meals remaining, recent orders</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
+      <c r="H7" s="5">
+        <f>IF(I7="","",IF(I7=G7,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="5" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr">
@@ -1122,7 +1129,10 @@
           <t>All links navigate to correct pages</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
+      <c r="H8" s="5">
+        <f>IF(I8="","",IF(I8=G8,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr"/>
       <c r="K8" s="6" t="inlineStr">
@@ -1171,7 +1181,10 @@
           <t>Each button performs correct action</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr"/>
+      <c r="H9" s="5">
+        <f>IF(I9="","",IF(I9=G9,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr">
@@ -1218,7 +1231,10 @@
           <t>All plans displayed with correct pricing and features</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr"/>
+      <c r="H10" s="5">
+        <f>IF(I10="","",IF(I10=G10,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I10" s="5" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="6" t="inlineStr">
@@ -1267,7 +1283,10 @@
           <t>Subscription activated, meals allocated</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr"/>
+      <c r="H11" s="5">
+        <f>IF(I11="","",IF(I11=G11,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr"/>
       <c r="K11" s="6" t="inlineStr">
@@ -1315,7 +1334,10 @@
           <t>Subscription activated with 10 meals/week</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr"/>
+      <c r="H12" s="5">
+        <f>IF(I12="","",IF(I12=G12,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I12" s="5" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr"/>
       <c r="K12" s="6" t="inlineStr">
@@ -1362,7 +1384,10 @@
           <t>Subscription activated with 15 meals/week</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="H13" s="5">
+        <f>IF(I13="","",IF(I13=G13,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr"/>
       <c r="K13" s="6" t="inlineStr">
@@ -1409,7 +1434,10 @@
           <t>Subscription activated with unlimited meals</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr"/>
+      <c r="H14" s="5">
+        <f>IF(I14="","",IF(I14=G14,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I14" s="5" t="inlineStr"/>
       <c r="J14" s="5" t="inlineStr"/>
       <c r="K14" s="6" t="inlineStr">
@@ -1458,7 +1486,10 @@
           <t>Plan upgraded, new meal limit applied</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr"/>
+      <c r="H15" s="5">
+        <f>IF(I15="","",IF(I15=G15,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I15" s="5" t="inlineStr"/>
       <c r="J15" s="5" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr">
@@ -1506,7 +1537,10 @@
           <t>Plan downgraded effective next billing cycle</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr"/>
+      <c r="H16" s="5">
+        <f>IF(I16="","",IF(I16=G16,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I16" s="5" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr">
@@ -1554,7 +1588,10 @@
           <t>Subscription paused, no new orders possible</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr"/>
+      <c r="H17" s="5">
+        <f>IF(I17="","",IF(I17=G17,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr"/>
       <c r="K17" s="7" t="inlineStr">
@@ -1602,7 +1639,10 @@
           <t>Subscription resumed, can order again</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr"/>
+      <c r="H18" s="5">
+        <f>IF(I18="","",IF(I18=G18,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I18" s="5" t="inlineStr"/>
       <c r="J18" s="5" t="inlineStr"/>
       <c r="K18" s="7" t="inlineStr">
@@ -1650,7 +1690,10 @@
           <t>Subscription cancelled, access until end date</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr"/>
+      <c r="H19" s="5">
+        <f>IF(I19="","",IF(I19=G19,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I19" s="5" t="inlineStr"/>
       <c r="J19" s="5" t="inlineStr"/>
       <c r="K19" s="7" t="inlineStr">
@@ -1697,7 +1740,10 @@
           <t>Correct number of meals remaining displayed</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr"/>
+      <c r="H20" s="5">
+        <f>IF(I20="","",IF(I20=G20,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I20" s="5" t="inlineStr"/>
       <c r="J20" s="5" t="inlineStr"/>
       <c r="K20" s="6" t="inlineStr">
@@ -1744,7 +1790,10 @@
           <t>All available meals displayed with images, names, restaurants</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr"/>
+      <c r="H21" s="5">
+        <f>IF(I21="","",IF(I21=G21,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I21" s="5" t="inlineStr"/>
       <c r="J21" s="5" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr">
@@ -1792,7 +1841,10 @@
           <t>Only meals from selected restaurant displayed</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr"/>
+      <c r="H22" s="5">
+        <f>IF(I22="","",IF(I22=G22,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I22" s="5" t="inlineStr"/>
       <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="6" t="inlineStr">
@@ -1840,7 +1892,10 @@
           <t>Only keto meals displayed</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr"/>
+      <c r="H23" s="5">
+        <f>IF(I23="","",IF(I23=G23,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I23" s="5" t="inlineStr"/>
       <c r="J23" s="5" t="inlineStr"/>
       <c r="K23" s="6" t="inlineStr">
@@ -1888,7 +1943,10 @@
           <t>Meals within calorie range displayed</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr"/>
+      <c r="H24" s="5">
+        <f>IF(I24="","",IF(I24=G24,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I24" s="5" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr"/>
       <c r="K24" s="7" t="inlineStr">
@@ -1935,7 +1993,10 @@
           <t>Search results displayed matching query</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr"/>
+      <c r="H25" s="5">
+        <f>IF(I25="","",IF(I25=G25,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I25" s="5" t="inlineStr"/>
       <c r="J25" s="5" t="inlineStr"/>
       <c r="K25" s="6" t="inlineStr">
@@ -1982,7 +2043,10 @@
           <t>Full meal info displayed: ingredients, nutrition, prep time, restaurant</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr"/>
+      <c r="H26" s="5">
+        <f>IF(I26="","",IF(I26=G26,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I26" s="5" t="inlineStr"/>
       <c r="J26" s="5" t="inlineStr"/>
       <c r="K26" s="6" t="inlineStr">
@@ -2030,7 +2094,10 @@
           <t>Meal added to cart, confirmation shown</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr"/>
+      <c r="H27" s="5">
+        <f>IF(I27="","",IF(I27=G27,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I27" s="5" t="inlineStr"/>
       <c r="J27" s="5" t="inlineStr"/>
       <c r="K27" s="6" t="inlineStr">
@@ -2077,7 +2144,10 @@
           <t>'Add to Order' button disabled or warning shown</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr"/>
+      <c r="H28" s="5">
+        <f>IF(I28="","",IF(I28=G28,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I28" s="5" t="inlineStr"/>
       <c r="J28" s="5" t="inlineStr"/>
       <c r="K28" s="6" t="inlineStr">
@@ -2124,7 +2194,10 @@
           <t>Meal appears in favorites list</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr"/>
+      <c r="H29" s="5">
+        <f>IF(I29="","",IF(I29=G29,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I29" s="5" t="inlineStr"/>
       <c r="J29" s="5" t="inlineStr"/>
       <c r="K29" s="5" t="inlineStr">
@@ -2173,7 +2246,10 @@
           <t>Order placed successfully, confirmation shown</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr"/>
+      <c r="H30" s="5">
+        <f>IF(I30="","",IF(I30=G30,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I30" s="5" t="inlineStr"/>
       <c r="J30" s="5" t="inlineStr"/>
       <c r="K30" s="8" t="inlineStr">
@@ -2220,7 +2296,10 @@
           <t>All past orders displayed with status</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr"/>
+      <c r="H31" s="5">
+        <f>IF(I31="","",IF(I31=G31,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I31" s="5" t="inlineStr"/>
       <c r="J31" s="5" t="inlineStr"/>
       <c r="K31" s="6" t="inlineStr">
@@ -2267,7 +2346,10 @@
           <t>Full order info: items, status, restaurant, total</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr"/>
+      <c r="H32" s="5">
+        <f>IF(I32="","",IF(I32=G32,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I32" s="5" t="inlineStr"/>
       <c r="J32" s="5" t="inlineStr"/>
       <c r="K32" s="6" t="inlineStr">
@@ -2314,7 +2396,10 @@
           <t>Current status and history displayed</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr"/>
+      <c r="H33" s="5">
+        <f>IF(I33="","",IF(I33=G33,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I33" s="5" t="inlineStr"/>
       <c r="J33" s="5" t="inlineStr"/>
       <c r="K33" s="6" t="inlineStr">
@@ -2362,7 +2447,10 @@
           <t>Order cancelled, meals refunded to weekly limit</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr"/>
+      <c r="H34" s="5">
+        <f>IF(I34="","",IF(I34=G34,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I34" s="5" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr"/>
       <c r="K34" s="7" t="inlineStr">
@@ -2411,7 +2499,10 @@
           <t>Rating submitted, thank you message shown</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr"/>
+      <c r="H35" s="5">
+        <f>IF(I35="","",IF(I35=G35,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I35" s="5" t="inlineStr"/>
       <c r="J35" s="5" t="inlineStr"/>
       <c r="K35" s="7" t="inlineStr">
@@ -2459,7 +2550,10 @@
           <t>Items added to cart, can modify before checkout</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr"/>
+      <c r="H36" s="5">
+        <f>IF(I36="","",IF(I36=G36,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I36" s="5" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr"/>
       <c r="K36" s="7" t="inlineStr">
@@ -2506,7 +2600,10 @@
           <t>Profile info displayed: name, email, subscription, referral code</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr"/>
+      <c r="H37" s="5">
+        <f>IF(I37="","",IF(I37=G37,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I37" s="5" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr"/>
       <c r="K37" s="6" t="inlineStr">
@@ -2555,7 +2652,10 @@
           <t>Profile updated successfully</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr"/>
+      <c r="H38" s="5">
+        <f>IF(I38="","",IF(I38=G38,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I38" s="5" t="inlineStr"/>
       <c r="J38" s="5" t="inlineStr"/>
       <c r="K38" s="7" t="inlineStr">
@@ -2604,7 +2704,10 @@
           <t>Password changed, confirmation shown</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr"/>
+      <c r="H39" s="5">
+        <f>IF(I39="","",IF(I39=G39,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I39" s="5" t="inlineStr"/>
       <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="7" t="inlineStr">
@@ -2653,7 +2756,10 @@
           <t>Address updated for future orders</t>
         </is>
       </c>
-      <c r="H40" s="5" t="inlineStr"/>
+      <c r="H40" s="5">
+        <f>IF(I40="","",IF(I40=G40,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I40" s="5" t="inlineStr"/>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="6" t="inlineStr">
@@ -2702,7 +2808,10 @@
           <t>Preferences saved, used for meal recommendations</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr"/>
+      <c r="H41" s="5">
+        <f>IF(I41="","",IF(I41=G41,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I41" s="5" t="inlineStr"/>
       <c r="J41" s="5" t="inlineStr"/>
       <c r="K41" s="5" t="inlineStr">
@@ -2749,7 +2858,10 @@
           <t>Unique referral code displayed</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr"/>
+      <c r="H42" s="5">
+        <f>IF(I42="","",IF(I42=G42,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I42" s="5" t="inlineStr"/>
       <c r="J42" s="5" t="inlineStr"/>
       <c r="K42" s="7" t="inlineStr">
@@ -2797,7 +2909,10 @@
           <t>Referral link shared via WhatsApp</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr"/>
+      <c r="H43" s="5">
+        <f>IF(I43="","",IF(I43=G43,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I43" s="5" t="inlineStr"/>
       <c r="J43" s="5" t="inlineStr"/>
       <c r="K43" s="7" t="inlineStr">
@@ -2844,7 +2959,10 @@
           <t>Current balance displayed with transaction history</t>
         </is>
       </c>
-      <c r="H44" s="5" t="inlineStr"/>
+      <c r="H44" s="5">
+        <f>IF(I44="","",IF(I44=G44,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I44" s="5" t="inlineStr"/>
       <c r="J44" s="5" t="inlineStr"/>
       <c r="K44" s="7" t="inlineStr">
@@ -2893,7 +3011,10 @@
           <t>Funds added, balance updated</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr"/>
+      <c r="H45" s="5">
+        <f>IF(I45="","",IF(I45=G45,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I45" s="5" t="inlineStr"/>
       <c r="J45" s="5" t="inlineStr"/>
       <c r="K45" s="7" t="inlineStr">
@@ -2940,7 +3061,10 @@
           <t>All transactions listed with dates and amounts</t>
         </is>
       </c>
-      <c r="H46" s="5" t="inlineStr"/>
+      <c r="H46" s="5">
+        <f>IF(I46="","",IF(I46=G46,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I46" s="5" t="inlineStr"/>
       <c r="J46" s="5" t="inlineStr"/>
       <c r="K46" s="5" t="inlineStr">
@@ -2989,7 +3113,10 @@
           <t>Partner logged in, redirected to partner dashboard</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr"/>
+      <c r="H47" s="5">
+        <f>IF(I47="","",IF(I47=G47,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I47" s="5" t="inlineStr"/>
       <c r="J47" s="5" t="inlineStr"/>
       <c r="K47" s="6" t="inlineStr">
@@ -3036,7 +3163,10 @@
           <t>Error message displayed</t>
         </is>
       </c>
-      <c r="H48" s="5" t="inlineStr"/>
+      <c r="H48" s="5">
+        <f>IF(I48="","",IF(I48=G48,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I48" s="5" t="inlineStr"/>
       <c r="J48" s="5" t="inlineStr"/>
       <c r="K48" s="6" t="inlineStr">
@@ -3083,7 +3213,10 @@
           <t>Logged out, redirected to login page</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr"/>
+      <c r="H49" s="5">
+        <f>IF(I49="","",IF(I49=G49,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I49" s="5" t="inlineStr"/>
       <c r="J49" s="5" t="inlineStr"/>
       <c r="K49" s="6" t="inlineStr">
@@ -3130,7 +3263,10 @@
           <t>Dashboard shows: today's orders, earnings, ratings, quick actions</t>
         </is>
       </c>
-      <c r="H50" s="5" t="inlineStr"/>
+      <c r="H50" s="5">
+        <f>IF(I50="","",IF(I50=G50,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I50" s="5" t="inlineStr"/>
       <c r="J50" s="5" t="inlineStr"/>
       <c r="K50" s="6" t="inlineStr">
@@ -3177,7 +3313,10 @@
           <t>Today's orders, weekly earnings, average rating correct</t>
         </is>
       </c>
-      <c r="H51" s="5" t="inlineStr"/>
+      <c r="H51" s="5">
+        <f>IF(I51="","",IF(I51=G51,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I51" s="5" t="inlineStr"/>
       <c r="J51" s="5" t="inlineStr"/>
       <c r="K51" s="6" t="inlineStr">
@@ -3225,7 +3364,10 @@
           <t>Each button navigates to correct page</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr"/>
+      <c r="H52" s="5">
+        <f>IF(I52="","",IF(I52=G52,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I52" s="5" t="inlineStr"/>
       <c r="J52" s="5" t="inlineStr"/>
       <c r="K52" s="7" t="inlineStr">
@@ -3272,7 +3414,10 @@
           <t>All pending/preparing orders displayed with details</t>
         </is>
       </c>
-      <c r="H53" s="5" t="inlineStr"/>
+      <c r="H53" s="5">
+        <f>IF(I53="","",IF(I53=G53,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I53" s="5" t="inlineStr"/>
       <c r="J53" s="5" t="inlineStr"/>
       <c r="K53" s="8" t="inlineStr">
@@ -3319,7 +3464,10 @@
           <t>Completed orders displayed with dates and amounts</t>
         </is>
       </c>
-      <c r="H54" s="5" t="inlineStr"/>
+      <c r="H54" s="5">
+        <f>IF(I54="","",IF(I54=G54,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I54" s="5" t="inlineStr"/>
       <c r="J54" s="5" t="inlineStr"/>
       <c r="K54" s="6" t="inlineStr">
@@ -3367,7 +3515,10 @@
           <t>Order status changes to Confirmed</t>
         </is>
       </c>
-      <c r="H55" s="5" t="inlineStr"/>
+      <c r="H55" s="5">
+        <f>IF(I55="","",IF(I55=G55,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I55" s="5" t="inlineStr"/>
       <c r="J55" s="5" t="inlineStr"/>
       <c r="K55" s="8" t="inlineStr">
@@ -3415,7 +3566,10 @@
           <t>Status updates, customer receives notification</t>
         </is>
       </c>
-      <c r="H56" s="5" t="inlineStr"/>
+      <c r="H56" s="5">
+        <f>IF(I56="","",IF(I56=G56,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I56" s="5" t="inlineStr"/>
       <c r="J56" s="5" t="inlineStr"/>
       <c r="K56" s="8" t="inlineStr">
@@ -3462,7 +3616,10 @@
           <t>Order items, customer info, delivery address, special instructions displayed</t>
         </is>
       </c>
-      <c r="H57" s="5" t="inlineStr"/>
+      <c r="H57" s="5">
+        <f>IF(I57="","",IF(I57=G57,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I57" s="5" t="inlineStr"/>
       <c r="J57" s="5" t="inlineStr"/>
       <c r="K57" s="6" t="inlineStr">
@@ -3509,7 +3666,10 @@
           <t>Order prints with kitchen ticket format</t>
         </is>
       </c>
-      <c r="H58" s="5" t="inlineStr"/>
+      <c r="H58" s="5">
+        <f>IF(I58="","",IF(I58=G58,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I58" s="5" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr"/>
       <c r="K58" s="5" t="inlineStr">
@@ -3556,7 +3716,10 @@
           <t>All menu items displayed with photos and status</t>
         </is>
       </c>
-      <c r="H59" s="5" t="inlineStr"/>
+      <c r="H59" s="5">
+        <f>IF(I59="","",IF(I59=G59,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I59" s="5" t="inlineStr"/>
       <c r="J59" s="5" t="inlineStr"/>
       <c r="K59" s="6" t="inlineStr">
@@ -3604,7 +3767,10 @@
           <t>Item added to menu, visible to customers</t>
         </is>
       </c>
-      <c r="H60" s="5" t="inlineStr"/>
+      <c r="H60" s="5">
+        <f>IF(I60="","",IF(I60=G60,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I60" s="5" t="inlineStr"/>
       <c r="J60" s="5" t="inlineStr"/>
       <c r="K60" s="6" t="inlineStr">
@@ -3653,7 +3819,10 @@
           <t>Item updated with new information</t>
         </is>
       </c>
-      <c r="H61" s="5" t="inlineStr"/>
+      <c r="H61" s="5">
+        <f>IF(I61="","",IF(I61=G61,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I61" s="5" t="inlineStr"/>
       <c r="J61" s="5" t="inlineStr"/>
       <c r="K61" s="6" t="inlineStr">
@@ -3701,7 +3870,10 @@
           <t>Item removed from menu</t>
         </is>
       </c>
-      <c r="H62" s="5" t="inlineStr"/>
+      <c r="H62" s="5">
+        <f>IF(I62="","",IF(I62=G62,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I62" s="5" t="inlineStr"/>
       <c r="J62" s="5" t="inlineStr"/>
       <c r="K62" s="7" t="inlineStr">
@@ -3749,7 +3921,10 @@
           <t>Item availability changes, customers see/hide item</t>
         </is>
       </c>
-      <c r="H63" s="5" t="inlineStr"/>
+      <c r="H63" s="5">
+        <f>IF(I63="","",IF(I63=G63,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I63" s="5" t="inlineStr"/>
       <c r="J63" s="5" t="inlineStr"/>
       <c r="K63" s="6" t="inlineStr">
@@ -3798,7 +3973,10 @@
           <t>Photo uploaded and displayed on meal card</t>
         </is>
       </c>
-      <c r="H64" s="5" t="inlineStr"/>
+      <c r="H64" s="5">
+        <f>IF(I64="","",IF(I64=G64,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I64" s="5" t="inlineStr"/>
       <c r="J64" s="5" t="inlineStr"/>
       <c r="K64" s="7" t="inlineStr">
@@ -3846,7 +4024,10 @@
           <t>Nutrition info saved and displayed to customers</t>
         </is>
       </c>
-      <c r="H65" s="5" t="inlineStr"/>
+      <c r="H65" s="5">
+        <f>IF(I65="","",IF(I65=G65,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I65" s="5" t="inlineStr"/>
       <c r="J65" s="5" t="inlineStr"/>
       <c r="K65" s="7" t="inlineStr">
@@ -3893,7 +4074,10 @@
           <t>Today's earnings, weekly, monthly totals displayed</t>
         </is>
       </c>
-      <c r="H66" s="5" t="inlineStr"/>
+      <c r="H66" s="5">
+        <f>IF(I66="","",IF(I66=G66,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I66" s="5" t="inlineStr"/>
       <c r="J66" s="5" t="inlineStr"/>
       <c r="K66" s="6" t="inlineStr">
@@ -3940,7 +4124,10 @@
           <t>All weekly payouts listed with dates and amounts</t>
         </is>
       </c>
-      <c r="H67" s="5" t="inlineStr"/>
+      <c r="H67" s="5">
+        <f>IF(I67="","",IF(I67=G67,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I67" s="5" t="inlineStr"/>
       <c r="J67" s="5" t="inlineStr"/>
       <c r="K67" s="6" t="inlineStr">
@@ -3987,7 +4174,10 @@
           <t>Daily breakdown of orders and earnings shown</t>
         </is>
       </c>
-      <c r="H68" s="5" t="inlineStr"/>
+      <c r="H68" s="5">
+        <f>IF(I68="","",IF(I68=G68,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I68" s="5" t="inlineStr"/>
       <c r="J68" s="5" t="inlineStr"/>
       <c r="K68" s="7" t="inlineStr">
@@ -4034,7 +4224,10 @@
           <t>Accurate statistics displayed</t>
         </is>
       </c>
-      <c r="H69" s="5" t="inlineStr"/>
+      <c r="H69" s="5">
+        <f>IF(I69="","",IF(I69=G69,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I69" s="5" t="inlineStr"/>
       <c r="J69" s="5" t="inlineStr"/>
       <c r="K69" s="7" t="inlineStr">
@@ -4081,7 +4274,10 @@
           <t>Restaurant details, hours, capacity displayed</t>
         </is>
       </c>
-      <c r="H70" s="5" t="inlineStr"/>
+      <c r="H70" s="5">
+        <f>IF(I70="","",IF(I70=G70,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I70" s="5" t="inlineStr"/>
       <c r="J70" s="5" t="inlineStr"/>
       <c r="K70" s="6" t="inlineStr">
@@ -4129,7 +4325,10 @@
           <t>Profile updated successfully</t>
         </is>
       </c>
-      <c r="H71" s="5" t="inlineStr"/>
+      <c r="H71" s="5">
+        <f>IF(I71="","",IF(I71=G71,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I71" s="5" t="inlineStr"/>
       <c r="J71" s="5" t="inlineStr"/>
       <c r="K71" s="7" t="inlineStr">
@@ -4177,7 +4376,10 @@
           <t>Bank details updated for future payouts</t>
         </is>
       </c>
-      <c r="H72" s="5" t="inlineStr"/>
+      <c r="H72" s="5">
+        <f>IF(I72="","",IF(I72=G72,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I72" s="5" t="inlineStr"/>
       <c r="J72" s="5" t="inlineStr"/>
       <c r="K72" s="6" t="inlineStr">
@@ -4225,7 +4427,10 @@
           <t>Capacity updated, affects order acceptance</t>
         </is>
       </c>
-      <c r="H73" s="5" t="inlineStr"/>
+      <c r="H73" s="5">
+        <f>IF(I73="","",IF(I73=G73,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I73" s="5" t="inlineStr"/>
       <c r="J73" s="5" t="inlineStr"/>
       <c r="K73" s="6" t="inlineStr">
@@ -4273,7 +4478,10 @@
           <t>Status changes, customers can/cannot place orders</t>
         </is>
       </c>
-      <c r="H74" s="5" t="inlineStr"/>
+      <c r="H74" s="5">
+        <f>IF(I74="","",IF(I74=G74,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I74" s="5" t="inlineStr"/>
       <c r="J74" s="5" t="inlineStr"/>
       <c r="K74" s="6" t="inlineStr">
@@ -4322,7 +4530,10 @@
           <t>Logo updated across platform</t>
         </is>
       </c>
-      <c r="H75" s="5" t="inlineStr"/>
+      <c r="H75" s="5">
+        <f>IF(I75="","",IF(I75=G75,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I75" s="5" t="inlineStr"/>
       <c r="J75" s="5" t="inlineStr"/>
       <c r="K75" s="5" t="inlineStr">
@@ -4370,7 +4581,10 @@
           <t>Photo gallery updated</t>
         </is>
       </c>
-      <c r="H76" s="5" t="inlineStr"/>
+      <c r="H76" s="5">
+        <f>IF(I76="","",IF(I76=G76,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I76" s="5" t="inlineStr"/>
       <c r="J76" s="5" t="inlineStr"/>
       <c r="K76" s="5" t="inlineStr">
@@ -4418,7 +4632,10 @@
           <t>Admin logged in, dashboard displayed</t>
         </is>
       </c>
-      <c r="H77" s="5" t="inlineStr"/>
+      <c r="H77" s="5">
+        <f>IF(I77="","",IF(I77=G77,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I77" s="5" t="inlineStr"/>
       <c r="J77" s="5" t="inlineStr"/>
       <c r="K77" s="6" t="inlineStr">
@@ -4465,7 +4682,10 @@
           <t>Access denied, error shown</t>
         </is>
       </c>
-      <c r="H78" s="5" t="inlineStr"/>
+      <c r="H78" s="5">
+        <f>IF(I78="","",IF(I78=G78,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I78" s="5" t="inlineStr"/>
       <c r="J78" s="5" t="inlineStr"/>
       <c r="K78" s="6" t="inlineStr">
@@ -4511,7 +4731,10 @@
           <t>Logged out, redirected to login</t>
         </is>
       </c>
-      <c r="H79" s="5" t="inlineStr"/>
+      <c r="H79" s="5">
+        <f>IF(I79="","",IF(I79=G79,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I79" s="5" t="inlineStr"/>
       <c r="J79" s="5" t="inlineStr"/>
       <c r="K79" s="6" t="inlineStr">
@@ -4558,7 +4781,10 @@
           <t>Access denied, redirected to dashboard</t>
         </is>
       </c>
-      <c r="H80" s="5" t="inlineStr"/>
+      <c r="H80" s="5">
+        <f>IF(I80="","",IF(I80=G80,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I80" s="5" t="inlineStr"/>
       <c r="J80" s="5" t="inlineStr"/>
       <c r="K80" s="8" t="inlineStr">
@@ -4605,7 +4831,10 @@
           <t>Dashboard shows: total users, orders, revenue, restaurants</t>
         </is>
       </c>
-      <c r="H81" s="5" t="inlineStr"/>
+      <c r="H81" s="5">
+        <f>IF(I81="","",IF(I81=G81,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I81" s="5" t="inlineStr"/>
       <c r="J81" s="5" t="inlineStr"/>
       <c r="K81" s="6" t="inlineStr">
@@ -4652,7 +4881,10 @@
           <t>All metrics accurate and up-to-date</t>
         </is>
       </c>
-      <c r="H82" s="5" t="inlineStr"/>
+      <c r="H82" s="5">
+        <f>IF(I82="","",IF(I82=G82,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I82" s="5" t="inlineStr"/>
       <c r="J82" s="5" t="inlineStr"/>
       <c r="K82" s="6" t="inlineStr">
@@ -4698,7 +4930,10 @@
           <t>Navigates to correct section</t>
         </is>
       </c>
-      <c r="H83" s="5" t="inlineStr"/>
+      <c r="H83" s="5">
+        <f>IF(I83="","",IF(I83=G83,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I83" s="5" t="inlineStr"/>
       <c r="J83" s="5" t="inlineStr"/>
       <c r="K83" s="7" t="inlineStr">
@@ -4745,7 +4980,10 @@
           <t>Recent orders, signups, restaurant applications shown</t>
         </is>
       </c>
-      <c r="H84" s="5" t="inlineStr"/>
+      <c r="H84" s="5">
+        <f>IF(I84="","",IF(I84=G84,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I84" s="5" t="inlineStr"/>
       <c r="J84" s="5" t="inlineStr"/>
       <c r="K84" s="7" t="inlineStr">
@@ -4792,7 +5030,10 @@
           <t>All users displayed with roles, status, subscription</t>
         </is>
       </c>
-      <c r="H85" s="5" t="inlineStr"/>
+      <c r="H85" s="5">
+        <f>IF(I85="","",IF(I85=G85,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I85" s="5" t="inlineStr"/>
       <c r="J85" s="5" t="inlineStr"/>
       <c r="K85" s="6" t="inlineStr">
@@ -4839,7 +5080,10 @@
           <t>Matching users displayed</t>
         </is>
       </c>
-      <c r="H86" s="5" t="inlineStr"/>
+      <c r="H86" s="5">
+        <f>IF(I86="","",IF(I86=G86,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I86" s="5" t="inlineStr"/>
       <c r="J86" s="5" t="inlineStr"/>
       <c r="K86" s="6" t="inlineStr">
@@ -4886,7 +5130,10 @@
           <t>Filtered user list displayed</t>
         </is>
       </c>
-      <c r="H87" s="5" t="inlineStr"/>
+      <c r="H87" s="5">
+        <f>IF(I87="","",IF(I87=G87,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I87" s="5" t="inlineStr"/>
       <c r="J87" s="5" t="inlineStr"/>
       <c r="K87" s="7" t="inlineStr">
@@ -4933,7 +5180,10 @@
           <t>Full user info: profile, orders, subscription, referrals</t>
         </is>
       </c>
-      <c r="H88" s="5" t="inlineStr"/>
+      <c r="H88" s="5">
+        <f>IF(I88="","",IF(I88=G88,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I88" s="5" t="inlineStr"/>
       <c r="J88" s="5" t="inlineStr"/>
       <c r="K88" s="6" t="inlineStr">
@@ -4982,7 +5232,10 @@
           <t>User information updated</t>
         </is>
       </c>
-      <c r="H89" s="5" t="inlineStr"/>
+      <c r="H89" s="5">
+        <f>IF(I89="","",IF(I89=G89,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I89" s="5" t="inlineStr"/>
       <c r="J89" s="5" t="inlineStr"/>
       <c r="K89" s="7" t="inlineStr">
@@ -5030,7 +5283,10 @@
           <t>User account deactivated</t>
         </is>
       </c>
-      <c r="H90" s="5" t="inlineStr"/>
+      <c r="H90" s="5">
+        <f>IF(I90="","",IF(I90=G90,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I90" s="5" t="inlineStr"/>
       <c r="J90" s="5" t="inlineStr"/>
       <c r="K90" s="7" t="inlineStr">
@@ -5078,7 +5334,10 @@
           <t>User permanently deleted</t>
         </is>
       </c>
-      <c r="H91" s="5" t="inlineStr"/>
+      <c r="H91" s="5">
+        <f>IF(I91="","",IF(I91=G91,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I91" s="5" t="inlineStr"/>
       <c r="J91" s="5" t="inlineStr"/>
       <c r="K91" s="7" t="inlineStr">
@@ -5125,7 +5384,10 @@
           <t>All restaurants displayed with status, ratings, earnings</t>
         </is>
       </c>
-      <c r="H92" s="5" t="inlineStr"/>
+      <c r="H92" s="5">
+        <f>IF(I92="","",IF(I92=G92,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I92" s="5" t="inlineStr"/>
       <c r="J92" s="5" t="inlineStr"/>
       <c r="K92" s="6" t="inlineStr">
@@ -5172,7 +5434,10 @@
           <t>All pending applications displayed</t>
         </is>
       </c>
-      <c r="H93" s="5" t="inlineStr"/>
+      <c r="H93" s="5">
+        <f>IF(I93="","",IF(I93=G93,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I93" s="5" t="inlineStr"/>
       <c r="J93" s="5" t="inlineStr"/>
       <c r="K93" s="6" t="inlineStr">
@@ -5221,7 +5486,10 @@
           <t>Restaurant approved, status changes to active</t>
         </is>
       </c>
-      <c r="H94" s="5" t="inlineStr"/>
+      <c r="H94" s="5">
+        <f>IF(I94="","",IF(I94=G94,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I94" s="5" t="inlineStr"/>
       <c r="J94" s="5" t="inlineStr"/>
       <c r="K94" s="8" t="inlineStr">
@@ -5270,7 +5538,10 @@
           <t>Application rejected, restaurant notified</t>
         </is>
       </c>
-      <c r="H95" s="5" t="inlineStr"/>
+      <c r="H95" s="5">
+        <f>IF(I95="","",IF(I95=G95,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I95" s="5" t="inlineStr"/>
       <c r="J95" s="5" t="inlineStr"/>
       <c r="K95" s="6" t="inlineStr">
@@ -5317,7 +5588,10 @@
           <t>All restaurant info: orders, earnings, ratings, menu</t>
         </is>
       </c>
-      <c r="H96" s="5" t="inlineStr"/>
+      <c r="H96" s="5">
+        <f>IF(I96="","",IF(I96=G96,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I96" s="5" t="inlineStr"/>
       <c r="J96" s="5" t="inlineStr"/>
       <c r="K96" s="6" t="inlineStr">
@@ -5366,7 +5640,10 @@
           <t>Restaurant information updated</t>
         </is>
       </c>
-      <c r="H97" s="5" t="inlineStr"/>
+      <c r="H97" s="5">
+        <f>IF(I97="","",IF(I97=G97,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I97" s="5" t="inlineStr"/>
       <c r="J97" s="5" t="inlineStr"/>
       <c r="K97" s="7" t="inlineStr">
@@ -5414,7 +5691,10 @@
           <t>New payout rate applied</t>
         </is>
       </c>
-      <c r="H98" s="5" t="inlineStr"/>
+      <c r="H98" s="5">
+        <f>IF(I98="","",IF(I98=G98,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I98" s="5" t="inlineStr"/>
       <c r="J98" s="5" t="inlineStr"/>
       <c r="K98" s="6" t="inlineStr">
@@ -5463,7 +5743,10 @@
           <t>Restaurant suspended, cannot receive orders</t>
         </is>
       </c>
-      <c r="H99" s="5" t="inlineStr"/>
+      <c r="H99" s="5">
+        <f>IF(I99="","",IF(I99=G99,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I99" s="5" t="inlineStr"/>
       <c r="J99" s="5" t="inlineStr"/>
       <c r="K99" s="6" t="inlineStr">
@@ -5511,7 +5794,10 @@
           <t>Restaurant reactivated, can receive orders</t>
         </is>
       </c>
-      <c r="H100" s="5" t="inlineStr"/>
+      <c r="H100" s="5">
+        <f>IF(I100="","",IF(I100=G100,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I100" s="5" t="inlineStr"/>
       <c r="J100" s="5" t="inlineStr"/>
       <c r="K100" s="6" t="inlineStr">
@@ -5559,7 +5845,10 @@
           <t>Restaurant removed from platform</t>
         </is>
       </c>
-      <c r="H101" s="5" t="inlineStr"/>
+      <c r="H101" s="5">
+        <f>IF(I101="","",IF(I101=G101,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I101" s="5" t="inlineStr"/>
       <c r="J101" s="5" t="inlineStr"/>
       <c r="K101" s="7" t="inlineStr">
@@ -5606,7 +5895,10 @@
           <t>All orders displayed with filters and search</t>
         </is>
       </c>
-      <c r="H102" s="5" t="inlineStr"/>
+      <c r="H102" s="5">
+        <f>IF(I102="","",IF(I102=G102,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I102" s="5" t="inlineStr"/>
       <c r="J102" s="5" t="inlineStr"/>
       <c r="K102" s="6" t="inlineStr">
@@ -5653,7 +5945,10 @@
           <t>Orders filtered by status</t>
         </is>
       </c>
-      <c r="H103" s="5" t="inlineStr"/>
+      <c r="H103" s="5">
+        <f>IF(I103="","",IF(I103=G103,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I103" s="5" t="inlineStr"/>
       <c r="J103" s="5" t="inlineStr"/>
       <c r="K103" s="6" t="inlineStr">
@@ -5700,7 +5995,10 @@
           <t>Matching orders displayed</t>
         </is>
       </c>
-      <c r="H104" s="5" t="inlineStr"/>
+      <c r="H104" s="5">
+        <f>IF(I104="","",IF(I104=G104,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I104" s="5" t="inlineStr"/>
       <c r="J104" s="5" t="inlineStr"/>
       <c r="K104" s="6" t="inlineStr">
@@ -5747,7 +6045,10 @@
           <t>Full order info: items, customer, restaurant, status, payment</t>
         </is>
       </c>
-      <c r="H105" s="5" t="inlineStr"/>
+      <c r="H105" s="5">
+        <f>IF(I105="","",IF(I105=G105,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I105" s="5" t="inlineStr"/>
       <c r="J105" s="5" t="inlineStr"/>
       <c r="K105" s="6" t="inlineStr">
@@ -5795,7 +6096,10 @@
           <t>Order status updated</t>
         </is>
       </c>
-      <c r="H106" s="5" t="inlineStr"/>
+      <c r="H106" s="5">
+        <f>IF(I106="","",IF(I106=G106,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I106" s="5" t="inlineStr"/>
       <c r="J106" s="5" t="inlineStr"/>
       <c r="K106" s="7" t="inlineStr">
@@ -5844,7 +6148,10 @@
           <t>Order cancelled, refund processed</t>
         </is>
       </c>
-      <c r="H107" s="5" t="inlineStr"/>
+      <c r="H107" s="5">
+        <f>IF(I107="","",IF(I107=G107,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I107" s="5" t="inlineStr"/>
       <c r="J107" s="5" t="inlineStr"/>
       <c r="K107" s="7" t="inlineStr">
@@ -5893,7 +6200,10 @@
           <t>Refund processed, customer notified</t>
         </is>
       </c>
-      <c r="H108" s="5" t="inlineStr"/>
+      <c r="H108" s="5">
+        <f>IF(I108="","",IF(I108=G108,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I108" s="5" t="inlineStr"/>
       <c r="J108" s="5" t="inlineStr"/>
       <c r="K108" s="6" t="inlineStr">
@@ -5942,7 +6252,10 @@
           <t>Driver assigned, notified</t>
         </is>
       </c>
-      <c r="H109" s="5" t="inlineStr"/>
+      <c r="H109" s="5">
+        <f>IF(I109="","",IF(I109=G109,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I109" s="5" t="inlineStr"/>
       <c r="J109" s="5" t="inlineStr"/>
       <c r="K109" s="7" t="inlineStr">
@@ -5989,7 +6302,10 @@
           <t>All active subscriptions displayed</t>
         </is>
       </c>
-      <c r="H110" s="5" t="inlineStr"/>
+      <c r="H110" s="5">
+        <f>IF(I110="","",IF(I110=G110,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I110" s="5" t="inlineStr"/>
       <c r="J110" s="5" t="inlineStr"/>
       <c r="K110" s="6" t="inlineStr">
@@ -6036,7 +6352,10 @@
           <t>All plans with pricing displayed</t>
         </is>
       </c>
-      <c r="H111" s="5" t="inlineStr"/>
+      <c r="H111" s="5">
+        <f>IF(I111="","",IF(I111=G111,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I111" s="5" t="inlineStr"/>
       <c r="J111" s="5" t="inlineStr"/>
       <c r="K111" s="6" t="inlineStr">
@@ -6084,7 +6403,10 @@
           <t>Plan updated</t>
         </is>
       </c>
-      <c r="H112" s="5" t="inlineStr"/>
+      <c r="H112" s="5">
+        <f>IF(I112="","",IF(I112=G112,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I112" s="5" t="inlineStr"/>
       <c r="J112" s="5" t="inlineStr"/>
       <c r="K112" s="7" t="inlineStr">
@@ -6132,7 +6454,10 @@
           <t>New plan created</t>
         </is>
       </c>
-      <c r="H113" s="5" t="inlineStr"/>
+      <c r="H113" s="5">
+        <f>IF(I113="","",IF(I113=G113,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I113" s="5" t="inlineStr"/>
       <c r="J113" s="5" t="inlineStr"/>
       <c r="K113" s="5" t="inlineStr">
@@ -6180,7 +6505,10 @@
           <t>Subscription cancelled</t>
         </is>
       </c>
-      <c r="H114" s="5" t="inlineStr"/>
+      <c r="H114" s="5">
+        <f>IF(I114="","",IF(I114=G114,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I114" s="5" t="inlineStr"/>
       <c r="J114" s="5" t="inlineStr"/>
       <c r="K114" s="7" t="inlineStr">
@@ -6228,7 +6556,10 @@
           <t>Subscription extended</t>
         </is>
       </c>
-      <c r="H115" s="5" t="inlineStr"/>
+      <c r="H115" s="5">
+        <f>IF(I115="","",IF(I115=G115,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I115" s="5" t="inlineStr"/>
       <c r="J115" s="5" t="inlineStr"/>
       <c r="K115" s="5" t="inlineStr">
@@ -6275,7 +6606,10 @@
           <t>All meals from all restaurants displayed</t>
         </is>
       </c>
-      <c r="H116" s="5" t="inlineStr"/>
+      <c r="H116" s="5">
+        <f>IF(I116="","",IF(I116=G116,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I116" s="5" t="inlineStr"/>
       <c r="J116" s="5" t="inlineStr"/>
       <c r="K116" s="7" t="inlineStr">
@@ -6324,7 +6658,10 @@
           <t>Meal updated</t>
         </is>
       </c>
-      <c r="H117" s="5" t="inlineStr"/>
+      <c r="H117" s="5">
+        <f>IF(I117="","",IF(I117=G117,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I117" s="5" t="inlineStr"/>
       <c r="J117" s="5" t="inlineStr"/>
       <c r="K117" s="7" t="inlineStr">
@@ -6372,7 +6709,10 @@
           <t>Meal deleted</t>
         </is>
       </c>
-      <c r="H118" s="5" t="inlineStr"/>
+      <c r="H118" s="5">
+        <f>IF(I118="","",IF(I118=G118,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I118" s="5" t="inlineStr"/>
       <c r="J118" s="5" t="inlineStr"/>
       <c r="K118" s="7" t="inlineStr">
@@ -6419,7 +6759,10 @@
           <t>Tags updated across platform</t>
         </is>
       </c>
-      <c r="H119" s="5" t="inlineStr"/>
+      <c r="H119" s="5">
+        <f>IF(I119="","",IF(I119=G119,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I119" s="5" t="inlineStr"/>
       <c r="J119" s="5" t="inlineStr"/>
       <c r="K119" s="5" t="inlineStr">
@@ -6467,7 +6810,10 @@
           <t>Announcement visible to users</t>
         </is>
       </c>
-      <c r="H120" s="5" t="inlineStr"/>
+      <c r="H120" s="5">
+        <f>IF(I120="","",IF(I120=G120,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I120" s="5" t="inlineStr"/>
       <c r="J120" s="5" t="inlineStr"/>
       <c r="K120" s="5" t="inlineStr">
@@ -6514,7 +6860,10 @@
           <t>Analytics displayed: revenue, orders, users, growth</t>
         </is>
       </c>
-      <c r="H121" s="5" t="inlineStr"/>
+      <c r="H121" s="5">
+        <f>IF(I121="","",IF(I121=G121,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I121" s="5" t="inlineStr"/>
       <c r="J121" s="5" t="inlineStr"/>
       <c r="K121" s="7" t="inlineStr">
@@ -6562,7 +6911,10 @@
           <t>Revenue report generated</t>
         </is>
       </c>
-      <c r="H122" s="5" t="inlineStr"/>
+      <c r="H122" s="5">
+        <f>IF(I122="","",IF(I122=G122,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I122" s="5" t="inlineStr"/>
       <c r="J122" s="5" t="inlineStr"/>
       <c r="K122" s="7" t="inlineStr">
@@ -6611,7 +6963,10 @@
           <t>Report downloaded</t>
         </is>
       </c>
-      <c r="H123" s="5" t="inlineStr"/>
+      <c r="H123" s="5">
+        <f>IF(I123="","",IF(I123=G123,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I123" s="5" t="inlineStr"/>
       <c r="J123" s="5" t="inlineStr"/>
       <c r="K123" s="5" t="inlineStr">
@@ -6658,7 +7013,10 @@
           <t>Per-restaurant stats displayed</t>
         </is>
       </c>
-      <c r="H124" s="5" t="inlineStr"/>
+      <c r="H124" s="5">
+        <f>IF(I124="","",IF(I124=G124,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I124" s="5" t="inlineStr"/>
       <c r="J124" s="5" t="inlineStr"/>
       <c r="K124" s="7" t="inlineStr">
@@ -6705,7 +7063,10 @@
           <t>All pending payouts displayed</t>
         </is>
       </c>
-      <c r="H125" s="5" t="inlineStr"/>
+      <c r="H125" s="5">
+        <f>IF(I125="","",IF(I125=G125,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I125" s="5" t="inlineStr"/>
       <c r="J125" s="5" t="inlineStr"/>
       <c r="K125" s="6" t="inlineStr">
@@ -6753,7 +7114,10 @@
           <t>Payouts processed, restaurants notified</t>
         </is>
       </c>
-      <c r="H126" s="5" t="inlineStr"/>
+      <c r="H126" s="5">
+        <f>IF(I126="","",IF(I126=G126,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I126" s="5" t="inlineStr"/>
       <c r="J126" s="5" t="inlineStr"/>
       <c r="K126" s="8" t="inlineStr">
@@ -6800,7 +7164,10 @@
           <t>All processed payouts listed</t>
         </is>
       </c>
-      <c r="H127" s="5" t="inlineStr"/>
+      <c r="H127" s="5">
+        <f>IF(I127="","",IF(I127=G127,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I127" s="5" t="inlineStr"/>
       <c r="J127" s="5" t="inlineStr"/>
       <c r="K127" s="7" t="inlineStr">
@@ -6849,7 +7216,10 @@
           <t>Payout adjusted with audit trail</t>
         </is>
       </c>
-      <c r="H128" s="5" t="inlineStr"/>
+      <c r="H128" s="5">
+        <f>IF(I128="","",IF(I128=G128,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I128" s="5" t="inlineStr"/>
       <c r="J128" s="5" t="inlineStr"/>
       <c r="K128" s="7" t="inlineStr">
@@ -6897,7 +7267,10 @@
           <t>Settings saved</t>
         </is>
       </c>
-      <c r="H129" s="5" t="inlineStr"/>
+      <c r="H129" s="5">
+        <f>IF(I129="","",IF(I129=G129,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I129" s="5" t="inlineStr"/>
       <c r="J129" s="5" t="inlineStr"/>
       <c r="K129" s="7" t="inlineStr">
@@ -6945,7 +7318,10 @@
           <t>Payment settings updated</t>
         </is>
       </c>
-      <c r="H130" s="5" t="inlineStr"/>
+      <c r="H130" s="5">
+        <f>IF(I130="","",IF(I130=G130,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I130" s="5" t="inlineStr"/>
       <c r="J130" s="5" t="inlineStr"/>
       <c r="K130" s="6" t="inlineStr">
@@ -6993,7 +7369,10 @@
           <t>Notification settings saved</t>
         </is>
       </c>
-      <c r="H131" s="5" t="inlineStr"/>
+      <c r="H131" s="5">
+        <f>IF(I131="","",IF(I131=G131,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I131" s="5" t="inlineStr"/>
       <c r="J131" s="5" t="inlineStr"/>
       <c r="K131" s="5" t="inlineStr">
@@ -7041,7 +7420,10 @@
           <t>Referral settings updated</t>
         </is>
       </c>
-      <c r="H132" s="5" t="inlineStr"/>
+      <c r="H132" s="5">
+        <f>IF(I132="","",IF(I132=G132,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I132" s="5" t="inlineStr"/>
       <c r="J132" s="5" t="inlineStr"/>
       <c r="K132" s="5" t="inlineStr">
@@ -7089,7 +7471,10 @@
           <t>Driver logged in, dashboard displayed</t>
         </is>
       </c>
-      <c r="H133" s="5" t="inlineStr"/>
+      <c r="H133" s="5">
+        <f>IF(I133="","",IF(I133=G133,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I133" s="5" t="inlineStr"/>
       <c r="J133" s="5" t="inlineStr"/>
       <c r="K133" s="6" t="inlineStr">
@@ -7135,7 +7520,10 @@
           <t>Driver logged out</t>
         </is>
       </c>
-      <c r="H134" s="5" t="inlineStr"/>
+      <c r="H134" s="5">
+        <f>IF(I134="","",IF(I134=G134,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I134" s="5" t="inlineStr"/>
       <c r="J134" s="5" t="inlineStr"/>
       <c r="K134" s="6" t="inlineStr">
@@ -7182,7 +7570,10 @@
           <t>Dashboard shows: available orders, today's earnings, active deliveries</t>
         </is>
       </c>
-      <c r="H135" s="5" t="inlineStr"/>
+      <c r="H135" s="5">
+        <f>IF(I135="","",IF(I135=G135,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I135" s="5" t="inlineStr"/>
       <c r="J135" s="5" t="inlineStr"/>
       <c r="K135" s="6" t="inlineStr">
@@ -7229,7 +7620,10 @@
           <t>Correct stats displayed</t>
         </is>
       </c>
-      <c r="H136" s="5" t="inlineStr"/>
+      <c r="H136" s="5">
+        <f>IF(I136="","",IF(I136=G136,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I136" s="5" t="inlineStr"/>
       <c r="J136" s="5" t="inlineStr"/>
       <c r="K136" s="7" t="inlineStr">
@@ -7276,7 +7670,10 @@
           <t>Orders ready for pickup displayed</t>
         </is>
       </c>
-      <c r="H137" s="5" t="inlineStr"/>
+      <c r="H137" s="5">
+        <f>IF(I137="","",IF(I137=G137,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I137" s="5" t="inlineStr"/>
       <c r="J137" s="5" t="inlineStr"/>
       <c r="K137" s="8" t="inlineStr">
@@ -7324,7 +7721,10 @@
           <t>Order assigned to driver</t>
         </is>
       </c>
-      <c r="H138" s="5" t="inlineStr"/>
+      <c r="H138" s="5">
+        <f>IF(I138="","",IF(I138=G138,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I138" s="5" t="inlineStr"/>
       <c r="J138" s="5" t="inlineStr"/>
       <c r="K138" s="8" t="inlineStr">
@@ -7371,7 +7771,10 @@
           <t>Accepted orders displayed with pickup details</t>
         </is>
       </c>
-      <c r="H139" s="5" t="inlineStr"/>
+      <c r="H139" s="5">
+        <f>IF(I139="","",IF(I139=G139,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I139" s="5" t="inlineStr"/>
       <c r="J139" s="5" t="inlineStr"/>
       <c r="K139" s="6" t="inlineStr">
@@ -7419,7 +7822,10 @@
           <t>Maps opens with route to restaurant</t>
         </is>
       </c>
-      <c r="H140" s="5" t="inlineStr"/>
+      <c r="H140" s="5">
+        <f>IF(I140="","",IF(I140=G140,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I140" s="5" t="inlineStr"/>
       <c r="J140" s="5" t="inlineStr"/>
       <c r="K140" s="6" t="inlineStr">
@@ -7467,7 +7873,10 @@
           <t>Status updated, customer notified</t>
         </is>
       </c>
-      <c r="H141" s="5" t="inlineStr"/>
+      <c r="H141" s="5">
+        <f>IF(I141="","",IF(I141=G141,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I141" s="5" t="inlineStr"/>
       <c r="J141" s="5" t="inlineStr"/>
       <c r="K141" s="8" t="inlineStr">
@@ -7514,7 +7923,10 @@
           <t>Maps opens with route to customer</t>
         </is>
       </c>
-      <c r="H142" s="5" t="inlineStr"/>
+      <c r="H142" s="5">
+        <f>IF(I142="","",IF(I142=G142,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I142" s="5" t="inlineStr"/>
       <c r="J142" s="5" t="inlineStr"/>
       <c r="K142" s="6" t="inlineStr">
@@ -7563,7 +7975,10 @@
           <t>Status updated, delivery complete</t>
         </is>
       </c>
-      <c r="H143" s="5" t="inlineStr"/>
+      <c r="H143" s="5">
+        <f>IF(I143="","",IF(I143=G143,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I143" s="5" t="inlineStr"/>
       <c r="J143" s="5" t="inlineStr"/>
       <c r="K143" s="8" t="inlineStr">
@@ -7610,7 +8025,10 @@
           <t>Completed deliveries with earnings displayed</t>
         </is>
       </c>
-      <c r="H144" s="5" t="inlineStr"/>
+      <c r="H144" s="5">
+        <f>IF(I144="","",IF(I144=G144,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I144" s="5" t="inlineStr"/>
       <c r="J144" s="5" t="inlineStr"/>
       <c r="K144" s="7" t="inlineStr">
@@ -7657,7 +8075,10 @@
           <t>Full info: restaurant, customer, address, items, earnings</t>
         </is>
       </c>
-      <c r="H145" s="5" t="inlineStr"/>
+      <c r="H145" s="5">
+        <f>IF(I145="","",IF(I145=G145,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I145" s="5" t="inlineStr"/>
       <c r="J145" s="5" t="inlineStr"/>
       <c r="K145" s="7" t="inlineStr">
@@ -7704,7 +8125,10 @@
           <t>Today's earnings, weekly, total displayed</t>
         </is>
       </c>
-      <c r="H146" s="5" t="inlineStr"/>
+      <c r="H146" s="5">
+        <f>IF(I146="","",IF(I146=G146,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I146" s="5" t="inlineStr"/>
       <c r="J146" s="5" t="inlineStr"/>
       <c r="K146" s="6" t="inlineStr">
@@ -7751,7 +8175,10 @@
           <t>Accurate earnings history</t>
         </is>
       </c>
-      <c r="H147" s="5" t="inlineStr"/>
+      <c r="H147" s="5">
+        <f>IF(I147="","",IF(I147=G147,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I147" s="5" t="inlineStr"/>
       <c r="J147" s="5" t="inlineStr"/>
       <c r="K147" s="7" t="inlineStr">
@@ -7798,7 +8225,10 @@
           <t>Payout status displayed</t>
         </is>
       </c>
-      <c r="H148" s="5" t="inlineStr"/>
+      <c r="H148" s="5">
+        <f>IF(I148="","",IF(I148=G148,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I148" s="5" t="inlineStr"/>
       <c r="J148" s="5" t="inlineStr"/>
       <c r="K148" s="7" t="inlineStr">
@@ -7845,7 +8275,10 @@
           <t>Driver details, vehicle info, ratings displayed</t>
         </is>
       </c>
-      <c r="H149" s="5" t="inlineStr"/>
+      <c r="H149" s="5">
+        <f>IF(I149="","",IF(I149=G149,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I149" s="5" t="inlineStr"/>
       <c r="J149" s="5" t="inlineStr"/>
       <c r="K149" s="7" t="inlineStr">
@@ -7893,7 +8326,10 @@
           <t>Profile updated</t>
         </is>
       </c>
-      <c r="H150" s="5" t="inlineStr"/>
+      <c r="H150" s="5">
+        <f>IF(I150="","",IF(I150=G150,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I150" s="5" t="inlineStr"/>
       <c r="J150" s="5" t="inlineStr"/>
       <c r="K150" s="7" t="inlineStr">
@@ -7940,7 +8376,10 @@
           <t>Vehicle info updated</t>
         </is>
       </c>
-      <c r="H151" s="5" t="inlineStr"/>
+      <c r="H151" s="5">
+        <f>IF(I151="","",IF(I151=G151,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I151" s="5" t="inlineStr"/>
       <c r="J151" s="5" t="inlineStr"/>
       <c r="K151" s="5" t="inlineStr">
@@ -7987,7 +8426,10 @@
           <t>Status updated, affects order availability</t>
         </is>
       </c>
-      <c r="H152" s="5" t="inlineStr"/>
+      <c r="H152" s="5">
+        <f>IF(I152="","",IF(I152=G152,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I152" s="5" t="inlineStr"/>
       <c r="J152" s="5" t="inlineStr"/>
       <c r="K152" s="6" t="inlineStr">
@@ -8034,7 +8476,10 @@
           <t>Bank details updated for payouts</t>
         </is>
       </c>
-      <c r="H153" s="5" t="inlineStr"/>
+      <c r="H153" s="5">
+        <f>IF(I153="","",IF(I153=G153,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I153" s="5" t="inlineStr"/>
       <c r="J153" s="5" t="inlineStr"/>
       <c r="K153" s="6" t="inlineStr">
@@ -8081,7 +8526,10 @@
           <t>Emails delivered correctly</t>
         </is>
       </c>
-      <c r="H154" s="5" t="inlineStr"/>
+      <c r="H154" s="5">
+        <f>IF(I154="","",IF(I154=G154,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I154" s="5" t="inlineStr"/>
       <c r="J154" s="5" t="inlineStr"/>
       <c r="K154" s="7" t="inlineStr">
@@ -8128,7 +8576,10 @@
           <t>WhatsApp messages delivered</t>
         </is>
       </c>
-      <c r="H155" s="5" t="inlineStr"/>
+      <c r="H155" s="5">
+        <f>IF(I155="","",IF(I155=G155,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I155" s="5" t="inlineStr"/>
       <c r="J155" s="5" t="inlineStr"/>
       <c r="K155" s="6" t="inlineStr">
@@ -8175,7 +8626,10 @@
           <t>Push notifications received</t>
         </is>
       </c>
-      <c r="H156" s="5" t="inlineStr"/>
+      <c r="H156" s="5">
+        <f>IF(I156="","",IF(I156=G156,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I156" s="5" t="inlineStr"/>
       <c r="J156" s="5" t="inlineStr"/>
       <c r="K156" s="5" t="inlineStr">
@@ -8223,7 +8677,10 @@
           <t>Payment processed, subscription activated</t>
         </is>
       </c>
-      <c r="H157" s="5" t="inlineStr"/>
+      <c r="H157" s="5">
+        <f>IF(I157="","",IF(I157=G157,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I157" s="5" t="inlineStr"/>
       <c r="J157" s="5" t="inlineStr"/>
       <c r="K157" s="8" t="inlineStr">
@@ -8270,7 +8727,10 @@
           <t>Refund processed correctly</t>
         </is>
       </c>
-      <c r="H158" s="5" t="inlineStr"/>
+      <c r="H158" s="5">
+        <f>IF(I158="","",IF(I158=G158,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I158" s="5" t="inlineStr"/>
       <c r="J158" s="5" t="inlineStr"/>
       <c r="K158" s="6" t="inlineStr">
@@ -8317,7 +8777,10 @@
           <t>Access denied for unauthorized data</t>
         </is>
       </c>
-      <c r="H159" s="5" t="inlineStr"/>
+      <c r="H159" s="5">
+        <f>IF(I159="","",IF(I159=G159,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I159" s="5" t="inlineStr"/>
       <c r="J159" s="5" t="inlineStr"/>
       <c r="K159" s="8" t="inlineStr">
@@ -8364,7 +8827,10 @@
           <t>Redirected to login page</t>
         </is>
       </c>
-      <c r="H160" s="5" t="inlineStr"/>
+      <c r="H160" s="5">
+        <f>IF(I160="","",IF(I160=G160,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I160" s="5" t="inlineStr"/>
       <c r="J160" s="5" t="inlineStr"/>
       <c r="K160" s="8" t="inlineStr">
@@ -8411,7 +8877,10 @@
           <t>All pages load within acceptable time</t>
         </is>
       </c>
-      <c r="H161" s="5" t="inlineStr"/>
+      <c r="H161" s="5">
+        <f>IF(I161="","",IF(I161=G161,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I161" s="5" t="inlineStr"/>
       <c r="J161" s="5" t="inlineStr"/>
       <c r="K161" s="7" t="inlineStr">
@@ -8458,7 +8927,10 @@
           <t>All features work on mobile</t>
         </is>
       </c>
-      <c r="H162" s="5" t="inlineStr"/>
+      <c r="H162" s="5">
+        <f>IF(I162="","",IF(I162=G162,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I162" s="5" t="inlineStr"/>
       <c r="J162" s="5" t="inlineStr"/>
       <c r="K162" s="6" t="inlineStr">
@@ -8505,7 +8977,10 @@
           <t>Backups running successfully</t>
         </is>
       </c>
-      <c r="H163" s="5" t="inlineStr"/>
+      <c r="H163" s="5">
+        <f>IF(I163="","",IF(I163=G163,"PASS","FAIL"))</f>
+        <v/>
+      </c>
       <c r="I163" s="5" t="inlineStr"/>
       <c r="J163" s="5" t="inlineStr"/>
       <c r="K163" s="7" t="inlineStr">

</xml_diff>

<commit_message>
add 47 additional Partner Portal tests for comprehensive coverage
</commit_message>
<xml_diff>
--- a/docs/plans/Nutrio-Fuel-E2E-Test-Plan.xlsx
+++ b/docs/plans/Nutrio-Fuel-E2E-Test-Plan.xlsx
@@ -577,7 +577,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -622,7 +621,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -702,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8989,6 +8987,4646 @@
         </is>
       </c>
       <c r="L163" s="5" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>TC153</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>Password Reset</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>Partner Password Reset Flow</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Forgot Password on partner login
+2. Enter registered email
+3. Check email for reset link
+4. Click link and set new password
+5. Login with new password</t>
+        </is>
+      </c>
+      <c r="G164" s="5" t="inlineStr">
+        <is>
+          <t>Password reset successful, can login with new credentials</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr"/>
+      <c r="I164" s="5" t="inlineStr"/>
+      <c r="J164" s="5" t="inlineStr"/>
+      <c r="K164" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L164" s="5" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>TC154</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 1</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 1 - Basic Info</t>
+        </is>
+      </c>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>1. Start partner registration
+2. Fill restaurant name
+3. Add description
+4. Select cuisine type
+5. Add dietary tags</t>
+        </is>
+      </c>
+      <c r="G165" s="5" t="inlineStr">
+        <is>
+          <t>Step 1 saved, can proceed to Step 2</t>
+        </is>
+      </c>
+      <c r="H165" s="5" t="inlineStr"/>
+      <c r="I165" s="5" t="inlineStr"/>
+      <c r="J165" s="5" t="inlineStr"/>
+      <c r="K165" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L165" s="5" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>TC155</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 2</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 2 - Location</t>
+        </is>
+      </c>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter address
+2. Pin location on map
+3. Add phone number
+4. Add email
+5. Set operating hours</t>
+        </is>
+      </c>
+      <c r="G166" s="5" t="inlineStr">
+        <is>
+          <t>Step 2 saved, can proceed to Step 3</t>
+        </is>
+      </c>
+      <c r="H166" s="5" t="inlineStr"/>
+      <c r="I166" s="5" t="inlineStr"/>
+      <c r="J166" s="5" t="inlineStr"/>
+      <c r="K166" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L166" s="5" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>TC156</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 3</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 3 - Media</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>1. Upload logo (required)
+2. Upload restaurant photos
+3. Verify image preview
+4. Check file size limits</t>
+        </is>
+      </c>
+      <c r="G167" s="5" t="inlineStr">
+        <is>
+          <t>Images uploaded and preview shown</t>
+        </is>
+      </c>
+      <c r="H167" s="5" t="inlineStr"/>
+      <c r="I167" s="5" t="inlineStr"/>
+      <c r="J167" s="5" t="inlineStr"/>
+      <c r="K167" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L167" s="5" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>TC157</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 4</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 4 - Kitchen Details</t>
+        </is>
+      </c>
+      <c r="F168" s="5" t="inlineStr">
+        <is>
+          <t>1. Set average prep time
+2. Set daily capacity
+3. Add bank account info
+4. Add bank name and IBAN</t>
+        </is>
+      </c>
+      <c r="G168" s="5" t="inlineStr">
+        <is>
+          <t>Kitchen details saved, can proceed to Step 5</t>
+        </is>
+      </c>
+      <c r="H168" s="5" t="inlineStr"/>
+      <c r="I168" s="5" t="inlineStr"/>
+      <c r="J168" s="5" t="inlineStr"/>
+      <c r="K168" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L168" s="5" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>TC158</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 5</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 5 - Review &amp; Submit</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>1. Review all entered information
+2. Check accuracy of details
+3. Accept terms and conditions
+4. Click Submit</t>
+        </is>
+      </c>
+      <c r="G169" s="5" t="inlineStr">
+        <is>
+          <t>Application submitted, status shows 'pending_approval'</t>
+        </is>
+      </c>
+      <c r="H169" s="5" t="inlineStr"/>
+      <c r="I169" s="5" t="inlineStr"/>
+      <c r="J169" s="5" t="inlineStr"/>
+      <c r="K169" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L169" s="5" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>TC159</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>Save Progress</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>Save Onboarding Progress</t>
+        </is>
+      </c>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>1. Fill partial information
+2. Click Save Progress
+3. Logout
+4. Login again
+5. Continue from where left off</t>
+        </is>
+      </c>
+      <c r="G170" s="5" t="inlineStr">
+        <is>
+          <t>Progress saved, can resume onboarding</t>
+        </is>
+      </c>
+      <c r="H170" s="5" t="inlineStr"/>
+      <c r="I170" s="5" t="inlineStr"/>
+      <c r="J170" s="5" t="inlineStr"/>
+      <c r="K170" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L170" s="5" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>TC160</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>Real-time Updates</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard Real-time Order Updates</t>
+        </is>
+      </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>1. Keep dashboard open
+2. Have customer place order
+3. Verify order appears without refresh
+4. Check notification received</t>
+        </is>
+      </c>
+      <c r="G171" s="5" t="inlineStr">
+        <is>
+          <t>New order appears automatically on dashboard</t>
+        </is>
+      </c>
+      <c r="H171" s="5" t="inlineStr"/>
+      <c r="I171" s="5" t="inlineStr"/>
+      <c r="J171" s="5" t="inlineStr"/>
+      <c r="K171" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L171" s="5" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>TC161</t>
+        </is>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D172" s="5" t="inlineStr">
+        <is>
+          <t>Performance Chart</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>View Performance Charts</t>
+        </is>
+      </c>
+      <c r="F172" s="5" t="inlineStr">
+        <is>
+          <t>1. On dashboard, scroll to charts
+2. View orders chart
+3. View earnings chart
+4. Hover for detailed values</t>
+        </is>
+      </c>
+      <c r="G172" s="5" t="inlineStr">
+        <is>
+          <t>Charts display correctly with accurate data</t>
+        </is>
+      </c>
+      <c r="H172" s="5" t="inlineStr"/>
+      <c r="I172" s="5" t="inlineStr"/>
+      <c r="J172" s="5" t="inlineStr"/>
+      <c r="K172" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L172" s="5" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>TC162</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>Recent Orders</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>View Recent Orders on Dashboard</t>
+        </is>
+      </c>
+      <c r="F173" s="5" t="inlineStr">
+        <is>
+          <t>1. Look at Recent Orders section
+2. Click View All
+3. Verify navigation to Orders page</t>
+        </is>
+      </c>
+      <c r="G173" s="5" t="inlineStr">
+        <is>
+          <t>Recent orders displayed, click navigates to full orders page</t>
+        </is>
+      </c>
+      <c r="H173" s="5" t="inlineStr"/>
+      <c r="I173" s="5" t="inlineStr"/>
+      <c r="J173" s="5" t="inlineStr"/>
+      <c r="K173" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L173" s="5" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="inlineStr">
+        <is>
+          <t>TC163</t>
+        </is>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D174" s="5" t="inlineStr">
+        <is>
+          <t>Quick Stats</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard Quick Stats Cards</t>
+        </is>
+      </c>
+      <c r="F174" s="5" t="inlineStr">
+        <is>
+          <t>1. Verify Today's Orders card
+2. Verify Today's Earnings card
+3. Verify Weekly Total card
+4. Verify Rating card
+5. Check all values are accurate</t>
+        </is>
+      </c>
+      <c r="G174" s="5" t="inlineStr">
+        <is>
+          <t>All stat cards show correct information</t>
+        </is>
+      </c>
+      <c r="H174" s="5" t="inlineStr"/>
+      <c r="I174" s="5" t="inlineStr"/>
+      <c r="J174" s="5" t="inlineStr"/>
+      <c r="K174" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L174" s="5" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>TC164</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Actions</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Order Actions</t>
+        </is>
+      </c>
+      <c r="F175" s="5" t="inlineStr">
+        <is>
+          <t>1. Select multiple orders
+2. Click bulk action
+3. Mark all as preparing
+4. Verify all updated</t>
+        </is>
+      </c>
+      <c r="G175" s="5" t="inlineStr">
+        <is>
+          <t>All selected orders updated to new status</t>
+        </is>
+      </c>
+      <c r="H175" s="5" t="inlineStr"/>
+      <c r="I175" s="5" t="inlineStr"/>
+      <c r="J175" s="5" t="inlineStr"/>
+      <c r="K175" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L175" s="5" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="inlineStr">
+        <is>
+          <t>TC165</t>
+        </is>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D176" s="5" t="inlineStr">
+        <is>
+          <t>Filter by Status</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>Filter Orders by Status</t>
+        </is>
+      </c>
+      <c r="F176" s="5" t="inlineStr">
+        <is>
+          <t>1. On orders page
+2. Click filter dropdown
+3. Select 'Preparing'
+4. Verify only preparing orders shown</t>
+        </is>
+      </c>
+      <c r="G176" s="5" t="inlineStr">
+        <is>
+          <t>Orders filtered by selected status</t>
+        </is>
+      </c>
+      <c r="H176" s="5" t="inlineStr"/>
+      <c r="I176" s="5" t="inlineStr"/>
+      <c r="J176" s="5" t="inlineStr"/>
+      <c r="K176" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L176" s="5" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>TC166</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>Filter by Date</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>Filter Orders by Date Range</t>
+        </is>
+      </c>
+      <c r="F177" s="5" t="inlineStr">
+        <is>
+          <t>1. Select date range
+2. Apply filter
+3. Verify orders within range displayed</t>
+        </is>
+      </c>
+      <c r="G177" s="5" t="inlineStr">
+        <is>
+          <t>Orders filtered by date range</t>
+        </is>
+      </c>
+      <c r="H177" s="5" t="inlineStr"/>
+      <c r="I177" s="5" t="inlineStr"/>
+      <c r="J177" s="5" t="inlineStr"/>
+      <c r="K177" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L177" s="5" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>TC167</t>
+        </is>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D178" s="5" t="inlineStr">
+        <is>
+          <t>Search Orders</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>Search Orders by Order ID or Customer</t>
+        </is>
+      </c>
+      <c r="F178" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter order ID in search
+2. Press Enter
+3. Verify matching order displayed
+4. Try searching by customer name</t>
+        </is>
+      </c>
+      <c r="G178" s="5" t="inlineStr">
+        <is>
+          <t>Search results show matching orders</t>
+        </is>
+      </c>
+      <c r="H178" s="5" t="inlineStr"/>
+      <c r="I178" s="5" t="inlineStr"/>
+      <c r="J178" s="5" t="inlineStr"/>
+      <c r="K178" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L178" s="5" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>TC168</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>Order Timeline</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>View Order Status Timeline</t>
+        </is>
+      </c>
+      <c r="F179" s="5" t="inlineStr">
+        <is>
+          <t>1. Open order details
+2. View status timeline
+3. Check all status changes logged
+4. Verify timestamps accurate</t>
+        </is>
+      </c>
+      <c r="G179" s="5" t="inlineStr">
+        <is>
+          <t>Complete timeline of order status changes shown</t>
+        </is>
+      </c>
+      <c r="H179" s="5" t="inlineStr"/>
+      <c r="I179" s="5" t="inlineStr"/>
+      <c r="J179" s="5" t="inlineStr"/>
+      <c r="K179" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L179" s="5" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="5" t="inlineStr">
+        <is>
+          <t>TC169</t>
+        </is>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D180" s="5" t="inlineStr">
+        <is>
+          <t>Customer Details</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>View Customer Details in Order</t>
+        </is>
+      </c>
+      <c r="F180" s="5" t="inlineStr">
+        <is>
+          <t>1. Open order details
+2. View customer section
+3. Verify name, phone, address shown
+4. Check delivery instructions</t>
+        </is>
+      </c>
+      <c r="G180" s="5" t="inlineStr">
+        <is>
+          <t>All customer information displayed accurately</t>
+        </is>
+      </c>
+      <c r="H180" s="5" t="inlineStr"/>
+      <c r="I180" s="5" t="inlineStr"/>
+      <c r="J180" s="5" t="inlineStr"/>
+      <c r="K180" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L180" s="5" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>TC170</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>Print Order</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>Print Order Ticket</t>
+        </is>
+      </c>
+      <c r="F181" s="5" t="inlineStr">
+        <is>
+          <t>1. Open order details
+2. Click Print button
+3. Verify print dialog opens
+4. Check ticket format</t>
+        </is>
+      </c>
+      <c r="G181" s="5" t="inlineStr">
+        <is>
+          <t>Print dialog opens with kitchen-friendly format</t>
+        </is>
+      </c>
+      <c r="H181" s="5" t="inlineStr"/>
+      <c r="I181" s="5" t="inlineStr"/>
+      <c r="J181" s="5" t="inlineStr"/>
+      <c r="K181" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L181" s="5" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="inlineStr">
+        <is>
+          <t>TC171</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D182" s="5" t="inlineStr">
+        <is>
+          <t>Order Notifications</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>Order Notification Settings</t>
+        </is>
+      </c>
+      <c r="F182" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Check notification settings
+3. Enable/disable order notifications
+4. Save settings</t>
+        </is>
+      </c>
+      <c r="G182" s="5" t="inlineStr">
+        <is>
+          <t>Notification preferences saved and applied</t>
+        </is>
+      </c>
+      <c r="H182" s="5" t="inlineStr"/>
+      <c r="I182" s="5" t="inlineStr"/>
+      <c r="J182" s="5" t="inlineStr"/>
+      <c r="K182" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L182" s="5" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>TC172</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Toggle</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Toggle Item Availability</t>
+        </is>
+      </c>
+      <c r="F183" s="5" t="inlineStr">
+        <is>
+          <t>1. Select multiple menu items
+2. Click Toggle Availability
+3. Verify all items status changed</t>
+        </is>
+      </c>
+      <c r="G183" s="5" t="inlineStr">
+        <is>
+          <t>All selected items availability toggled</t>
+        </is>
+      </c>
+      <c r="H183" s="5" t="inlineStr"/>
+      <c r="I183" s="5" t="inlineStr"/>
+      <c r="J183" s="5" t="inlineStr"/>
+      <c r="K183" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L183" s="5" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="inlineStr">
+        <is>
+          <t>TC173</t>
+        </is>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D184" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate Item</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate Menu Item</t>
+        </is>
+      </c>
+      <c r="F184" s="5" t="inlineStr">
+        <is>
+          <t>1. Find existing item
+2. Click Duplicate
+3. Modify details
+4. Save as new item</t>
+        </is>
+      </c>
+      <c r="G184" s="5" t="inlineStr">
+        <is>
+          <t>Item duplicated with editable copy</t>
+        </is>
+      </c>
+      <c r="H184" s="5" t="inlineStr"/>
+      <c r="I184" s="5" t="inlineStr"/>
+      <c r="J184" s="5" t="inlineStr"/>
+      <c r="K184" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L184" s="5" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>TC174</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>Image Crop</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>Crop Uploaded Image</t>
+        </is>
+      </c>
+      <c r="F185" s="5" t="inlineStr">
+        <is>
+          <t>1. Upload meal photo
+2. Click crop tool
+3. Adjust crop area
+4. Save cropped image</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>Image cropped and saved correctly</t>
+        </is>
+      </c>
+      <c r="H185" s="5" t="inlineStr"/>
+      <c r="I185" s="5" t="inlineStr"/>
+      <c r="J185" s="5" t="inlineStr"/>
+      <c r="K185" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L185" s="5" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="5" t="inlineStr">
+        <is>
+          <t>TC175</t>
+        </is>
+      </c>
+      <c r="B186" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D186" s="5" t="inlineStr">
+        <is>
+          <t>Nutrition Calculator</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>Use Nutrition Calculator</t>
+        </is>
+      </c>
+      <c r="F186" s="5" t="inlineStr">
+        <is>
+          <t>1. Add new meal
+2. Enter ingredients
+3. Use nutrition calculator
+4. Verify auto-calculated values</t>
+        </is>
+      </c>
+      <c r="G186" s="5" t="inlineStr">
+        <is>
+          <t>Nutrition values auto-calculated from ingredients</t>
+        </is>
+      </c>
+      <c r="H186" s="5" t="inlineStr"/>
+      <c r="I186" s="5" t="inlineStr"/>
+      <c r="J186" s="5" t="inlineStr"/>
+      <c r="K186" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L186" s="5" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>TC176</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>Menu Categories</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>Organize Menu by Categories</t>
+        </is>
+      </c>
+      <c r="F187" s="5" t="inlineStr">
+        <is>
+          <t>1. Create category (e.g., 'Main Course')
+2. Assign meals to category
+3. View menu by category
+4. Reorder categories</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>Meals organized by categories</t>
+        </is>
+      </c>
+      <c r="H187" s="5" t="inlineStr"/>
+      <c r="I187" s="5" t="inlineStr"/>
+      <c r="J187" s="5" t="inlineStr"/>
+      <c r="K187" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L187" s="5" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="inlineStr">
+        <is>
+          <t>TC177</t>
+        </is>
+      </c>
+      <c r="B188" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D188" s="5" t="inlineStr">
+        <is>
+          <t>Preview Menu</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>Preview Menu as Customer Sees It</t>
+        </is>
+      </c>
+      <c r="F188" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Preview button
+2. View menu as customer sees it
+3. Verify all items display correctly
+4. Check photos and descriptions</t>
+        </is>
+      </c>
+      <c r="G188" s="5" t="inlineStr">
+        <is>
+          <t>Menu preview matches customer view</t>
+        </is>
+      </c>
+      <c r="H188" s="5" t="inlineStr"/>
+      <c r="I188" s="5" t="inlineStr"/>
+      <c r="J188" s="5" t="inlineStr"/>
+      <c r="K188" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L188" s="5" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>TC178</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>Export Menu</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>Export Menu Data</t>
+        </is>
+      </c>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to menu
+2. Click Export
+3. Select format (CSV/Excel)
+4. Download file</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>Menu data exported successfully</t>
+        </is>
+      </c>
+      <c r="H189" s="5" t="inlineStr"/>
+      <c r="I189" s="5" t="inlineStr"/>
+      <c r="J189" s="5" t="inlineStr"/>
+      <c r="K189" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L189" s="5" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="inlineStr">
+        <is>
+          <t>TC179</t>
+        </is>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>Import Menu</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr">
+        <is>
+          <t>Import Menu Items</t>
+        </is>
+      </c>
+      <c r="F190" s="5" t="inlineStr">
+        <is>
+          <t>1. Prepare import file
+2. Click Import
+3. Upload file
+4. Map fields
+5. Complete import</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t>Menu items imported successfully</t>
+        </is>
+      </c>
+      <c r="H190" s="5" t="inlineStr"/>
+      <c r="I190" s="5" t="inlineStr"/>
+      <c r="J190" s="5" t="inlineStr"/>
+      <c r="K190" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L190" s="5" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>TC180</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>Earnings Chart</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>View Earnings Chart</t>
+        </is>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to earnings page
+2. View earnings chart
+3. Switch between daily/weekly/monthly views
+4. Hover for detailed values</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>Chart displays earnings trends accurately</t>
+        </is>
+      </c>
+      <c r="H191" s="5" t="inlineStr"/>
+      <c r="I191" s="5" t="inlineStr"/>
+      <c r="J191" s="5" t="inlineStr"/>
+      <c r="K191" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L191" s="5" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="inlineStr">
+        <is>
+          <t>TC181</t>
+        </is>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>Top Meals</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>View Top Performing Meals</t>
+        </is>
+      </c>
+      <c r="F192" s="5" t="inlineStr">
+        <is>
+          <t>1. Scroll to Top Meals section
+2. View best-selling items
+3. Check quantities sold
+4. View revenue per item</t>
+        </is>
+      </c>
+      <c r="G192" s="5" t="inlineStr">
+        <is>
+          <t>Top performing meals displayed with stats</t>
+        </is>
+      </c>
+      <c r="H192" s="5" t="inlineStr"/>
+      <c r="I192" s="5" t="inlineStr"/>
+      <c r="J192" s="5" t="inlineStr"/>
+      <c r="K192" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L192" s="5" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>TC182</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>Payout Invoice</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>Download Payout Invoice</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to payout history
+2. Click on payout
+3. Click Download Invoice
+4. Verify PDF contains correct details</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>Invoice downloaded with accurate information</t>
+        </is>
+      </c>
+      <c r="H193" s="5" t="inlineStr"/>
+      <c r="I193" s="5" t="inlineStr"/>
+      <c r="J193" s="5" t="inlineStr"/>
+      <c r="K193" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L193" s="5" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="inlineStr">
+        <is>
+          <t>TC183</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>Dispute Payout</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>Dispute a Payout</t>
+        </is>
+      </c>
+      <c r="F194" s="5" t="inlineStr">
+        <is>
+          <t>1. Find payout in history
+2. Click Dispute
+3. Enter reason
+4. Submit dispute
+5. Verify confirmation</t>
+        </is>
+      </c>
+      <c r="G194" s="5" t="inlineStr">
+        <is>
+          <t>Dispute submitted, under review status shown</t>
+        </is>
+      </c>
+      <c r="H194" s="5" t="inlineStr"/>
+      <c r="I194" s="5" t="inlineStr"/>
+      <c r="J194" s="5" t="inlineStr"/>
+      <c r="K194" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L194" s="5" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="inlineStr">
+        <is>
+          <t>TC184</t>
+        </is>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>Tax Report</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>Generate Tax Report</t>
+        </is>
+      </c>
+      <c r="F195" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to earnings
+2. Click Tax Report
+3. Select year
+4. Generate report
+5. Download PDF</t>
+        </is>
+      </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>Tax report generated with all earnings data</t>
+        </is>
+      </c>
+      <c r="H195" s="5" t="inlineStr"/>
+      <c r="I195" s="5" t="inlineStr"/>
+      <c r="J195" s="5" t="inlineStr"/>
+      <c r="K195" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L195" s="5" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="5" t="inlineStr">
+        <is>
+          <t>TC185</t>
+        </is>
+      </c>
+      <c r="B196" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D196" s="5" t="inlineStr">
+        <is>
+          <t>Compare Periods</t>
+        </is>
+      </c>
+      <c r="E196" s="5" t="inlineStr">
+        <is>
+          <t>Compare Earnings Periods</t>
+        </is>
+      </c>
+      <c r="F196" s="5" t="inlineStr">
+        <is>
+          <t>1. Select first period
+2. Select comparison period
+3. View comparison chart
+4. Analyze differences</t>
+        </is>
+      </c>
+      <c r="G196" s="5" t="inlineStr">
+        <is>
+          <t>Period comparison displayed with growth/decline metrics</t>
+        </is>
+      </c>
+      <c r="H196" s="5" t="inlineStr"/>
+      <c r="I196" s="5" t="inlineStr"/>
+      <c r="J196" s="5" t="inlineStr"/>
+      <c r="K196" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L196" s="5" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="inlineStr">
+        <is>
+          <t>TC186</t>
+        </is>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D197" s="5" t="inlineStr">
+        <is>
+          <t>Change Password</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>Change Account Password</t>
+        </is>
+      </c>
+      <c r="F197" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Click Change Password
+3. Enter current password
+4. Enter new password
+5. Confirm
+6. Logout and test new password</t>
+        </is>
+      </c>
+      <c r="G197" s="5" t="inlineStr">
+        <is>
+          <t>Password changed successfully</t>
+        </is>
+      </c>
+      <c r="H197" s="5" t="inlineStr"/>
+      <c r="I197" s="5" t="inlineStr"/>
+      <c r="J197" s="5" t="inlineStr"/>
+      <c r="K197" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L197" s="5" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="5" t="inlineStr">
+        <is>
+          <t>TC187</t>
+        </is>
+      </c>
+      <c r="B198" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D198" s="5" t="inlineStr">
+        <is>
+          <t>Two-Factor Auth</t>
+        </is>
+      </c>
+      <c r="E198" s="5" t="inlineStr">
+        <is>
+          <t>Enable Two-Factor Authentication</t>
+        </is>
+      </c>
+      <c r="F198" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to security settings
+2. Enable 2FA
+3. Scan QR code
+4. Enter verification code
+5. Save backup codes</t>
+        </is>
+      </c>
+      <c r="G198" s="5" t="inlineStr">
+        <is>
+          <t>2FA enabled, backup codes provided</t>
+        </is>
+      </c>
+      <c r="H198" s="5" t="inlineStr"/>
+      <c r="I198" s="5" t="inlineStr"/>
+      <c r="J198" s="5" t="inlineStr"/>
+      <c r="K198" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L198" s="5" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="inlineStr">
+        <is>
+          <t>TC188</t>
+        </is>
+      </c>
+      <c r="B199" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D199" s="5" t="inlineStr">
+        <is>
+          <t>Notification Preferences</t>
+        </is>
+      </c>
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>Set Notification Preferences</t>
+        </is>
+      </c>
+      <c r="F199" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Click Notifications
+3. Toggle email notifications
+4. Toggle WhatsApp notifications
+5. Set quiet hours</t>
+        </is>
+      </c>
+      <c r="G199" s="5" t="inlineStr">
+        <is>
+          <t>Notification preferences saved</t>
+        </is>
+      </c>
+      <c r="H199" s="5" t="inlineStr"/>
+      <c r="I199" s="5" t="inlineStr"/>
+      <c r="J199" s="5" t="inlineStr"/>
+      <c r="K199" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L199" s="5" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="5" t="inlineStr">
+        <is>
+          <t>TC189</t>
+        </is>
+      </c>
+      <c r="B200" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D200" s="5" t="inlineStr">
+        <is>
+          <t>API Access</t>
+        </is>
+      </c>
+      <c r="E200" s="5" t="inlineStr">
+        <is>
+          <t>Generate API Key</t>
+        </is>
+      </c>
+      <c r="F200" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Click API Access
+3. Generate new key
+4. Copy and save key
+5. View API documentation</t>
+        </is>
+      </c>
+      <c r="G200" s="5" t="inlineStr">
+        <is>
+          <t>API key generated and displayed</t>
+        </is>
+      </c>
+      <c r="H200" s="5" t="inlineStr"/>
+      <c r="I200" s="5" t="inlineStr"/>
+      <c r="J200" s="5" t="inlineStr"/>
+      <c r="K200" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L200" s="5" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="5" t="inlineStr">
+        <is>
+          <t>TC190</t>
+        </is>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C201" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D201" s="5" t="inlineStr">
+        <is>
+          <t>Business Hours</t>
+        </is>
+      </c>
+      <c r="E201" s="5" t="inlineStr">
+        <is>
+          <t>Set Special Hours</t>
+        </is>
+      </c>
+      <c r="F201" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to operating hours
+2. Set regular hours
+3. Add special hours (holidays)
+4. Mark temporary closures
+5. Save</t>
+        </is>
+      </c>
+      <c r="G201" s="5" t="inlineStr">
+        <is>
+          <t>Special hours saved and applied</t>
+        </is>
+      </c>
+      <c r="H201" s="5" t="inlineStr"/>
+      <c r="I201" s="5" t="inlineStr"/>
+      <c r="J201" s="5" t="inlineStr"/>
+      <c r="K201" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L201" s="5" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="5" t="inlineStr">
+        <is>
+          <t>TC191</t>
+        </is>
+      </c>
+      <c r="B202" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C202" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D202" s="5" t="inlineStr">
+        <is>
+          <t>Delivery Zones</t>
+        </is>
+      </c>
+      <c r="E202" s="5" t="inlineStr">
+        <is>
+          <t>Set Delivery Zones</t>
+        </is>
+      </c>
+      <c r="F202" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to delivery settings
+2. View map
+3. Draw delivery zone
+4. Set minimum order
+5. Set delivery fee
+6. Save</t>
+        </is>
+      </c>
+      <c r="G202" s="5" t="inlineStr">
+        <is>
+          <t>Delivery zone saved and shown on map</t>
+        </is>
+      </c>
+      <c r="H202" s="5" t="inlineStr"/>
+      <c r="I202" s="5" t="inlineStr"/>
+      <c r="J202" s="5" t="inlineStr"/>
+      <c r="K202" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L202" s="5" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="5" t="inlineStr">
+        <is>
+          <t>TC192</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D203" s="5" t="inlineStr">
+        <is>
+          <t>Team Members</t>
+        </is>
+      </c>
+      <c r="E203" s="5" t="inlineStr">
+        <is>
+          <t>Add Team Members</t>
+        </is>
+      </c>
+      <c r="F203" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to team management
+2. Click Add Member
+3. Enter email
+4. Set role (Admin/Staff)
+5. Send invitation</t>
+        </is>
+      </c>
+      <c r="G203" s="5" t="inlineStr">
+        <is>
+          <t>Invitation sent, member can access with limited permissions</t>
+        </is>
+      </c>
+      <c r="H203" s="5" t="inlineStr"/>
+      <c r="I203" s="5" t="inlineStr"/>
+      <c r="J203" s="5" t="inlineStr"/>
+      <c r="K203" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L203" s="5" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="5" t="inlineStr">
+        <is>
+          <t>TC193</t>
+        </is>
+      </c>
+      <c r="B204" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D204" s="5" t="inlineStr">
+        <is>
+          <t>Remove Team Member</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="inlineStr">
+        <is>
+          <t>Remove Team Member</t>
+        </is>
+      </c>
+      <c r="F204" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to team management
+2. Find member
+3. Click Remove
+4. Confirm removal</t>
+        </is>
+      </c>
+      <c r="G204" s="5" t="inlineStr">
+        <is>
+          <t>Member removed, access revoked</t>
+        </is>
+      </c>
+      <c r="H204" s="5" t="inlineStr"/>
+      <c r="I204" s="5" t="inlineStr"/>
+      <c r="J204" s="5" t="inlineStr"/>
+      <c r="K204" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L204" s="5" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="inlineStr">
+        <is>
+          <t>TC194</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D205" s="5" t="inlineStr">
+        <is>
+          <t>View Analytics</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>View Business Analytics</t>
+        </is>
+      </c>
+      <c r="F205" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to Analytics page
+2. View order trends
+3. View customer insights
+4. View peak hours
+5. Export analytics report</t>
+        </is>
+      </c>
+      <c r="G205" s="5" t="inlineStr">
+        <is>
+          <t>Analytics displayed with actionable insights</t>
+        </is>
+      </c>
+      <c r="H205" s="5" t="inlineStr"/>
+      <c r="I205" s="5" t="inlineStr"/>
+      <c r="J205" s="5" t="inlineStr"/>
+      <c r="K205" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L205" s="5" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="inlineStr">
+        <is>
+          <t>TC195</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D206" s="5" t="inlineStr">
+        <is>
+          <t>Customer Feedback</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="inlineStr">
+        <is>
+          <t>View Customer Feedback</t>
+        </is>
+      </c>
+      <c r="F206" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to Reviews section
+2. View all customer reviews
+3. Filter by rating
+4. Respond to review
+5. Mark as resolved</t>
+        </is>
+      </c>
+      <c r="G206" s="5" t="inlineStr">
+        <is>
+          <t>Reviews displayed, can respond to customers</t>
+        </is>
+      </c>
+      <c r="H206" s="5" t="inlineStr"/>
+      <c r="I206" s="5" t="inlineStr"/>
+      <c r="J206" s="5" t="inlineStr"/>
+      <c r="K206" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L206" s="5" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="inlineStr">
+        <is>
+          <t>TC196</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D207" s="5" t="inlineStr">
+        <is>
+          <t>Performance Metrics</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>View Detailed Performance Metrics</t>
+        </is>
+      </c>
+      <c r="F207" s="5" t="inlineStr">
+        <is>
+          <t>1. View order fulfillment rate
+2. View average prep time
+3. View on-time delivery rate
+4. Compare with industry average</t>
+        </is>
+      </c>
+      <c r="G207" s="5" t="inlineStr">
+        <is>
+          <t>All performance metrics displayed</t>
+        </is>
+      </c>
+      <c r="H207" s="5" t="inlineStr"/>
+      <c r="I207" s="5" t="inlineStr"/>
+      <c r="J207" s="5" t="inlineStr"/>
+      <c r="K207" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L207" s="5" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="inlineStr">
+        <is>
+          <t>TC197</t>
+        </is>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D208" s="5" t="inlineStr">
+        <is>
+          <t>Contact Support</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
+        <is>
+          <t>Contact Support via Dashboard</t>
+        </is>
+      </c>
+      <c r="F208" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Support button
+2. Select issue type
+3. Describe problem
+4. Attach screenshot
+5. Submit ticket</t>
+        </is>
+      </c>
+      <c r="G208" s="5" t="inlineStr">
+        <is>
+          <t>Support ticket created, confirmation shown</t>
+        </is>
+      </c>
+      <c r="H208" s="5" t="inlineStr"/>
+      <c r="I208" s="5" t="inlineStr"/>
+      <c r="J208" s="5" t="inlineStr"/>
+      <c r="K208" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L208" s="5" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="5" t="inlineStr">
+        <is>
+          <t>TC198</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D209" s="5" t="inlineStr">
+        <is>
+          <t>View Knowledge Base</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>Access Knowledge Base</t>
+        </is>
+      </c>
+      <c r="F209" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Help
+2. Browse articles
+3. Search for topic
+4. View article</t>
+        </is>
+      </c>
+      <c r="G209" s="5" t="inlineStr">
+        <is>
+          <t>Knowledge base articles displayed</t>
+        </is>
+      </c>
+      <c r="H209" s="5" t="inlineStr"/>
+      <c r="I209" s="5" t="inlineStr"/>
+      <c r="J209" s="5" t="inlineStr"/>
+      <c r="K209" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L209" s="5" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="5" t="inlineStr">
+        <is>
+          <t>TC199</t>
+        </is>
+      </c>
+      <c r="B210" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C210" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D210" s="5" t="inlineStr">
+        <is>
+          <t>Live Chat</t>
+        </is>
+      </c>
+      <c r="E210" s="5" t="inlineStr">
+        <is>
+          <t>Start Live Chat</t>
+        </is>
+      </c>
+      <c r="F210" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Chat icon
+2. Start conversation
+3. Send message
+4. Receive response</t>
+        </is>
+      </c>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>Chat connected, messages exchanged</t>
+        </is>
+      </c>
+      <c r="H210" s="5" t="inlineStr"/>
+      <c r="I210" s="5" t="inlineStr"/>
+      <c r="J210" s="5" t="inlineStr"/>
+      <c r="K210" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L210" s="5" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="5" t="inlineStr">
+        <is>
+          <t>TC153</t>
+        </is>
+      </c>
+      <c r="B211" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C211" s="5" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D211" s="5" t="inlineStr">
+        <is>
+          <t>Password Reset</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="inlineStr">
+        <is>
+          <t>Partner Password Reset Flow</t>
+        </is>
+      </c>
+      <c r="F211" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Forgot Password on partner login
+2. Enter registered email
+3. Check email for reset link
+4. Click link and set new password
+5. Login with new password</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t>Password reset successful, can login with new credentials</t>
+        </is>
+      </c>
+      <c r="H211" s="5" t="inlineStr"/>
+      <c r="I211" s="5" t="inlineStr"/>
+      <c r="J211" s="5" t="inlineStr"/>
+      <c r="K211" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L211" s="5" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="5" t="inlineStr">
+        <is>
+          <t>TC154</t>
+        </is>
+      </c>
+      <c r="B212" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C212" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D212" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 1</t>
+        </is>
+      </c>
+      <c r="E212" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 1 - Basic Info</t>
+        </is>
+      </c>
+      <c r="F212" s="5" t="inlineStr">
+        <is>
+          <t>1. Start partner registration
+2. Fill restaurant name
+3. Add description
+4. Select cuisine type
+5. Add dietary tags</t>
+        </is>
+      </c>
+      <c r="G212" s="5" t="inlineStr">
+        <is>
+          <t>Step 1 saved, can proceed to Step 2</t>
+        </is>
+      </c>
+      <c r="H212" s="5" t="inlineStr"/>
+      <c r="I212" s="5" t="inlineStr"/>
+      <c r="J212" s="5" t="inlineStr"/>
+      <c r="K212" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L212" s="5" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="5" t="inlineStr">
+        <is>
+          <t>TC155</t>
+        </is>
+      </c>
+      <c r="B213" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C213" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D213" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 2</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 2 - Location</t>
+        </is>
+      </c>
+      <c r="F213" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter address
+2. Pin location on map
+3. Add phone number
+4. Add email
+5. Set operating hours</t>
+        </is>
+      </c>
+      <c r="G213" s="5" t="inlineStr">
+        <is>
+          <t>Step 2 saved, can proceed to Step 3</t>
+        </is>
+      </c>
+      <c r="H213" s="5" t="inlineStr"/>
+      <c r="I213" s="5" t="inlineStr"/>
+      <c r="J213" s="5" t="inlineStr"/>
+      <c r="K213" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L213" s="5" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="5" t="inlineStr">
+        <is>
+          <t>TC156</t>
+        </is>
+      </c>
+      <c r="B214" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C214" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D214" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 3</t>
+        </is>
+      </c>
+      <c r="E214" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 3 - Media</t>
+        </is>
+      </c>
+      <c r="F214" s="5" t="inlineStr">
+        <is>
+          <t>1. Upload logo (required)
+2. Upload restaurant photos
+3. Verify image preview
+4. Check file size limits</t>
+        </is>
+      </c>
+      <c r="G214" s="5" t="inlineStr">
+        <is>
+          <t>Images uploaded and preview shown</t>
+        </is>
+      </c>
+      <c r="H214" s="5" t="inlineStr"/>
+      <c r="I214" s="5" t="inlineStr"/>
+      <c r="J214" s="5" t="inlineStr"/>
+      <c r="K214" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L214" s="5" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="5" t="inlineStr">
+        <is>
+          <t>TC157</t>
+        </is>
+      </c>
+      <c r="B215" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C215" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D215" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 4</t>
+        </is>
+      </c>
+      <c r="E215" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 4 - Kitchen Details</t>
+        </is>
+      </c>
+      <c r="F215" s="5" t="inlineStr">
+        <is>
+          <t>1. Set average prep time
+2. Set daily capacity
+3. Add bank account info
+4. Add bank name and IBAN</t>
+        </is>
+      </c>
+      <c r="G215" s="5" t="inlineStr">
+        <is>
+          <t>Kitchen details saved, can proceed to Step 5</t>
+        </is>
+      </c>
+      <c r="H215" s="5" t="inlineStr"/>
+      <c r="I215" s="5" t="inlineStr"/>
+      <c r="J215" s="5" t="inlineStr"/>
+      <c r="K215" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L215" s="5" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="5" t="inlineStr">
+        <is>
+          <t>TC158</t>
+        </is>
+      </c>
+      <c r="B216" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C216" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D216" s="5" t="inlineStr">
+        <is>
+          <t>Wizard Step 5</t>
+        </is>
+      </c>
+      <c r="E216" s="5" t="inlineStr">
+        <is>
+          <t>Complete Onboarding Step 5 - Review &amp; Submit</t>
+        </is>
+      </c>
+      <c r="F216" s="5" t="inlineStr">
+        <is>
+          <t>1. Review all entered information
+2. Check accuracy of details
+3. Accept terms and conditions
+4. Click Submit</t>
+        </is>
+      </c>
+      <c r="G216" s="5" t="inlineStr">
+        <is>
+          <t>Application submitted, status shows 'pending_approval'</t>
+        </is>
+      </c>
+      <c r="H216" s="5" t="inlineStr"/>
+      <c r="I216" s="5" t="inlineStr"/>
+      <c r="J216" s="5" t="inlineStr"/>
+      <c r="K216" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L216" s="5" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="5" t="inlineStr">
+        <is>
+          <t>TC159</t>
+        </is>
+      </c>
+      <c r="B217" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C217" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="D217" s="5" t="inlineStr">
+        <is>
+          <t>Save Progress</t>
+        </is>
+      </c>
+      <c r="E217" s="5" t="inlineStr">
+        <is>
+          <t>Save Onboarding Progress</t>
+        </is>
+      </c>
+      <c r="F217" s="5" t="inlineStr">
+        <is>
+          <t>1. Fill partial information
+2. Click Save Progress
+3. Logout
+4. Login again
+5. Continue from where left off</t>
+        </is>
+      </c>
+      <c r="G217" s="5" t="inlineStr">
+        <is>
+          <t>Progress saved, can resume onboarding</t>
+        </is>
+      </c>
+      <c r="H217" s="5" t="inlineStr"/>
+      <c r="I217" s="5" t="inlineStr"/>
+      <c r="J217" s="5" t="inlineStr"/>
+      <c r="K217" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L217" s="5" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="5" t="inlineStr">
+        <is>
+          <t>TC160</t>
+        </is>
+      </c>
+      <c r="B218" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C218" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D218" s="5" t="inlineStr">
+        <is>
+          <t>Real-time Updates</t>
+        </is>
+      </c>
+      <c r="E218" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard Real-time Order Updates</t>
+        </is>
+      </c>
+      <c r="F218" s="5" t="inlineStr">
+        <is>
+          <t>1. Keep dashboard open
+2. Have customer place order
+3. Verify order appears without refresh
+4. Check notification received</t>
+        </is>
+      </c>
+      <c r="G218" s="5" t="inlineStr">
+        <is>
+          <t>New order appears automatically on dashboard</t>
+        </is>
+      </c>
+      <c r="H218" s="5" t="inlineStr"/>
+      <c r="I218" s="5" t="inlineStr"/>
+      <c r="J218" s="5" t="inlineStr"/>
+      <c r="K218" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L218" s="5" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="5" t="inlineStr">
+        <is>
+          <t>TC161</t>
+        </is>
+      </c>
+      <c r="B219" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C219" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D219" s="5" t="inlineStr">
+        <is>
+          <t>Performance Chart</t>
+        </is>
+      </c>
+      <c r="E219" s="5" t="inlineStr">
+        <is>
+          <t>View Performance Charts</t>
+        </is>
+      </c>
+      <c r="F219" s="5" t="inlineStr">
+        <is>
+          <t>1. On dashboard, scroll to charts
+2. View orders chart
+3. View earnings chart
+4. Hover for detailed values</t>
+        </is>
+      </c>
+      <c r="G219" s="5" t="inlineStr">
+        <is>
+          <t>Charts display correctly with accurate data</t>
+        </is>
+      </c>
+      <c r="H219" s="5" t="inlineStr"/>
+      <c r="I219" s="5" t="inlineStr"/>
+      <c r="J219" s="5" t="inlineStr"/>
+      <c r="K219" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L219" s="5" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="5" t="inlineStr">
+        <is>
+          <t>TC162</t>
+        </is>
+      </c>
+      <c r="B220" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C220" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D220" s="5" t="inlineStr">
+        <is>
+          <t>Recent Orders</t>
+        </is>
+      </c>
+      <c r="E220" s="5" t="inlineStr">
+        <is>
+          <t>View Recent Orders on Dashboard</t>
+        </is>
+      </c>
+      <c r="F220" s="5" t="inlineStr">
+        <is>
+          <t>1. Look at Recent Orders section
+2. Click View All
+3. Verify navigation to Orders page</t>
+        </is>
+      </c>
+      <c r="G220" s="5" t="inlineStr">
+        <is>
+          <t>Recent orders displayed, click navigates to full orders page</t>
+        </is>
+      </c>
+      <c r="H220" s="5" t="inlineStr"/>
+      <c r="I220" s="5" t="inlineStr"/>
+      <c r="J220" s="5" t="inlineStr"/>
+      <c r="K220" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L220" s="5" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="5" t="inlineStr">
+        <is>
+          <t>TC163</t>
+        </is>
+      </c>
+      <c r="B221" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C221" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D221" s="5" t="inlineStr">
+        <is>
+          <t>Quick Stats</t>
+        </is>
+      </c>
+      <c r="E221" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard Quick Stats Cards</t>
+        </is>
+      </c>
+      <c r="F221" s="5" t="inlineStr">
+        <is>
+          <t>1. Verify Today's Orders card
+2. Verify Today's Earnings card
+3. Verify Weekly Total card
+4. Verify Rating card
+5. Check all values are accurate</t>
+        </is>
+      </c>
+      <c r="G221" s="5" t="inlineStr">
+        <is>
+          <t>All stat cards show correct information</t>
+        </is>
+      </c>
+      <c r="H221" s="5" t="inlineStr"/>
+      <c r="I221" s="5" t="inlineStr"/>
+      <c r="J221" s="5" t="inlineStr"/>
+      <c r="K221" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L221" s="5" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="5" t="inlineStr">
+        <is>
+          <t>TC164</t>
+        </is>
+      </c>
+      <c r="B222" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C222" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D222" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Actions</t>
+        </is>
+      </c>
+      <c r="E222" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Order Actions</t>
+        </is>
+      </c>
+      <c r="F222" s="5" t="inlineStr">
+        <is>
+          <t>1. Select multiple orders
+2. Click bulk action
+3. Mark all as preparing
+4. Verify all updated</t>
+        </is>
+      </c>
+      <c r="G222" s="5" t="inlineStr">
+        <is>
+          <t>All selected orders updated to new status</t>
+        </is>
+      </c>
+      <c r="H222" s="5" t="inlineStr"/>
+      <c r="I222" s="5" t="inlineStr"/>
+      <c r="J222" s="5" t="inlineStr"/>
+      <c r="K222" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L222" s="5" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="5" t="inlineStr">
+        <is>
+          <t>TC165</t>
+        </is>
+      </c>
+      <c r="B223" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C223" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D223" s="5" t="inlineStr">
+        <is>
+          <t>Filter by Status</t>
+        </is>
+      </c>
+      <c r="E223" s="5" t="inlineStr">
+        <is>
+          <t>Filter Orders by Status</t>
+        </is>
+      </c>
+      <c r="F223" s="5" t="inlineStr">
+        <is>
+          <t>1. On orders page
+2. Click filter dropdown
+3. Select 'Preparing'
+4. Verify only preparing orders shown</t>
+        </is>
+      </c>
+      <c r="G223" s="5" t="inlineStr">
+        <is>
+          <t>Orders filtered by selected status</t>
+        </is>
+      </c>
+      <c r="H223" s="5" t="inlineStr"/>
+      <c r="I223" s="5" t="inlineStr"/>
+      <c r="J223" s="5" t="inlineStr"/>
+      <c r="K223" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L223" s="5" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="5" t="inlineStr">
+        <is>
+          <t>TC166</t>
+        </is>
+      </c>
+      <c r="B224" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C224" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D224" s="5" t="inlineStr">
+        <is>
+          <t>Filter by Date</t>
+        </is>
+      </c>
+      <c r="E224" s="5" t="inlineStr">
+        <is>
+          <t>Filter Orders by Date Range</t>
+        </is>
+      </c>
+      <c r="F224" s="5" t="inlineStr">
+        <is>
+          <t>1. Select date range
+2. Apply filter
+3. Verify orders within range displayed</t>
+        </is>
+      </c>
+      <c r="G224" s="5" t="inlineStr">
+        <is>
+          <t>Orders filtered by date range</t>
+        </is>
+      </c>
+      <c r="H224" s="5" t="inlineStr"/>
+      <c r="I224" s="5" t="inlineStr"/>
+      <c r="J224" s="5" t="inlineStr"/>
+      <c r="K224" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L224" s="5" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="5" t="inlineStr">
+        <is>
+          <t>TC167</t>
+        </is>
+      </c>
+      <c r="B225" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C225" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D225" s="5" t="inlineStr">
+        <is>
+          <t>Search Orders</t>
+        </is>
+      </c>
+      <c r="E225" s="5" t="inlineStr">
+        <is>
+          <t>Search Orders by Order ID or Customer</t>
+        </is>
+      </c>
+      <c r="F225" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter order ID in search
+2. Press Enter
+3. Verify matching order displayed
+4. Try searching by customer name</t>
+        </is>
+      </c>
+      <c r="G225" s="5" t="inlineStr">
+        <is>
+          <t>Search results show matching orders</t>
+        </is>
+      </c>
+      <c r="H225" s="5" t="inlineStr"/>
+      <c r="I225" s="5" t="inlineStr"/>
+      <c r="J225" s="5" t="inlineStr"/>
+      <c r="K225" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L225" s="5" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="5" t="inlineStr">
+        <is>
+          <t>TC168</t>
+        </is>
+      </c>
+      <c r="B226" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C226" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D226" s="5" t="inlineStr">
+        <is>
+          <t>Order Timeline</t>
+        </is>
+      </c>
+      <c r="E226" s="5" t="inlineStr">
+        <is>
+          <t>View Order Status Timeline</t>
+        </is>
+      </c>
+      <c r="F226" s="5" t="inlineStr">
+        <is>
+          <t>1. Open order details
+2. View status timeline
+3. Check all status changes logged
+4. Verify timestamps accurate</t>
+        </is>
+      </c>
+      <c r="G226" s="5" t="inlineStr">
+        <is>
+          <t>Complete timeline of order status changes shown</t>
+        </is>
+      </c>
+      <c r="H226" s="5" t="inlineStr"/>
+      <c r="I226" s="5" t="inlineStr"/>
+      <c r="J226" s="5" t="inlineStr"/>
+      <c r="K226" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L226" s="5" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="5" t="inlineStr">
+        <is>
+          <t>TC169</t>
+        </is>
+      </c>
+      <c r="B227" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C227" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D227" s="5" t="inlineStr">
+        <is>
+          <t>Customer Details</t>
+        </is>
+      </c>
+      <c r="E227" s="5" t="inlineStr">
+        <is>
+          <t>View Customer Details in Order</t>
+        </is>
+      </c>
+      <c r="F227" s="5" t="inlineStr">
+        <is>
+          <t>1. Open order details
+2. View customer section
+3. Verify name, phone, address shown
+4. Check delivery instructions</t>
+        </is>
+      </c>
+      <c r="G227" s="5" t="inlineStr">
+        <is>
+          <t>All customer information displayed accurately</t>
+        </is>
+      </c>
+      <c r="H227" s="5" t="inlineStr"/>
+      <c r="I227" s="5" t="inlineStr"/>
+      <c r="J227" s="5" t="inlineStr"/>
+      <c r="K227" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L227" s="5" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="5" t="inlineStr">
+        <is>
+          <t>TC170</t>
+        </is>
+      </c>
+      <c r="B228" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C228" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D228" s="5" t="inlineStr">
+        <is>
+          <t>Print Order</t>
+        </is>
+      </c>
+      <c r="E228" s="5" t="inlineStr">
+        <is>
+          <t>Print Order Ticket</t>
+        </is>
+      </c>
+      <c r="F228" s="5" t="inlineStr">
+        <is>
+          <t>1. Open order details
+2. Click Print button
+3. Verify print dialog opens
+4. Check ticket format</t>
+        </is>
+      </c>
+      <c r="G228" s="5" t="inlineStr">
+        <is>
+          <t>Print dialog opens with kitchen-friendly format</t>
+        </is>
+      </c>
+      <c r="H228" s="5" t="inlineStr"/>
+      <c r="I228" s="5" t="inlineStr"/>
+      <c r="J228" s="5" t="inlineStr"/>
+      <c r="K228" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L228" s="5" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="5" t="inlineStr">
+        <is>
+          <t>TC171</t>
+        </is>
+      </c>
+      <c r="B229" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C229" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="D229" s="5" t="inlineStr">
+        <is>
+          <t>Order Notifications</t>
+        </is>
+      </c>
+      <c r="E229" s="5" t="inlineStr">
+        <is>
+          <t>Order Notification Settings</t>
+        </is>
+      </c>
+      <c r="F229" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Check notification settings
+3. Enable/disable order notifications
+4. Save settings</t>
+        </is>
+      </c>
+      <c r="G229" s="5" t="inlineStr">
+        <is>
+          <t>Notification preferences saved and applied</t>
+        </is>
+      </c>
+      <c r="H229" s="5" t="inlineStr"/>
+      <c r="I229" s="5" t="inlineStr"/>
+      <c r="J229" s="5" t="inlineStr"/>
+      <c r="K229" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L229" s="5" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="5" t="inlineStr">
+        <is>
+          <t>TC172</t>
+        </is>
+      </c>
+      <c r="B230" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C230" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D230" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Toggle</t>
+        </is>
+      </c>
+      <c r="E230" s="5" t="inlineStr">
+        <is>
+          <t>Bulk Toggle Item Availability</t>
+        </is>
+      </c>
+      <c r="F230" s="5" t="inlineStr">
+        <is>
+          <t>1. Select multiple menu items
+2. Click Toggle Availability
+3. Verify all items status changed</t>
+        </is>
+      </c>
+      <c r="G230" s="5" t="inlineStr">
+        <is>
+          <t>All selected items availability toggled</t>
+        </is>
+      </c>
+      <c r="H230" s="5" t="inlineStr"/>
+      <c r="I230" s="5" t="inlineStr"/>
+      <c r="J230" s="5" t="inlineStr"/>
+      <c r="K230" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L230" s="5" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="5" t="inlineStr">
+        <is>
+          <t>TC173</t>
+        </is>
+      </c>
+      <c r="B231" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C231" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D231" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate Item</t>
+        </is>
+      </c>
+      <c r="E231" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate Menu Item</t>
+        </is>
+      </c>
+      <c r="F231" s="5" t="inlineStr">
+        <is>
+          <t>1. Find existing item
+2. Click Duplicate
+3. Modify details
+4. Save as new item</t>
+        </is>
+      </c>
+      <c r="G231" s="5" t="inlineStr">
+        <is>
+          <t>Item duplicated with editable copy</t>
+        </is>
+      </c>
+      <c r="H231" s="5" t="inlineStr"/>
+      <c r="I231" s="5" t="inlineStr"/>
+      <c r="J231" s="5" t="inlineStr"/>
+      <c r="K231" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L231" s="5" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="5" t="inlineStr">
+        <is>
+          <t>TC174</t>
+        </is>
+      </c>
+      <c r="B232" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C232" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D232" s="5" t="inlineStr">
+        <is>
+          <t>Image Crop</t>
+        </is>
+      </c>
+      <c r="E232" s="5" t="inlineStr">
+        <is>
+          <t>Crop Uploaded Image</t>
+        </is>
+      </c>
+      <c r="F232" s="5" t="inlineStr">
+        <is>
+          <t>1. Upload meal photo
+2. Click crop tool
+3. Adjust crop area
+4. Save cropped image</t>
+        </is>
+      </c>
+      <c r="G232" s="5" t="inlineStr">
+        <is>
+          <t>Image cropped and saved correctly</t>
+        </is>
+      </c>
+      <c r="H232" s="5" t="inlineStr"/>
+      <c r="I232" s="5" t="inlineStr"/>
+      <c r="J232" s="5" t="inlineStr"/>
+      <c r="K232" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L232" s="5" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="5" t="inlineStr">
+        <is>
+          <t>TC175</t>
+        </is>
+      </c>
+      <c r="B233" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C233" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D233" s="5" t="inlineStr">
+        <is>
+          <t>Nutrition Calculator</t>
+        </is>
+      </c>
+      <c r="E233" s="5" t="inlineStr">
+        <is>
+          <t>Use Nutrition Calculator</t>
+        </is>
+      </c>
+      <c r="F233" s="5" t="inlineStr">
+        <is>
+          <t>1. Add new meal
+2. Enter ingredients
+3. Use nutrition calculator
+4. Verify auto-calculated values</t>
+        </is>
+      </c>
+      <c r="G233" s="5" t="inlineStr">
+        <is>
+          <t>Nutrition values auto-calculated from ingredients</t>
+        </is>
+      </c>
+      <c r="H233" s="5" t="inlineStr"/>
+      <c r="I233" s="5" t="inlineStr"/>
+      <c r="J233" s="5" t="inlineStr"/>
+      <c r="K233" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L233" s="5" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="5" t="inlineStr">
+        <is>
+          <t>TC176</t>
+        </is>
+      </c>
+      <c r="B234" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C234" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D234" s="5" t="inlineStr">
+        <is>
+          <t>Menu Categories</t>
+        </is>
+      </c>
+      <c r="E234" s="5" t="inlineStr">
+        <is>
+          <t>Organize Menu by Categories</t>
+        </is>
+      </c>
+      <c r="F234" s="5" t="inlineStr">
+        <is>
+          <t>1. Create category (e.g., 'Main Course')
+2. Assign meals to category
+3. View menu by category
+4. Reorder categories</t>
+        </is>
+      </c>
+      <c r="G234" s="5" t="inlineStr">
+        <is>
+          <t>Meals organized by categories</t>
+        </is>
+      </c>
+      <c r="H234" s="5" t="inlineStr"/>
+      <c r="I234" s="5" t="inlineStr"/>
+      <c r="J234" s="5" t="inlineStr"/>
+      <c r="K234" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L234" s="5" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="5" t="inlineStr">
+        <is>
+          <t>TC177</t>
+        </is>
+      </c>
+      <c r="B235" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C235" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D235" s="5" t="inlineStr">
+        <is>
+          <t>Preview Menu</t>
+        </is>
+      </c>
+      <c r="E235" s="5" t="inlineStr">
+        <is>
+          <t>Preview Menu as Customer Sees It</t>
+        </is>
+      </c>
+      <c r="F235" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Preview button
+2. View menu as customer sees it
+3. Verify all items display correctly
+4. Check photos and descriptions</t>
+        </is>
+      </c>
+      <c r="G235" s="5" t="inlineStr">
+        <is>
+          <t>Menu preview matches customer view</t>
+        </is>
+      </c>
+      <c r="H235" s="5" t="inlineStr"/>
+      <c r="I235" s="5" t="inlineStr"/>
+      <c r="J235" s="5" t="inlineStr"/>
+      <c r="K235" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L235" s="5" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="5" t="inlineStr">
+        <is>
+          <t>TC178</t>
+        </is>
+      </c>
+      <c r="B236" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C236" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D236" s="5" t="inlineStr">
+        <is>
+          <t>Export Menu</t>
+        </is>
+      </c>
+      <c r="E236" s="5" t="inlineStr">
+        <is>
+          <t>Export Menu Data</t>
+        </is>
+      </c>
+      <c r="F236" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to menu
+2. Click Export
+3. Select format (CSV/Excel)
+4. Download file</t>
+        </is>
+      </c>
+      <c r="G236" s="5" t="inlineStr">
+        <is>
+          <t>Menu data exported successfully</t>
+        </is>
+      </c>
+      <c r="H236" s="5" t="inlineStr"/>
+      <c r="I236" s="5" t="inlineStr"/>
+      <c r="J236" s="5" t="inlineStr"/>
+      <c r="K236" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L236" s="5" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="5" t="inlineStr">
+        <is>
+          <t>TC179</t>
+        </is>
+      </c>
+      <c r="B237" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C237" s="5" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D237" s="5" t="inlineStr">
+        <is>
+          <t>Import Menu</t>
+        </is>
+      </c>
+      <c r="E237" s="5" t="inlineStr">
+        <is>
+          <t>Import Menu Items</t>
+        </is>
+      </c>
+      <c r="F237" s="5" t="inlineStr">
+        <is>
+          <t>1. Prepare import file
+2. Click Import
+3. Upload file
+4. Map fields
+5. Complete import</t>
+        </is>
+      </c>
+      <c r="G237" s="5" t="inlineStr">
+        <is>
+          <t>Menu items imported successfully</t>
+        </is>
+      </c>
+      <c r="H237" s="5" t="inlineStr"/>
+      <c r="I237" s="5" t="inlineStr"/>
+      <c r="J237" s="5" t="inlineStr"/>
+      <c r="K237" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L237" s="5" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="5" t="inlineStr">
+        <is>
+          <t>TC180</t>
+        </is>
+      </c>
+      <c r="B238" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C238" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D238" s="5" t="inlineStr">
+        <is>
+          <t>Earnings Chart</t>
+        </is>
+      </c>
+      <c r="E238" s="5" t="inlineStr">
+        <is>
+          <t>View Earnings Chart</t>
+        </is>
+      </c>
+      <c r="F238" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to earnings page
+2. View earnings chart
+3. Switch between daily/weekly/monthly views
+4. Hover for detailed values</t>
+        </is>
+      </c>
+      <c r="G238" s="5" t="inlineStr">
+        <is>
+          <t>Chart displays earnings trends accurately</t>
+        </is>
+      </c>
+      <c r="H238" s="5" t="inlineStr"/>
+      <c r="I238" s="5" t="inlineStr"/>
+      <c r="J238" s="5" t="inlineStr"/>
+      <c r="K238" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L238" s="5" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="5" t="inlineStr">
+        <is>
+          <t>TC181</t>
+        </is>
+      </c>
+      <c r="B239" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C239" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D239" s="5" t="inlineStr">
+        <is>
+          <t>Top Meals</t>
+        </is>
+      </c>
+      <c r="E239" s="5" t="inlineStr">
+        <is>
+          <t>View Top Performing Meals</t>
+        </is>
+      </c>
+      <c r="F239" s="5" t="inlineStr">
+        <is>
+          <t>1. Scroll to Top Meals section
+2. View best-selling items
+3. Check quantities sold
+4. View revenue per item</t>
+        </is>
+      </c>
+      <c r="G239" s="5" t="inlineStr">
+        <is>
+          <t>Top performing meals displayed with stats</t>
+        </is>
+      </c>
+      <c r="H239" s="5" t="inlineStr"/>
+      <c r="I239" s="5" t="inlineStr"/>
+      <c r="J239" s="5" t="inlineStr"/>
+      <c r="K239" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L239" s="5" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="5" t="inlineStr">
+        <is>
+          <t>TC182</t>
+        </is>
+      </c>
+      <c r="B240" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C240" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D240" s="5" t="inlineStr">
+        <is>
+          <t>Payout Invoice</t>
+        </is>
+      </c>
+      <c r="E240" s="5" t="inlineStr">
+        <is>
+          <t>Download Payout Invoice</t>
+        </is>
+      </c>
+      <c r="F240" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to payout history
+2. Click on payout
+3. Click Download Invoice
+4. Verify PDF contains correct details</t>
+        </is>
+      </c>
+      <c r="G240" s="5" t="inlineStr">
+        <is>
+          <t>Invoice downloaded with accurate information</t>
+        </is>
+      </c>
+      <c r="H240" s="5" t="inlineStr"/>
+      <c r="I240" s="5" t="inlineStr"/>
+      <c r="J240" s="5" t="inlineStr"/>
+      <c r="K240" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L240" s="5" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="5" t="inlineStr">
+        <is>
+          <t>TC183</t>
+        </is>
+      </c>
+      <c r="B241" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C241" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D241" s="5" t="inlineStr">
+        <is>
+          <t>Dispute Payout</t>
+        </is>
+      </c>
+      <c r="E241" s="5" t="inlineStr">
+        <is>
+          <t>Dispute a Payout</t>
+        </is>
+      </c>
+      <c r="F241" s="5" t="inlineStr">
+        <is>
+          <t>1. Find payout in history
+2. Click Dispute
+3. Enter reason
+4. Submit dispute
+5. Verify confirmation</t>
+        </is>
+      </c>
+      <c r="G241" s="5" t="inlineStr">
+        <is>
+          <t>Dispute submitted, under review status shown</t>
+        </is>
+      </c>
+      <c r="H241" s="5" t="inlineStr"/>
+      <c r="I241" s="5" t="inlineStr"/>
+      <c r="J241" s="5" t="inlineStr"/>
+      <c r="K241" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L241" s="5" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="5" t="inlineStr">
+        <is>
+          <t>TC184</t>
+        </is>
+      </c>
+      <c r="B242" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C242" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D242" s="5" t="inlineStr">
+        <is>
+          <t>Tax Report</t>
+        </is>
+      </c>
+      <c r="E242" s="5" t="inlineStr">
+        <is>
+          <t>Generate Tax Report</t>
+        </is>
+      </c>
+      <c r="F242" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to earnings
+2. Click Tax Report
+3. Select year
+4. Generate report
+5. Download PDF</t>
+        </is>
+      </c>
+      <c r="G242" s="5" t="inlineStr">
+        <is>
+          <t>Tax report generated with all earnings data</t>
+        </is>
+      </c>
+      <c r="H242" s="5" t="inlineStr"/>
+      <c r="I242" s="5" t="inlineStr"/>
+      <c r="J242" s="5" t="inlineStr"/>
+      <c r="K242" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L242" s="5" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="5" t="inlineStr">
+        <is>
+          <t>TC185</t>
+        </is>
+      </c>
+      <c r="B243" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C243" s="5" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="D243" s="5" t="inlineStr">
+        <is>
+          <t>Compare Periods</t>
+        </is>
+      </c>
+      <c r="E243" s="5" t="inlineStr">
+        <is>
+          <t>Compare Earnings Periods</t>
+        </is>
+      </c>
+      <c r="F243" s="5" t="inlineStr">
+        <is>
+          <t>1. Select first period
+2. Select comparison period
+3. View comparison chart
+4. Analyze differences</t>
+        </is>
+      </c>
+      <c r="G243" s="5" t="inlineStr">
+        <is>
+          <t>Period comparison displayed with growth/decline metrics</t>
+        </is>
+      </c>
+      <c r="H243" s="5" t="inlineStr"/>
+      <c r="I243" s="5" t="inlineStr"/>
+      <c r="J243" s="5" t="inlineStr"/>
+      <c r="K243" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L243" s="5" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="5" t="inlineStr">
+        <is>
+          <t>TC186</t>
+        </is>
+      </c>
+      <c r="B244" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C244" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D244" s="5" t="inlineStr">
+        <is>
+          <t>Change Password</t>
+        </is>
+      </c>
+      <c r="E244" s="5" t="inlineStr">
+        <is>
+          <t>Change Account Password</t>
+        </is>
+      </c>
+      <c r="F244" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Click Change Password
+3. Enter current password
+4. Enter new password
+5. Confirm
+6. Logout and test new password</t>
+        </is>
+      </c>
+      <c r="G244" s="5" t="inlineStr">
+        <is>
+          <t>Password changed successfully</t>
+        </is>
+      </c>
+      <c r="H244" s="5" t="inlineStr"/>
+      <c r="I244" s="5" t="inlineStr"/>
+      <c r="J244" s="5" t="inlineStr"/>
+      <c r="K244" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L244" s="5" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="5" t="inlineStr">
+        <is>
+          <t>TC187</t>
+        </is>
+      </c>
+      <c r="B245" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C245" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D245" s="5" t="inlineStr">
+        <is>
+          <t>Two-Factor Auth</t>
+        </is>
+      </c>
+      <c r="E245" s="5" t="inlineStr">
+        <is>
+          <t>Enable Two-Factor Authentication</t>
+        </is>
+      </c>
+      <c r="F245" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to security settings
+2. Enable 2FA
+3. Scan QR code
+4. Enter verification code
+5. Save backup codes</t>
+        </is>
+      </c>
+      <c r="G245" s="5" t="inlineStr">
+        <is>
+          <t>2FA enabled, backup codes provided</t>
+        </is>
+      </c>
+      <c r="H245" s="5" t="inlineStr"/>
+      <c r="I245" s="5" t="inlineStr"/>
+      <c r="J245" s="5" t="inlineStr"/>
+      <c r="K245" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L245" s="5" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="5" t="inlineStr">
+        <is>
+          <t>TC188</t>
+        </is>
+      </c>
+      <c r="B246" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C246" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D246" s="5" t="inlineStr">
+        <is>
+          <t>Notification Preferences</t>
+        </is>
+      </c>
+      <c r="E246" s="5" t="inlineStr">
+        <is>
+          <t>Set Notification Preferences</t>
+        </is>
+      </c>
+      <c r="F246" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Click Notifications
+3. Toggle email notifications
+4. Toggle WhatsApp notifications
+5. Set quiet hours</t>
+        </is>
+      </c>
+      <c r="G246" s="5" t="inlineStr">
+        <is>
+          <t>Notification preferences saved</t>
+        </is>
+      </c>
+      <c r="H246" s="5" t="inlineStr"/>
+      <c r="I246" s="5" t="inlineStr"/>
+      <c r="J246" s="5" t="inlineStr"/>
+      <c r="K246" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L246" s="5" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="5" t="inlineStr">
+        <is>
+          <t>TC189</t>
+        </is>
+      </c>
+      <c r="B247" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C247" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D247" s="5" t="inlineStr">
+        <is>
+          <t>API Access</t>
+        </is>
+      </c>
+      <c r="E247" s="5" t="inlineStr">
+        <is>
+          <t>Generate API Key</t>
+        </is>
+      </c>
+      <c r="F247" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to profile
+2. Click API Access
+3. Generate new key
+4. Copy and save key
+5. View API documentation</t>
+        </is>
+      </c>
+      <c r="G247" s="5" t="inlineStr">
+        <is>
+          <t>API key generated and displayed</t>
+        </is>
+      </c>
+      <c r="H247" s="5" t="inlineStr"/>
+      <c r="I247" s="5" t="inlineStr"/>
+      <c r="J247" s="5" t="inlineStr"/>
+      <c r="K247" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L247" s="5" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="5" t="inlineStr">
+        <is>
+          <t>TC190</t>
+        </is>
+      </c>
+      <c r="B248" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C248" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D248" s="5" t="inlineStr">
+        <is>
+          <t>Business Hours</t>
+        </is>
+      </c>
+      <c r="E248" s="5" t="inlineStr">
+        <is>
+          <t>Set Special Hours</t>
+        </is>
+      </c>
+      <c r="F248" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to operating hours
+2. Set regular hours
+3. Add special hours (holidays)
+4. Mark temporary closures
+5. Save</t>
+        </is>
+      </c>
+      <c r="G248" s="5" t="inlineStr">
+        <is>
+          <t>Special hours saved and applied</t>
+        </is>
+      </c>
+      <c r="H248" s="5" t="inlineStr"/>
+      <c r="I248" s="5" t="inlineStr"/>
+      <c r="J248" s="5" t="inlineStr"/>
+      <c r="K248" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L248" s="5" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="5" t="inlineStr">
+        <is>
+          <t>TC191</t>
+        </is>
+      </c>
+      <c r="B249" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C249" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D249" s="5" t="inlineStr">
+        <is>
+          <t>Delivery Zones</t>
+        </is>
+      </c>
+      <c r="E249" s="5" t="inlineStr">
+        <is>
+          <t>Set Delivery Zones</t>
+        </is>
+      </c>
+      <c r="F249" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to delivery settings
+2. View map
+3. Draw delivery zone
+4. Set minimum order
+5. Set delivery fee
+6. Save</t>
+        </is>
+      </c>
+      <c r="G249" s="5" t="inlineStr">
+        <is>
+          <t>Delivery zone saved and shown on map</t>
+        </is>
+      </c>
+      <c r="H249" s="5" t="inlineStr"/>
+      <c r="I249" s="5" t="inlineStr"/>
+      <c r="J249" s="5" t="inlineStr"/>
+      <c r="K249" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L249" s="5" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="5" t="inlineStr">
+        <is>
+          <t>TC192</t>
+        </is>
+      </c>
+      <c r="B250" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C250" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D250" s="5" t="inlineStr">
+        <is>
+          <t>Team Members</t>
+        </is>
+      </c>
+      <c r="E250" s="5" t="inlineStr">
+        <is>
+          <t>Add Team Members</t>
+        </is>
+      </c>
+      <c r="F250" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to team management
+2. Click Add Member
+3. Enter email
+4. Set role (Admin/Staff)
+5. Send invitation</t>
+        </is>
+      </c>
+      <c r="G250" s="5" t="inlineStr">
+        <is>
+          <t>Invitation sent, member can access with limited permissions</t>
+        </is>
+      </c>
+      <c r="H250" s="5" t="inlineStr"/>
+      <c r="I250" s="5" t="inlineStr"/>
+      <c r="J250" s="5" t="inlineStr"/>
+      <c r="K250" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L250" s="5" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="5" t="inlineStr">
+        <is>
+          <t>TC193</t>
+        </is>
+      </c>
+      <c r="B251" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C251" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="D251" s="5" t="inlineStr">
+        <is>
+          <t>Remove Team Member</t>
+        </is>
+      </c>
+      <c r="E251" s="5" t="inlineStr">
+        <is>
+          <t>Remove Team Member</t>
+        </is>
+      </c>
+      <c r="F251" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to team management
+2. Find member
+3. Click Remove
+4. Confirm removal</t>
+        </is>
+      </c>
+      <c r="G251" s="5" t="inlineStr">
+        <is>
+          <t>Member removed, access revoked</t>
+        </is>
+      </c>
+      <c r="H251" s="5" t="inlineStr"/>
+      <c r="I251" s="5" t="inlineStr"/>
+      <c r="J251" s="5" t="inlineStr"/>
+      <c r="K251" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L251" s="5" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="5" t="inlineStr">
+        <is>
+          <t>TC194</t>
+        </is>
+      </c>
+      <c r="B252" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C252" s="5" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D252" s="5" t="inlineStr">
+        <is>
+          <t>View Analytics</t>
+        </is>
+      </c>
+      <c r="E252" s="5" t="inlineStr">
+        <is>
+          <t>View Business Analytics</t>
+        </is>
+      </c>
+      <c r="F252" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to Analytics page
+2. View order trends
+3. View customer insights
+4. View peak hours
+5. Export analytics report</t>
+        </is>
+      </c>
+      <c r="G252" s="5" t="inlineStr">
+        <is>
+          <t>Analytics displayed with actionable insights</t>
+        </is>
+      </c>
+      <c r="H252" s="5" t="inlineStr"/>
+      <c r="I252" s="5" t="inlineStr"/>
+      <c r="J252" s="5" t="inlineStr"/>
+      <c r="K252" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L252" s="5" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="5" t="inlineStr">
+        <is>
+          <t>TC195</t>
+        </is>
+      </c>
+      <c r="B253" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C253" s="5" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D253" s="5" t="inlineStr">
+        <is>
+          <t>Customer Feedback</t>
+        </is>
+      </c>
+      <c r="E253" s="5" t="inlineStr">
+        <is>
+          <t>View Customer Feedback</t>
+        </is>
+      </c>
+      <c r="F253" s="5" t="inlineStr">
+        <is>
+          <t>1. Go to Reviews section
+2. View all customer reviews
+3. Filter by rating
+4. Respond to review
+5. Mark as resolved</t>
+        </is>
+      </c>
+      <c r="G253" s="5" t="inlineStr">
+        <is>
+          <t>Reviews displayed, can respond to customers</t>
+        </is>
+      </c>
+      <c r="H253" s="5" t="inlineStr"/>
+      <c r="I253" s="5" t="inlineStr"/>
+      <c r="J253" s="5" t="inlineStr"/>
+      <c r="K253" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L253" s="5" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="5" t="inlineStr">
+        <is>
+          <t>TC196</t>
+        </is>
+      </c>
+      <c r="B254" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C254" s="5" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="D254" s="5" t="inlineStr">
+        <is>
+          <t>Performance Metrics</t>
+        </is>
+      </c>
+      <c r="E254" s="5" t="inlineStr">
+        <is>
+          <t>View Detailed Performance Metrics</t>
+        </is>
+      </c>
+      <c r="F254" s="5" t="inlineStr">
+        <is>
+          <t>1. View order fulfillment rate
+2. View average prep time
+3. View on-time delivery rate
+4. Compare with industry average</t>
+        </is>
+      </c>
+      <c r="G254" s="5" t="inlineStr">
+        <is>
+          <t>All performance metrics displayed</t>
+        </is>
+      </c>
+      <c r="H254" s="5" t="inlineStr"/>
+      <c r="I254" s="5" t="inlineStr"/>
+      <c r="J254" s="5" t="inlineStr"/>
+      <c r="K254" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L254" s="5" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="5" t="inlineStr">
+        <is>
+          <t>TC197</t>
+        </is>
+      </c>
+      <c r="B255" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C255" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D255" s="5" t="inlineStr">
+        <is>
+          <t>Contact Support</t>
+        </is>
+      </c>
+      <c r="E255" s="5" t="inlineStr">
+        <is>
+          <t>Contact Support via Dashboard</t>
+        </is>
+      </c>
+      <c r="F255" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Support button
+2. Select issue type
+3. Describe problem
+4. Attach screenshot
+5. Submit ticket</t>
+        </is>
+      </c>
+      <c r="G255" s="5" t="inlineStr">
+        <is>
+          <t>Support ticket created, confirmation shown</t>
+        </is>
+      </c>
+      <c r="H255" s="5" t="inlineStr"/>
+      <c r="I255" s="5" t="inlineStr"/>
+      <c r="J255" s="5" t="inlineStr"/>
+      <c r="K255" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L255" s="5" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="5" t="inlineStr">
+        <is>
+          <t>TC198</t>
+        </is>
+      </c>
+      <c r="B256" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C256" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D256" s="5" t="inlineStr">
+        <is>
+          <t>View Knowledge Base</t>
+        </is>
+      </c>
+      <c r="E256" s="5" t="inlineStr">
+        <is>
+          <t>Access Knowledge Base</t>
+        </is>
+      </c>
+      <c r="F256" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Help
+2. Browse articles
+3. Search for topic
+4. View article</t>
+        </is>
+      </c>
+      <c r="G256" s="5" t="inlineStr">
+        <is>
+          <t>Knowledge base articles displayed</t>
+        </is>
+      </c>
+      <c r="H256" s="5" t="inlineStr"/>
+      <c r="I256" s="5" t="inlineStr"/>
+      <c r="J256" s="5" t="inlineStr"/>
+      <c r="K256" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L256" s="5" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="5" t="inlineStr">
+        <is>
+          <t>TC199</t>
+        </is>
+      </c>
+      <c r="B257" s="5" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C257" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D257" s="5" t="inlineStr">
+        <is>
+          <t>Live Chat</t>
+        </is>
+      </c>
+      <c r="E257" s="5" t="inlineStr">
+        <is>
+          <t>Start Live Chat</t>
+        </is>
+      </c>
+      <c r="F257" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Chat icon
+2. Start conversation
+3. Send message
+4. Receive response</t>
+        </is>
+      </c>
+      <c r="G257" s="5" t="inlineStr">
+        <is>
+          <t>Chat connected, messages exchanged</t>
+        </is>
+      </c>
+      <c r="H257" s="5" t="inlineStr"/>
+      <c r="I257" s="5" t="inlineStr"/>
+      <c r="J257" s="5" t="inlineStr"/>
+      <c r="K257" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L257" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix Status column formulas in all portal tabs - now auto-calculates correctly
</commit_message>
<xml_diff>
--- a/docs/plans/Nutrio-Fuel-E2E-Test-Plan.xlsx
+++ b/docs/plans/Nutrio-Fuel-E2E-Test-Plan.xlsx
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="I2" s="5">
-        <f>IF(I2="","",IF(I2=G2,"PASS","FAIL"))</f>
+        <f>IF(J2="","",IF(J2=H2,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="I3" s="5">
-        <f>IF(I3="","",IF(I3=G3,"PASS","FAIL"))</f>
+        <f>IF(J3="","",IF(J3=H3,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J3" s="5" t="n"/>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="I4" s="5">
-        <f>IF(I4="","",IF(I4=G4,"PASS","FAIL"))</f>
+        <f>IF(J4="","",IF(J4=H4,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="I5" s="5">
-        <f>IF(I5="","",IF(I5=G5,"PASS","FAIL"))</f>
+        <f>IF(J5="","",IF(J5=H5,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="I6" s="5">
-        <f>IF(I6="","",IF(I6=G6,"PASS","FAIL"))</f>
+        <f>IF(J6="","",IF(J6=H6,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="I7" s="5">
-        <f>IF(I7="","",IF(I7=G7,"PASS","FAIL"))</f>
+        <f>IF(J7="","",IF(J7=H7,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="I8" s="5">
-        <f>IF(I8="","",IF(I8=G8,"PASS","FAIL"))</f>
+        <f>IF(J8="","",IF(J8=H8,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="I9" s="5">
-        <f>IF(I9="","",IF(I9=G9,"PASS","FAIL"))</f>
+        <f>IF(J9="","",IF(J9=H9,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J9" s="5" t="n"/>
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="I10" s="5">
-        <f>IF(I10="","",IF(I10=G10,"PASS","FAIL"))</f>
+        <f>IF(J10="","",IF(J10=H10,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J10" s="5" t="n"/>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="I11" s="5">
-        <f>IF(I11="","",IF(I11=G11,"PASS","FAIL"))</f>
+        <f>IF(J11="","",IF(J11=H11,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J11" s="5" t="n"/>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="I12" s="5">
-        <f>IF(I12="","",IF(I12=G12,"PASS","FAIL"))</f>
+        <f>IF(J12="","",IF(J12=H12,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J12" s="5" t="n"/>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="I13" s="5">
-        <f>IF(I13="","",IF(I13=G13,"PASS","FAIL"))</f>
+        <f>IF(J13="","",IF(J13=H13,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J13" s="5" t="n"/>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="I14" s="5">
-        <f>IF(I14="","",IF(I14=G14,"PASS","FAIL"))</f>
+        <f>IF(J14="","",IF(J14=H14,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J14" s="5" t="n"/>
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="I15" s="5">
-        <f>IF(I15="","",IF(I15=G15,"PASS","FAIL"))</f>
+        <f>IF(J15="","",IF(J15=H15,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J15" s="5" t="n"/>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="I16" s="5">
-        <f>IF(I16="","",IF(I16=G16,"PASS","FAIL"))</f>
+        <f>IF(J16="","",IF(J16=H16,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="I17" s="5">
-        <f>IF(I17="","",IF(I17=G17,"PASS","FAIL"))</f>
+        <f>IF(J17="","",IF(J17=H17,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J17" s="5" t="n"/>
@@ -1850,7 +1850,7 @@
         </is>
       </c>
       <c r="I18" s="5">
-        <f>IF(I18="","",IF(I18=G18,"PASS","FAIL"))</f>
+        <f>IF(J18="","",IF(J18=H18,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J18" s="5" t="n"/>
@@ -1906,7 +1906,7 @@
         </is>
       </c>
       <c r="I19" s="5">
-        <f>IF(I19="","",IF(I19=G19,"PASS","FAIL"))</f>
+        <f>IF(J19="","",IF(J19=H19,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J19" s="5" t="n"/>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="I20" s="5">
-        <f>IF(I20="","",IF(I20=G20,"PASS","FAIL"))</f>
+        <f>IF(J20="","",IF(J20=H20,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J20" s="5" t="n"/>
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="I21" s="5">
-        <f>IF(I21="","",IF(I21=G21,"PASS","FAIL"))</f>
+        <f>IF(J21="","",IF(J21=H21,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J21" s="5" t="n"/>
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="I22" s="5">
-        <f>IF(I22="","",IF(I22=G22,"PASS","FAIL"))</f>
+        <f>IF(J22="","",IF(J22=H22,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J22" s="5" t="n"/>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
       <c r="I23" s="5">
-        <f>IF(I23="","",IF(I23=G23,"PASS","FAIL"))</f>
+        <f>IF(J23="","",IF(J23=H23,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J23" s="5" t="n"/>
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="I24" s="5">
-        <f>IF(I24="","",IF(I24=G24,"PASS","FAIL"))</f>
+        <f>IF(J24="","",IF(J24=H24,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J24" s="5" t="n"/>
@@ -2239,7 +2239,7 @@
         </is>
       </c>
       <c r="I25" s="5">
-        <f>IF(I25="","",IF(I25=G25,"PASS","FAIL"))</f>
+        <f>IF(J25="","",IF(J25=H25,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J25" s="5" t="n"/>
@@ -2294,7 +2294,7 @@
         </is>
       </c>
       <c r="I26" s="5">
-        <f>IF(I26="","",IF(I26=G26,"PASS","FAIL"))</f>
+        <f>IF(J26="","",IF(J26=H26,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J26" s="5" t="n"/>
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="I27" s="5">
-        <f>IF(I27="","",IF(I27=G27,"PASS","FAIL"))</f>
+        <f>IF(J27="","",IF(J27=H27,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J27" s="5" t="n"/>
@@ -2405,7 +2405,7 @@
         </is>
       </c>
       <c r="I28" s="5">
-        <f>IF(I28="","",IF(I28=G28,"PASS","FAIL"))</f>
+        <f>IF(J28="","",IF(J28=H28,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J28" s="5" t="n"/>
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="I29" s="5">
-        <f>IF(I29="","",IF(I29=G29,"PASS","FAIL"))</f>
+        <f>IF(J29="","",IF(J29=H29,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J29" s="5" t="n"/>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="I30" s="5">
-        <f>IF(I30="","",IF(I30=G30,"PASS","FAIL"))</f>
+        <f>IF(J30="","",IF(J30=H30,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J30" s="5" t="n"/>
@@ -2572,7 +2572,7 @@
         </is>
       </c>
       <c r="I31" s="5">
-        <f>IF(I31="","",IF(I31=G31,"PASS","FAIL"))</f>
+        <f>IF(J31="","",IF(J31=H31,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J31" s="5" t="n"/>
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="I32" s="5">
-        <f>IF(I32="","",IF(I32=G32,"PASS","FAIL"))</f>
+        <f>IF(J32="","",IF(J32=H32,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J32" s="5" t="n"/>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="I33" s="5">
-        <f>IF(I33="","",IF(I33=G33,"PASS","FAIL"))</f>
+        <f>IF(J33="","",IF(J33=H33,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J33" s="5" t="n"/>
@@ -2738,7 +2738,7 @@
         </is>
       </c>
       <c r="I34" s="5">
-        <f>IF(I34="","",IF(I34=G34,"PASS","FAIL"))</f>
+        <f>IF(J34="","",IF(J34=H34,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J34" s="5" t="n"/>
@@ -2795,7 +2795,7 @@
         </is>
       </c>
       <c r="I35" s="5">
-        <f>IF(I35="","",IF(I35=G35,"PASS","FAIL"))</f>
+        <f>IF(J35="","",IF(J35=H35,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J35" s="5" t="n"/>
@@ -2851,7 +2851,7 @@
         </is>
       </c>
       <c r="I36" s="5">
-        <f>IF(I36="","",IF(I36=G36,"PASS","FAIL"))</f>
+        <f>IF(J36="","",IF(J36=H36,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J36" s="5" t="n"/>
@@ -2906,7 +2906,7 @@
         </is>
       </c>
       <c r="I37" s="5">
-        <f>IF(I37="","",IF(I37=G37,"PASS","FAIL"))</f>
+        <f>IF(J37="","",IF(J37=H37,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J37" s="5" t="n"/>
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="I38" s="5">
-        <f>IF(I38="","",IF(I38=G38,"PASS","FAIL"))</f>
+        <f>IF(J38="","",IF(J38=H38,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J38" s="5" t="n"/>
@@ -3020,7 +3020,7 @@
         </is>
       </c>
       <c r="I39" s="5">
-        <f>IF(I39="","",IF(I39=G39,"PASS","FAIL"))</f>
+        <f>IF(J39="","",IF(J39=H39,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J39" s="5" t="n"/>
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="I40" s="5">
-        <f>IF(I40="","",IF(I40=G40,"PASS","FAIL"))</f>
+        <f>IF(J40="","",IF(J40=H40,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J40" s="5" t="n"/>
@@ -3134,7 +3134,7 @@
         </is>
       </c>
       <c r="I41" s="5">
-        <f>IF(I41="","",IF(I41=G41,"PASS","FAIL"))</f>
+        <f>IF(J41="","",IF(J41=H41,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J41" s="5" t="n"/>
@@ -3189,7 +3189,7 @@
         </is>
       </c>
       <c r="I42" s="5">
-        <f>IF(I42="","",IF(I42=G42,"PASS","FAIL"))</f>
+        <f>IF(J42="","",IF(J42=H42,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J42" s="5" t="n"/>
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="I43" s="5">
-        <f>IF(I43="","",IF(I43=G43,"PASS","FAIL"))</f>
+        <f>IF(J43="","",IF(J43=H43,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J43" s="5" t="n"/>
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="I44" s="5">
-        <f>IF(I44="","",IF(I44=G44,"PASS","FAIL"))</f>
+        <f>IF(J44="","",IF(J44=H44,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J44" s="5" t="n"/>
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="I45" s="5">
-        <f>IF(I45="","",IF(I45=G45,"PASS","FAIL"))</f>
+        <f>IF(J45="","",IF(J45=H45,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J45" s="5" t="n"/>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="I46" s="5">
-        <f>IF(I46="","",IF(I46=G46,"PASS","FAIL"))</f>
+        <f>IF(J46="","",IF(J46=H46,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J46" s="5" t="n"/>
@@ -3468,7 +3468,7 @@
         </is>
       </c>
       <c r="I47" s="5">
-        <f>IF(I47="","",IF(I47=G47,"PASS","FAIL"))</f>
+        <f>IF(J47="","",IF(J47=H47,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J47" s="5" t="n"/>
@@ -3526,7 +3526,7 @@
         </is>
       </c>
       <c r="I48" s="5">
-        <f>IF(I48="","",IF(I48=G48,"PASS","FAIL"))</f>
+        <f>IF(J48="","",IF(J48=H48,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J48" s="5" t="n"/>
@@ -3582,7 +3582,7 @@
         </is>
       </c>
       <c r="I49" s="5">
-        <f>IF(I49="","",IF(I49=G49,"PASS","FAIL"))</f>
+        <f>IF(J49="","",IF(J49=H49,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J49" s="5" t="n"/>
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="I50" s="5">
-        <f>IF(I50="","",IF(I50=G50,"PASS","FAIL"))</f>
+        <f>IF(J50="","",IF(J50=H50,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J50" s="5" t="n"/>
@@ -3695,7 +3695,7 @@
         </is>
       </c>
       <c r="I51" s="5">
-        <f>IF(I51="","",IF(I51=G51,"PASS","FAIL"))</f>
+        <f>IF(J51="","",IF(J51=H51,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J51" s="5" t="n"/>
@@ -3752,7 +3752,7 @@
         </is>
       </c>
       <c r="I52" s="5">
-        <f>IF(I52="","",IF(I52=G52,"PASS","FAIL"))</f>
+        <f>IF(J52="","",IF(J52=H52,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J52" s="5" t="n"/>
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="I53" s="5">
-        <f>IF(I53="","",IF(I53=G53,"PASS","FAIL"))</f>
+        <f>IF(J53="","",IF(J53=H53,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J53" s="5" t="n"/>
@@ -3866,7 +3866,7 @@
         </is>
       </c>
       <c r="I54" s="5">
-        <f>IF(I54="","",IF(I54=G54,"PASS","FAIL"))</f>
+        <f>IF(J54="","",IF(J54=H54,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J54" s="5" t="n"/>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="I55" s="5">
-        <f>IF(I55="","",IF(I55=G55,"PASS","FAIL"))</f>
+        <f>IF(J55="","",IF(J55=H55,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J55" s="5" t="n"/>
@@ -3979,7 +3979,7 @@
         </is>
       </c>
       <c r="I56" s="5">
-        <f>IF(I56="","",IF(I56=G56,"PASS","FAIL"))</f>
+        <f>IF(J56="","",IF(J56=H56,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J56" s="5" t="n"/>
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="I57" s="5">
-        <f>IF(I57="","",IF(I57=G57,"PASS","FAIL"))</f>
+        <f>IF(J57="","",IF(J57=H57,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J57" s="5" t="n"/>
@@ -4094,7 +4094,7 @@
         </is>
       </c>
       <c r="I58" s="5">
-        <f>IF(I58="","",IF(I58=G58,"PASS","FAIL"))</f>
+        <f>IF(J58="","",IF(J58=H58,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J58" s="5" t="n"/>
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="I59" s="5">
-        <f>IF(I59="","",IF(I59=G59,"PASS","FAIL"))</f>
+        <f>IF(J59="","",IF(J59=H59,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J59" s="5" t="n"/>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="I60" s="5">
-        <f>IF(I60="","",IF(I60=G60,"PASS","FAIL"))</f>
+        <f>IF(J60="","",IF(J60=H60,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J60" s="5" t="n"/>
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="I61" s="5">
-        <f>IF(I61="","",IF(I61=G61,"PASS","FAIL"))</f>
+        <f>IF(J61="","",IF(J61=H61,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J61" s="5" t="n"/>
@@ -4322,7 +4322,7 @@
         </is>
       </c>
       <c r="I62" s="5">
-        <f>IF(I62="","",IF(I62=G62,"PASS","FAIL"))</f>
+        <f>IF(J62="","",IF(J62=H62,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J62" s="5" t="n"/>
@@ -4378,7 +4378,7 @@
         </is>
       </c>
       <c r="I63" s="5">
-        <f>IF(I63="","",IF(I63=G63,"PASS","FAIL"))</f>
+        <f>IF(J63="","",IF(J63=H63,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J63" s="5" t="n"/>
@@ -4435,7 +4435,7 @@
         </is>
       </c>
       <c r="I64" s="5">
-        <f>IF(I64="","",IF(I64=G64,"PASS","FAIL"))</f>
+        <f>IF(J64="","",IF(J64=H64,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J64" s="5" t="n"/>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="I65" s="5">
-        <f>IF(I65="","",IF(I65=G65,"PASS","FAIL"))</f>
+        <f>IF(J65="","",IF(J65=H65,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J65" s="5" t="n"/>
@@ -4549,7 +4549,7 @@
         </is>
       </c>
       <c r="I66" s="5">
-        <f>IF(I66="","",IF(I66=G66,"PASS","FAIL"))</f>
+        <f>IF(J66="","",IF(J66=H66,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J66" s="5" t="n"/>
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="I67" s="5">
-        <f>IF(I67="","",IF(I67=G67,"PASS","FAIL"))</f>
+        <f>IF(J67="","",IF(J67=H67,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J67" s="5" t="n"/>
@@ -4663,7 +4663,7 @@
         </is>
       </c>
       <c r="I68" s="5">
-        <f>IF(I68="","",IF(I68=G68,"PASS","FAIL"))</f>
+        <f>IF(J68="","",IF(J68=H68,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J68" s="5" t="n"/>
@@ -4720,7 +4720,7 @@
         </is>
       </c>
       <c r="I69" s="5">
-        <f>IF(I69="","",IF(I69=G69,"PASS","FAIL"))</f>
+        <f>IF(J69="","",IF(J69=H69,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J69" s="5" t="n"/>
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="I70" s="5">
-        <f>IF(I70="","",IF(I70=G70,"PASS","FAIL"))</f>
+        <f>IF(J70="","",IF(J70=H70,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J70" s="5" t="n"/>
@@ -4834,7 +4834,7 @@
         </is>
       </c>
       <c r="I71" s="5">
-        <f>IF(I71="","",IF(I71=G71,"PASS","FAIL"))</f>
+        <f>IF(J71="","",IF(J71=H71,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J71" s="5" t="n"/>
@@ -4891,7 +4891,7 @@
         </is>
       </c>
       <c r="I72" s="5">
-        <f>IF(I72="","",IF(I72=G72,"PASS","FAIL"))</f>
+        <f>IF(J72="","",IF(J72=H72,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J72" s="5" t="n"/>
@@ -4949,7 +4949,7 @@
         </is>
       </c>
       <c r="I73" s="5">
-        <f>IF(I73="","",IF(I73=G73,"PASS","FAIL"))</f>
+        <f>IF(J73="","",IF(J73=H73,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J73" s="5" t="n"/>
@@ -5006,7 +5006,7 @@
         </is>
       </c>
       <c r="I74" s="5">
-        <f>IF(I74="","",IF(I74=G74,"PASS","FAIL"))</f>
+        <f>IF(J74="","",IF(J74=H74,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J74" s="5" t="n"/>
@@ -5063,7 +5063,7 @@
         </is>
       </c>
       <c r="I75" s="5">
-        <f>IF(I75="","",IF(I75=G75,"PASS","FAIL"))</f>
+        <f>IF(J75="","",IF(J75=H75,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J75" s="5" t="n"/>
@@ -5120,7 +5120,7 @@
         </is>
       </c>
       <c r="I76" s="5">
-        <f>IF(I76="","",IF(I76=G76,"PASS","FAIL"))</f>
+        <f>IF(J76="","",IF(J76=H76,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J76" s="5" t="n"/>
@@ -5138,6 +5138,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I77">
+        <f>IF(J77="","",IF(J77=H77,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="13" t="inlineStr">
@@ -5150,6 +5154,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I78">
+        <f>IF(J78="","",IF(J78=H78,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5165,6 +5173,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I79">
+        <f>IF(J79="","",IF(J79=H79,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5181,6 +5193,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I80">
+        <f>IF(J80="","",IF(J80=H80,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5197,6 +5213,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I81">
+        <f>IF(J81="","",IF(J81=H81,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5212,6 +5232,10 @@
         <is>
           <t>https://your-domain.com/</t>
         </is>
+      </c>
+      <c r="I82">
+        <f>IF(J82="","",IF(J82=H82,"PASS","FAIL"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -5437,7 +5461,7 @@
         </is>
       </c>
       <c r="I2" s="5">
-        <f>IF(I2="","",IF(I2=G2,"PASS","FAIL"))</f>
+        <f>IF(J2="","",IF(J2=H2,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -5492,7 +5516,7 @@
         </is>
       </c>
       <c r="I3" s="5">
-        <f>IF(I3="","",IF(I3=G3,"PASS","FAIL"))</f>
+        <f>IF(J3="","",IF(J3=H3,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J3" s="5" t="n"/>
@@ -5547,7 +5571,7 @@
         </is>
       </c>
       <c r="I4" s="5">
-        <f>IF(I4="","",IF(I4=G4,"PASS","FAIL"))</f>
+        <f>IF(J4="","",IF(J4=H4,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -5602,7 +5626,7 @@
         </is>
       </c>
       <c r="I5" s="5">
-        <f>IF(I5="","",IF(I5=G5,"PASS","FAIL"))</f>
+        <f>IF(J5="","",IF(J5=H5,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -5657,7 +5681,7 @@
         </is>
       </c>
       <c r="I6" s="5">
-        <f>IF(I6="","",IF(I6=G6,"PASS","FAIL"))</f>
+        <f>IF(J6="","",IF(J6=H6,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -5713,7 +5737,7 @@
         </is>
       </c>
       <c r="I7" s="5">
-        <f>IF(I7="","",IF(I7=G7,"PASS","FAIL"))</f>
+        <f>IF(J7="","",IF(J7=H7,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -5768,7 +5792,7 @@
         </is>
       </c>
       <c r="I8" s="5">
-        <f>IF(I8="","",IF(I8=G8,"PASS","FAIL"))</f>
+        <f>IF(J8="","",IF(J8=H8,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -5823,7 +5847,7 @@
         </is>
       </c>
       <c r="I9" s="5">
-        <f>IF(I9="","",IF(I9=G9,"PASS","FAIL"))</f>
+        <f>IF(J9="","",IF(J9=H9,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J9" s="5" t="n"/>
@@ -5879,7 +5903,7 @@
         </is>
       </c>
       <c r="I10" s="5">
-        <f>IF(I10="","",IF(I10=G10,"PASS","FAIL"))</f>
+        <f>IF(J10="","",IF(J10=H10,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J10" s="5" t="n"/>
@@ -5935,7 +5959,7 @@
         </is>
       </c>
       <c r="I11" s="5">
-        <f>IF(I11="","",IF(I11=G11,"PASS","FAIL"))</f>
+        <f>IF(J11="","",IF(J11=H11,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J11" s="5" t="n"/>
@@ -5990,7 +6014,7 @@
         </is>
       </c>
       <c r="I12" s="5">
-        <f>IF(I12="","",IF(I12=G12,"PASS","FAIL"))</f>
+        <f>IF(J12="","",IF(J12=H12,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J12" s="5" t="n"/>
@@ -6045,7 +6069,7 @@
         </is>
       </c>
       <c r="I13" s="5">
-        <f>IF(I13="","",IF(I13=G13,"PASS","FAIL"))</f>
+        <f>IF(J13="","",IF(J13=H13,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J13" s="5" t="n"/>
@@ -6100,7 +6124,7 @@
         </is>
       </c>
       <c r="I14" s="5">
-        <f>IF(I14="","",IF(I14=G14,"PASS","FAIL"))</f>
+        <f>IF(J14="","",IF(J14=H14,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J14" s="5" t="n"/>
@@ -6156,7 +6180,7 @@
         </is>
       </c>
       <c r="I15" s="5">
-        <f>IF(I15="","",IF(I15=G15,"PASS","FAIL"))</f>
+        <f>IF(J15="","",IF(J15=H15,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J15" s="5" t="n"/>
@@ -6213,7 +6237,7 @@
         </is>
       </c>
       <c r="I16" s="5">
-        <f>IF(I16="","",IF(I16=G16,"PASS","FAIL"))</f>
+        <f>IF(J16="","",IF(J16=H16,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -6269,7 +6293,7 @@
         </is>
       </c>
       <c r="I17" s="5">
-        <f>IF(I17="","",IF(I17=G17,"PASS","FAIL"))</f>
+        <f>IF(J17="","",IF(J17=H17,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J17" s="5" t="n"/>
@@ -6325,7 +6349,7 @@
         </is>
       </c>
       <c r="I18" s="5">
-        <f>IF(I18="","",IF(I18=G18,"PASS","FAIL"))</f>
+        <f>IF(J18="","",IF(J18=H18,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J18" s="5" t="n"/>
@@ -6382,7 +6406,7 @@
         </is>
       </c>
       <c r="I19" s="5">
-        <f>IF(I19="","",IF(I19=G19,"PASS","FAIL"))</f>
+        <f>IF(J19="","",IF(J19=H19,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J19" s="5" t="n"/>
@@ -6438,7 +6462,7 @@
         </is>
       </c>
       <c r="I20" s="5">
-        <f>IF(I20="","",IF(I20=G20,"PASS","FAIL"))</f>
+        <f>IF(J20="","",IF(J20=H20,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J20" s="5" t="n"/>
@@ -6493,7 +6517,7 @@
         </is>
       </c>
       <c r="I21" s="5">
-        <f>IF(I21="","",IF(I21=G21,"PASS","FAIL"))</f>
+        <f>IF(J21="","",IF(J21=H21,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J21" s="5" t="n"/>
@@ -6548,7 +6572,7 @@
         </is>
       </c>
       <c r="I22" s="5">
-        <f>IF(I22="","",IF(I22=G22,"PASS","FAIL"))</f>
+        <f>IF(J22="","",IF(J22=H22,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J22" s="5" t="n"/>
@@ -6603,7 +6627,7 @@
         </is>
       </c>
       <c r="I23" s="5">
-        <f>IF(I23="","",IF(I23=G23,"PASS","FAIL"))</f>
+        <f>IF(J23="","",IF(J23=H23,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J23" s="5" t="n"/>
@@ -6658,7 +6682,7 @@
         </is>
       </c>
       <c r="I24" s="5">
-        <f>IF(I24="","",IF(I24=G24,"PASS","FAIL"))</f>
+        <f>IF(J24="","",IF(J24=H24,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J24" s="5" t="n"/>
@@ -6713,7 +6737,7 @@
         </is>
       </c>
       <c r="I25" s="5">
-        <f>IF(I25="","",IF(I25=G25,"PASS","FAIL"))</f>
+        <f>IF(J25="","",IF(J25=H25,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J25" s="5" t="n"/>
@@ -6769,7 +6793,7 @@
         </is>
       </c>
       <c r="I26" s="5">
-        <f>IF(I26="","",IF(I26=G26,"PASS","FAIL"))</f>
+        <f>IF(J26="","",IF(J26=H26,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J26" s="5" t="n"/>
@@ -6825,7 +6849,7 @@
         </is>
       </c>
       <c r="I27" s="5">
-        <f>IF(I27="","",IF(I27=G27,"PASS","FAIL"))</f>
+        <f>IF(J27="","",IF(J27=H27,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J27" s="5" t="n"/>
@@ -6881,7 +6905,7 @@
         </is>
       </c>
       <c r="I28" s="5">
-        <f>IF(I28="","",IF(I28=G28,"PASS","FAIL"))</f>
+        <f>IF(J28="","",IF(J28=H28,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J28" s="5" t="n"/>
@@ -6937,7 +6961,7 @@
         </is>
       </c>
       <c r="I29" s="5">
-        <f>IF(I29="","",IF(I29=G29,"PASS","FAIL"))</f>
+        <f>IF(J29="","",IF(J29=H29,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J29" s="5" t="n"/>
@@ -6994,7 +7018,7 @@
         </is>
       </c>
       <c r="I30" s="5">
-        <f>IF(I30="","",IF(I30=G30,"PASS","FAIL"))</f>
+        <f>IF(J30="","",IF(J30=H30,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J30" s="5" t="n"/>
@@ -7050,7 +7074,7 @@
         </is>
       </c>
       <c r="I31" s="5">
-        <f>IF(I31="","",IF(I31=G31,"PASS","FAIL"))</f>
+        <f>IF(J31="","",IF(J31=H31,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J31" s="5" t="n"/>
@@ -7108,7 +7132,7 @@
         </is>
       </c>
       <c r="I32" s="5">
-        <f>IF(I32="","",IF(I32=G32,"PASS","FAIL"))</f>
+        <f>IF(J32="","",IF(J32=H32,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J32" s="5" t="n"/>
@@ -7166,7 +7190,7 @@
         </is>
       </c>
       <c r="I33" s="5">
-        <f>IF(I33="","",IF(I33=G33,"PASS","FAIL"))</f>
+        <f>IF(J33="","",IF(J33=H33,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J33" s="5" t="n"/>
@@ -7224,7 +7248,7 @@
         </is>
       </c>
       <c r="I34" s="5">
-        <f>IF(I34="","",IF(I34=G34,"PASS","FAIL"))</f>
+        <f>IF(J34="","",IF(J34=H34,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J34" s="5" t="n"/>
@@ -7281,7 +7305,7 @@
         </is>
       </c>
       <c r="I35" s="5">
-        <f>IF(I35="","",IF(I35=G35,"PASS","FAIL"))</f>
+        <f>IF(J35="","",IF(J35=H35,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J35" s="5" t="n"/>
@@ -7338,7 +7362,7 @@
         </is>
       </c>
       <c r="I36" s="5">
-        <f>IF(I36="","",IF(I36=G36,"PASS","FAIL"))</f>
+        <f>IF(J36="","",IF(J36=H36,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J36" s="5" t="n"/>
@@ -7395,7 +7419,7 @@
         </is>
       </c>
       <c r="I37" s="5">
-        <f>IF(I37="","",IF(I37=G37,"PASS","FAIL"))</f>
+        <f>IF(J37="","",IF(J37=H37,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J37" s="5" t="n"/>
@@ -7453,7 +7477,7 @@
         </is>
       </c>
       <c r="I38" s="5">
-        <f>IF(I38="","",IF(I38=G38,"PASS","FAIL"))</f>
+        <f>IF(J38="","",IF(J38=H38,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J38" s="5" t="n"/>
@@ -7510,7 +7534,7 @@
         </is>
       </c>
       <c r="I39" s="5">
-        <f>IF(I39="","",IF(I39=G39,"PASS","FAIL"))</f>
+        <f>IF(J39="","",IF(J39=H39,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J39" s="5" t="n"/>
@@ -7567,7 +7591,7 @@
         </is>
       </c>
       <c r="I40" s="5">
-        <f>IF(I40="","",IF(I40=G40,"PASS","FAIL"))</f>
+        <f>IF(J40="","",IF(J40=H40,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J40" s="5" t="n"/>
@@ -7623,7 +7647,7 @@
         </is>
       </c>
       <c r="I41" s="5">
-        <f>IF(I41="","",IF(I41=G41,"PASS","FAIL"))</f>
+        <f>IF(J41="","",IF(J41=H41,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J41" s="5" t="n"/>
@@ -7681,7 +7705,7 @@
         </is>
       </c>
       <c r="I42" s="5">
-        <f>IF(I42="","",IF(I42=G42,"PASS","FAIL"))</f>
+        <f>IF(J42="","",IF(J42=H42,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J42" s="5" t="n"/>
@@ -7738,7 +7762,7 @@
         </is>
       </c>
       <c r="I43" s="5">
-        <f>IF(I43="","",IF(I43=G43,"PASS","FAIL"))</f>
+        <f>IF(J43="","",IF(J43=H43,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J43" s="5" t="n"/>
@@ -7795,7 +7819,7 @@
         </is>
       </c>
       <c r="I44" s="5">
-        <f>IF(I44="","",IF(I44=G44,"PASS","FAIL"))</f>
+        <f>IF(J44="","",IF(J44=H44,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J44" s="5" t="n"/>
@@ -7851,7 +7875,7 @@
         </is>
       </c>
       <c r="I45" s="5">
-        <f>IF(I45="","",IF(I45=G45,"PASS","FAIL"))</f>
+        <f>IF(J45="","",IF(J45=H45,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J45" s="5" t="n"/>
@@ -7908,7 +7932,7 @@
         </is>
       </c>
       <c r="I46" s="5">
-        <f>IF(I46="","",IF(I46=G46,"PASS","FAIL"))</f>
+        <f>IF(J46="","",IF(J46=H46,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J46" s="5" t="n"/>
@@ -7965,7 +7989,7 @@
         </is>
       </c>
       <c r="I47" s="5">
-        <f>IF(I47="","",IF(I47=G47,"PASS","FAIL"))</f>
+        <f>IF(J47="","",IF(J47=H47,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J47" s="5" t="n"/>
@@ -8022,7 +8046,7 @@
         </is>
       </c>
       <c r="I48" s="5">
-        <f>IF(I48="","",IF(I48=G48,"PASS","FAIL"))</f>
+        <f>IF(J48="","",IF(J48=H48,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J48" s="5" t="n"/>
@@ -8079,7 +8103,7 @@
         </is>
       </c>
       <c r="I49" s="5">
-        <f>IF(I49="","",IF(I49=G49,"PASS","FAIL"))</f>
+        <f>IF(J49="","",IF(J49=H49,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J49" s="5" t="n"/>
@@ -8136,7 +8160,7 @@
         </is>
       </c>
       <c r="I50" s="5">
-        <f>IF(I50="","",IF(I50=G50,"PASS","FAIL"))</f>
+        <f>IF(J50="","",IF(J50=H50,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J50" s="5" t="n"/>
@@ -8192,7 +8216,7 @@
         </is>
       </c>
       <c r="I51" s="5">
-        <f>IF(I51="","",IF(I51=G51,"PASS","FAIL"))</f>
+        <f>IF(J51="","",IF(J51=H51,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J51" s="5" t="n"/>
@@ -8249,7 +8273,7 @@
         </is>
       </c>
       <c r="I52" s="5">
-        <f>IF(I52="","",IF(I52=G52,"PASS","FAIL"))</f>
+        <f>IF(J52="","",IF(J52=H52,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J52" s="5" t="n"/>
@@ -8306,7 +8330,7 @@
         </is>
       </c>
       <c r="I53" s="5">
-        <f>IF(I53="","",IF(I53=G53,"PASS","FAIL"))</f>
+        <f>IF(J53="","",IF(J53=H53,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J53" s="5" t="n"/>
@@ -8363,7 +8387,7 @@
         </is>
       </c>
       <c r="I54" s="5">
-        <f>IF(I54="","",IF(I54=G54,"PASS","FAIL"))</f>
+        <f>IF(J54="","",IF(J54=H54,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J54" s="5" t="n"/>
@@ -8420,7 +8444,7 @@
         </is>
       </c>
       <c r="I55" s="5">
-        <f>IF(I55="","",IF(I55=G55,"PASS","FAIL"))</f>
+        <f>IF(J55="","",IF(J55=H55,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J55" s="5" t="n"/>
@@ -8477,7 +8501,7 @@
         </is>
       </c>
       <c r="I56" s="5">
-        <f>IF(I56="","",IF(I56=G56,"PASS","FAIL"))</f>
+        <f>IF(J56="","",IF(J56=H56,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J56" s="5" t="n"/>
@@ -8534,7 +8558,7 @@
         </is>
       </c>
       <c r="I57" s="5">
-        <f>IF(I57="","",IF(I57=G57,"PASS","FAIL"))</f>
+        <f>IF(J57="","",IF(J57=H57,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J57" s="5" t="n"/>
@@ -8592,7 +8616,7 @@
         </is>
       </c>
       <c r="I58" s="5">
-        <f>IF(I58="","",IF(I58=G58,"PASS","FAIL"))</f>
+        <f>IF(J58="","",IF(J58=H58,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J58" s="5" t="n"/>
@@ -8649,7 +8673,7 @@
         </is>
       </c>
       <c r="I59" s="5">
-        <f>IF(I59="","",IF(I59=G59,"PASS","FAIL"))</f>
+        <f>IF(J59="","",IF(J59=H59,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J59" s="5" t="n"/>
@@ -8706,7 +8730,7 @@
         </is>
       </c>
       <c r="I60" s="5">
-        <f>IF(I60="","",IF(I60=G60,"PASS","FAIL"))</f>
+        <f>IF(J60="","",IF(J60=H60,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J60" s="5" t="n"/>
@@ -8763,7 +8787,7 @@
         </is>
       </c>
       <c r="I61" s="5">
-        <f>IF(I61="","",IF(I61=G61,"PASS","FAIL"))</f>
+        <f>IF(J61="","",IF(J61=H61,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J61" s="5" t="n"/>
@@ -8821,7 +8845,7 @@
         </is>
       </c>
       <c r="I62" s="5">
-        <f>IF(I62="","",IF(I62=G62,"PASS","FAIL"))</f>
+        <f>IF(J62="","",IF(J62=H62,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J62" s="5" t="n"/>
@@ -8879,7 +8903,7 @@
         </is>
       </c>
       <c r="I63" s="5">
-        <f>IF(I63="","",IF(I63=G63,"PASS","FAIL"))</f>
+        <f>IF(J63="","",IF(J63=H63,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J63" s="5" t="n"/>
@@ -8936,7 +8960,7 @@
         </is>
       </c>
       <c r="I64" s="5">
-        <f>IF(I64="","",IF(I64=G64,"PASS","FAIL"))</f>
+        <f>IF(J64="","",IF(J64=H64,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J64" s="5" t="n"/>
@@ -8995,7 +9019,7 @@
         </is>
       </c>
       <c r="I65" s="5">
-        <f>IF(I65="","",IF(I65=G65,"PASS","FAIL"))</f>
+        <f>IF(J65="","",IF(J65=H65,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J65" s="5" t="n"/>
@@ -9053,7 +9077,7 @@
         </is>
       </c>
       <c r="I66" s="5">
-        <f>IF(I66="","",IF(I66=G66,"PASS","FAIL"))</f>
+        <f>IF(J66="","",IF(J66=H66,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J66" s="5" t="n"/>
@@ -9111,7 +9135,7 @@
         </is>
       </c>
       <c r="I67" s="5">
-        <f>IF(I67="","",IF(I67=G67,"PASS","FAIL"))</f>
+        <f>IF(J67="","",IF(J67=H67,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J67" s="5" t="n"/>
@@ -9169,7 +9193,7 @@
         </is>
       </c>
       <c r="I68" s="5">
-        <f>IF(I68="","",IF(I68=G68,"PASS","FAIL"))</f>
+        <f>IF(J68="","",IF(J68=H68,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J68" s="5" t="n"/>
@@ -9227,7 +9251,7 @@
         </is>
       </c>
       <c r="I69" s="5">
-        <f>IF(I69="","",IF(I69=G69,"PASS","FAIL"))</f>
+        <f>IF(J69="","",IF(J69=H69,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J69" s="5" t="n"/>
@@ -9286,7 +9310,7 @@
         </is>
       </c>
       <c r="I70" s="5">
-        <f>IF(I70="","",IF(I70=G70,"PASS","FAIL"))</f>
+        <f>IF(J70="","",IF(J70=H70,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J70" s="5" t="n"/>
@@ -9344,7 +9368,7 @@
         </is>
       </c>
       <c r="I71" s="5">
-        <f>IF(I71="","",IF(I71=G71,"PASS","FAIL"))</f>
+        <f>IF(J71="","",IF(J71=H71,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J71" s="5" t="n"/>
@@ -9401,7 +9425,7 @@
         </is>
       </c>
       <c r="I72" s="5">
-        <f>IF(I72="","",IF(I72=G72,"PASS","FAIL"))</f>
+        <f>IF(J72="","",IF(J72=H72,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J72" s="5" t="n"/>
@@ -9459,7 +9483,7 @@
         </is>
       </c>
       <c r="I73" s="5">
-        <f>IF(I73="","",IF(I73=G73,"PASS","FAIL"))</f>
+        <f>IF(J73="","",IF(J73=H73,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J73" s="5" t="n"/>
@@ -9517,7 +9541,7 @@
         </is>
       </c>
       <c r="I74" s="5">
-        <f>IF(I74="","",IF(I74=G74,"PASS","FAIL"))</f>
+        <f>IF(J74="","",IF(J74=H74,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J74" s="5" t="n"/>
@@ -9574,7 +9598,7 @@
         </is>
       </c>
       <c r="I75" s="5">
-        <f>IF(I75="","",IF(I75=G75,"PASS","FAIL"))</f>
+        <f>IF(J75="","",IF(J75=H75,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J75" s="5" t="n"/>
@@ -9632,7 +9656,7 @@
         </is>
       </c>
       <c r="I76" s="5">
-        <f>IF(I76="","",IF(I76=G76,"PASS","FAIL"))</f>
+        <f>IF(J76="","",IF(J76=H76,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J76" s="5" t="n"/>
@@ -9689,7 +9713,7 @@
         </is>
       </c>
       <c r="I77" s="5">
-        <f>IF(I77="","",IF(I77=G77,"PASS","FAIL"))</f>
+        <f>IF(J77="","",IF(J77=H77,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J77" s="5" t="n"/>
@@ -9746,7 +9770,7 @@
         </is>
       </c>
       <c r="I78" s="5">
-        <f>IF(I78="","",IF(I78=G78,"PASS","FAIL"))</f>
+        <f>IF(J78="","",IF(J78=H78,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J78" s="5" t="n"/>
@@ -9804,7 +9828,7 @@
         </is>
       </c>
       <c r="I79" s="5">
-        <f>IF(I79="","",IF(I79=G79,"PASS","FAIL"))</f>
+        <f>IF(J79="","",IF(J79=H79,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J79" s="5" t="n"/>
@@ -9862,7 +9886,7 @@
         </is>
       </c>
       <c r="I80" s="5">
-        <f>IF(I80="","",IF(I80=G80,"PASS","FAIL"))</f>
+        <f>IF(J80="","",IF(J80=H80,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J80" s="5" t="n"/>
@@ -9920,7 +9944,7 @@
         </is>
       </c>
       <c r="I81" s="5">
-        <f>IF(I81="","",IF(I81=G81,"PASS","FAIL"))</f>
+        <f>IF(J81="","",IF(J81=H81,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J81" s="5" t="n"/>
@@ -9977,7 +10001,7 @@
         </is>
       </c>
       <c r="I82" s="5">
-        <f>IF(I82="","",IF(I82=G82,"PASS","FAIL"))</f>
+        <f>IF(J82="","",IF(J82=H82,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J82" s="5" t="n"/>
@@ -10034,7 +10058,7 @@
         </is>
       </c>
       <c r="I83" s="5">
-        <f>IF(I83="","",IF(I83=G83,"PASS","FAIL"))</f>
+        <f>IF(J83="","",IF(J83=H83,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J83" s="5" t="n"/>
@@ -10091,7 +10115,7 @@
         </is>
       </c>
       <c r="I84" s="5">
-        <f>IF(I84="","",IF(I84=G84,"PASS","FAIL"))</f>
+        <f>IF(J84="","",IF(J84=H84,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J84" s="5" t="n"/>
@@ -10149,7 +10173,7 @@
         </is>
       </c>
       <c r="I85" s="5">
-        <f>IF(I85="","",IF(I85=G85,"PASS","FAIL"))</f>
+        <f>IF(J85="","",IF(J85=H85,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J85" s="5" t="n"/>
@@ -10206,7 +10230,7 @@
         </is>
       </c>
       <c r="I86" s="5">
-        <f>IF(I86="","",IF(I86=G86,"PASS","FAIL"))</f>
+        <f>IF(J86="","",IF(J86=H86,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J86" s="5" t="n"/>
@@ -10263,7 +10287,7 @@
         </is>
       </c>
       <c r="I87" s="5">
-        <f>IF(I87="","",IF(I87=G87,"PASS","FAIL"))</f>
+        <f>IF(J87="","",IF(J87=H87,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J87" s="5" t="n"/>
@@ -10319,7 +10343,7 @@
         </is>
       </c>
       <c r="I88" s="5">
-        <f>IF(I88="","",IF(I88=G88,"PASS","FAIL"))</f>
+        <f>IF(J88="","",IF(J88=H88,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J88" s="5" t="n"/>
@@ -10377,7 +10401,7 @@
         </is>
       </c>
       <c r="I89" s="5">
-        <f>IF(I89="","",IF(I89=G89,"PASS","FAIL"))</f>
+        <f>IF(J89="","",IF(J89=H89,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J89" s="5" t="n"/>
@@ -10434,7 +10458,7 @@
         </is>
       </c>
       <c r="I90" s="5">
-        <f>IF(I90="","",IF(I90=G90,"PASS","FAIL"))</f>
+        <f>IF(J90="","",IF(J90=H90,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J90" s="5" t="n"/>
@@ -10491,7 +10515,7 @@
         </is>
       </c>
       <c r="I91" s="5">
-        <f>IF(I91="","",IF(I91=G91,"PASS","FAIL"))</f>
+        <f>IF(J91="","",IF(J91=H91,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J91" s="5" t="n"/>
@@ -10547,7 +10571,7 @@
         </is>
       </c>
       <c r="I92" s="5">
-        <f>IF(I92="","",IF(I92=G92,"PASS","FAIL"))</f>
+        <f>IF(J92="","",IF(J92=H92,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J92" s="5" t="n"/>
@@ -10604,7 +10628,7 @@
         </is>
       </c>
       <c r="I93" s="5">
-        <f>IF(I93="","",IF(I93=G93,"PASS","FAIL"))</f>
+        <f>IF(J93="","",IF(J93=H93,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J93" s="5" t="n"/>
@@ -10661,7 +10685,7 @@
         </is>
       </c>
       <c r="I94" s="5">
-        <f>IF(I94="","",IF(I94=G94,"PASS","FAIL"))</f>
+        <f>IF(J94="","",IF(J94=H94,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J94" s="5" t="n"/>
@@ -10718,7 +10742,7 @@
         </is>
       </c>
       <c r="I95" s="5">
-        <f>IF(I95="","",IF(I95=G95,"PASS","FAIL"))</f>
+        <f>IF(J95="","",IF(J95=H95,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J95" s="5" t="n"/>
@@ -10775,7 +10799,7 @@
         </is>
       </c>
       <c r="I96" s="5">
-        <f>IF(I96="","",IF(I96=G96,"PASS","FAIL"))</f>
+        <f>IF(J96="","",IF(J96=H96,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J96" s="5" t="n"/>
@@ -10832,7 +10856,7 @@
         </is>
       </c>
       <c r="I97" s="5">
-        <f>IF(I97="","",IF(I97=G97,"PASS","FAIL"))</f>
+        <f>IF(J97="","",IF(J97=H97,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J97" s="5" t="n"/>
@@ -10888,7 +10912,7 @@
         </is>
       </c>
       <c r="I98" s="5">
-        <f>IF(I98="","",IF(I98=G98,"PASS","FAIL"))</f>
+        <f>IF(J98="","",IF(J98=H98,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J98" s="5" t="n"/>
@@ -10945,7 +10969,7 @@
         </is>
       </c>
       <c r="I99" s="5">
-        <f>IF(I99="","",IF(I99=G99,"PASS","FAIL"))</f>
+        <f>IF(J99="","",IF(J99=H99,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J99" s="5" t="n"/>
@@ -11002,7 +11026,7 @@
         </is>
       </c>
       <c r="I100" s="5">
-        <f>IF(I100="","",IF(I100=G100,"PASS","FAIL"))</f>
+        <f>IF(J100="","",IF(J100=H100,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J100" s="5" t="n"/>
@@ -11059,7 +11083,7 @@
         </is>
       </c>
       <c r="I101" s="5">
-        <f>IF(I101="","",IF(I101=G101,"PASS","FAIL"))</f>
+        <f>IF(J101="","",IF(J101=H101,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J101" s="5" t="n"/>
@@ -11116,7 +11140,7 @@
         </is>
       </c>
       <c r="I102" s="5">
-        <f>IF(I102="","",IF(I102=G102,"PASS","FAIL"))</f>
+        <f>IF(J102="","",IF(J102=H102,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J102" s="5" t="n"/>
@@ -11173,7 +11197,7 @@
         </is>
       </c>
       <c r="I103" s="5">
-        <f>IF(I103="","",IF(I103=G103,"PASS","FAIL"))</f>
+        <f>IF(J103="","",IF(J103=H103,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J103" s="5" t="n"/>
@@ -11230,7 +11254,7 @@
         </is>
       </c>
       <c r="I104" s="5">
-        <f>IF(I104="","",IF(I104=G104,"PASS","FAIL"))</f>
+        <f>IF(J104="","",IF(J104=H104,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J104" s="5" t="n"/>
@@ -11288,7 +11312,7 @@
         </is>
       </c>
       <c r="I105" s="5">
-        <f>IF(I105="","",IF(I105=G105,"PASS","FAIL"))</f>
+        <f>IF(J105="","",IF(J105=H105,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J105" s="5" t="n"/>
@@ -11345,7 +11369,7 @@
         </is>
       </c>
       <c r="I106" s="5">
-        <f>IF(I106="","",IF(I106=G106,"PASS","FAIL"))</f>
+        <f>IF(J106="","",IF(J106=H106,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J106" s="5" t="n"/>
@@ -11402,7 +11426,7 @@
         </is>
       </c>
       <c r="I107" s="5">
-        <f>IF(I107="","",IF(I107=G107,"PASS","FAIL"))</f>
+        <f>IF(J107="","",IF(J107=H107,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J107" s="5" t="n"/>
@@ -11459,7 +11483,7 @@
         </is>
       </c>
       <c r="I108" s="5">
-        <f>IF(I108="","",IF(I108=G108,"PASS","FAIL"))</f>
+        <f>IF(J108="","",IF(J108=H108,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J108" s="5" t="n"/>
@@ -11517,7 +11541,7 @@
         </is>
       </c>
       <c r="I109" s="5">
-        <f>IF(I109="","",IF(I109=G109,"PASS","FAIL"))</f>
+        <f>IF(J109="","",IF(J109=H109,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J109" s="5" t="n"/>
@@ -11575,7 +11599,7 @@
         </is>
       </c>
       <c r="I110" s="5">
-        <f>IF(I110="","",IF(I110=G110,"PASS","FAIL"))</f>
+        <f>IF(J110="","",IF(J110=H110,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J110" s="5" t="n"/>
@@ -11632,7 +11656,7 @@
         </is>
       </c>
       <c r="I111" s="5">
-        <f>IF(I111="","",IF(I111=G111,"PASS","FAIL"))</f>
+        <f>IF(J111="","",IF(J111=H111,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J111" s="5" t="n"/>
@@ -11691,7 +11715,7 @@
         </is>
       </c>
       <c r="I112" s="5">
-        <f>IF(I112="","",IF(I112=G112,"PASS","FAIL"))</f>
+        <f>IF(J112="","",IF(J112=H112,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J112" s="5" t="n"/>
@@ -11749,7 +11773,7 @@
         </is>
       </c>
       <c r="I113" s="5">
-        <f>IF(I113="","",IF(I113=G113,"PASS","FAIL"))</f>
+        <f>IF(J113="","",IF(J113=H113,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J113" s="5" t="n"/>
@@ -11807,7 +11831,7 @@
         </is>
       </c>
       <c r="I114" s="5">
-        <f>IF(I114="","",IF(I114=G114,"PASS","FAIL"))</f>
+        <f>IF(J114="","",IF(J114=H114,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J114" s="5" t="n"/>
@@ -11865,7 +11889,7 @@
         </is>
       </c>
       <c r="I115" s="5">
-        <f>IF(I115="","",IF(I115=G115,"PASS","FAIL"))</f>
+        <f>IF(J115="","",IF(J115=H115,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J115" s="5" t="n"/>
@@ -11923,7 +11947,7 @@
         </is>
       </c>
       <c r="I116" s="5">
-        <f>IF(I116="","",IF(I116=G116,"PASS","FAIL"))</f>
+        <f>IF(J116="","",IF(J116=H116,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J116" s="5" t="n"/>
@@ -11982,7 +12006,7 @@
         </is>
       </c>
       <c r="I117" s="5">
-        <f>IF(I117="","",IF(I117=G117,"PASS","FAIL"))</f>
+        <f>IF(J117="","",IF(J117=H117,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J117" s="5" t="n"/>
@@ -12040,7 +12064,7 @@
         </is>
       </c>
       <c r="I118" s="5">
-        <f>IF(I118="","",IF(I118=G118,"PASS","FAIL"))</f>
+        <f>IF(J118="","",IF(J118=H118,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J118" s="5" t="n"/>
@@ -12097,7 +12121,7 @@
         </is>
       </c>
       <c r="I119" s="5">
-        <f>IF(I119="","",IF(I119=G119,"PASS","FAIL"))</f>
+        <f>IF(J119="","",IF(J119=H119,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J119" s="5" t="n"/>
@@ -12155,7 +12179,7 @@
         </is>
       </c>
       <c r="I120" s="5">
-        <f>IF(I120="","",IF(I120=G120,"PASS","FAIL"))</f>
+        <f>IF(J120="","",IF(J120=H120,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J120" s="5" t="n"/>
@@ -12213,7 +12237,7 @@
         </is>
       </c>
       <c r="I121" s="5">
-        <f>IF(I121="","",IF(I121=G121,"PASS","FAIL"))</f>
+        <f>IF(J121="","",IF(J121=H121,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J121" s="5" t="n"/>
@@ -12270,7 +12294,7 @@
         </is>
       </c>
       <c r="I122" s="5">
-        <f>IF(I122="","",IF(I122=G122,"PASS","FAIL"))</f>
+        <f>IF(J122="","",IF(J122=H122,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J122" s="5" t="n"/>
@@ -12328,7 +12352,7 @@
         </is>
       </c>
       <c r="I123" s="5">
-        <f>IF(I123="","",IF(I123=G123,"PASS","FAIL"))</f>
+        <f>IF(J123="","",IF(J123=H123,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J123" s="5" t="n"/>
@@ -12385,7 +12409,7 @@
         </is>
       </c>
       <c r="I124" s="5">
-        <f>IF(I124="","",IF(I124=G124,"PASS","FAIL"))</f>
+        <f>IF(J124="","",IF(J124=H124,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J124" s="5" t="n"/>
@@ -12442,7 +12466,7 @@
         </is>
       </c>
       <c r="I125" s="5">
-        <f>IF(I125="","",IF(I125=G125,"PASS","FAIL"))</f>
+        <f>IF(J125="","",IF(J125=H125,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J125" s="5" t="n"/>
@@ -12460,6 +12484,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I126">
+        <f>IF(J126="","",IF(J126=H126,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="13" t="inlineStr">
@@ -12472,6 +12500,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I127">
+        <f>IF(J127="","",IF(J127=H127,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -12487,6 +12519,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I128">
+        <f>IF(J128="","",IF(J128=H128,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -12503,6 +12539,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I129">
+        <f>IF(J129="","",IF(J129=H129,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -12519,6 +12559,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I130">
+        <f>IF(J130="","",IF(J130=H130,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -12534,6 +12578,10 @@
         <is>
           <t>https://your-domain.com/</t>
         </is>
+      </c>
+      <c r="I131">
+        <f>IF(J131="","",IF(J131=H131,"PASS","FAIL"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -12807,7 +12855,7 @@
         </is>
       </c>
       <c r="I2" s="5">
-        <f>IF(I2="","",IF(I2=G2,"PASS","FAIL"))</f>
+        <f>IF(J2="","",IF(J2=H2,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -12862,7 +12910,7 @@
         </is>
       </c>
       <c r="I3" s="5">
-        <f>IF(I3="","",IF(I3=G3,"PASS","FAIL"))</f>
+        <f>IF(J3="","",IF(J3=H3,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J3" s="5" t="n"/>
@@ -12916,7 +12964,7 @@
         </is>
       </c>
       <c r="I4" s="5">
-        <f>IF(I4="","",IF(I4=G4,"PASS","FAIL"))</f>
+        <f>IF(J4="","",IF(J4=H4,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -12971,7 +13019,7 @@
         </is>
       </c>
       <c r="I5" s="5">
-        <f>IF(I5="","",IF(I5=G5,"PASS","FAIL"))</f>
+        <f>IF(J5="","",IF(J5=H5,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -13026,7 +13074,7 @@
         </is>
       </c>
       <c r="I6" s="5">
-        <f>IF(I6="","",IF(I6=G6,"PASS","FAIL"))</f>
+        <f>IF(J6="","",IF(J6=H6,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -13081,7 +13129,7 @@
         </is>
       </c>
       <c r="I7" s="5">
-        <f>IF(I7="","",IF(I7=G7,"PASS","FAIL"))</f>
+        <f>IF(J7="","",IF(J7=H7,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -13135,7 +13183,7 @@
         </is>
       </c>
       <c r="I8" s="5">
-        <f>IF(I8="","",IF(I8=G8,"PASS","FAIL"))</f>
+        <f>IF(J8="","",IF(J8=H8,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -13190,7 +13238,7 @@
         </is>
       </c>
       <c r="I9" s="5">
-        <f>IF(I9="","",IF(I9=G9,"PASS","FAIL"))</f>
+        <f>IF(J9="","",IF(J9=H9,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J9" s="5" t="n"/>
@@ -13245,7 +13293,7 @@
         </is>
       </c>
       <c r="I10" s="5">
-        <f>IF(I10="","",IF(I10=G10,"PASS","FAIL"))</f>
+        <f>IF(J10="","",IF(J10=H10,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J10" s="5" t="n"/>
@@ -13300,7 +13348,7 @@
         </is>
       </c>
       <c r="I11" s="5">
-        <f>IF(I11="","",IF(I11=G11,"PASS","FAIL"))</f>
+        <f>IF(J11="","",IF(J11=H11,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J11" s="5" t="n"/>
@@ -13355,7 +13403,7 @@
         </is>
       </c>
       <c r="I12" s="5">
-        <f>IF(I12="","",IF(I12=G12,"PASS","FAIL"))</f>
+        <f>IF(J12="","",IF(J12=H12,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J12" s="5" t="n"/>
@@ -13410,7 +13458,7 @@
         </is>
       </c>
       <c r="I13" s="5">
-        <f>IF(I13="","",IF(I13=G13,"PASS","FAIL"))</f>
+        <f>IF(J13="","",IF(J13=H13,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J13" s="5" t="n"/>
@@ -13467,7 +13515,7 @@
         </is>
       </c>
       <c r="I14" s="5">
-        <f>IF(I14="","",IF(I14=G14,"PASS","FAIL"))</f>
+        <f>IF(J14="","",IF(J14=H14,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J14" s="5" t="n"/>
@@ -13523,7 +13571,7 @@
         </is>
       </c>
       <c r="I15" s="5">
-        <f>IF(I15="","",IF(I15=G15,"PASS","FAIL"))</f>
+        <f>IF(J15="","",IF(J15=H15,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J15" s="5" t="n"/>
@@ -13579,7 +13627,7 @@
         </is>
       </c>
       <c r="I16" s="5">
-        <f>IF(I16="","",IF(I16=G16,"PASS","FAIL"))</f>
+        <f>IF(J16="","",IF(J16=H16,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -13634,7 +13682,7 @@
         </is>
       </c>
       <c r="I17" s="5">
-        <f>IF(I17="","",IF(I17=G17,"PASS","FAIL"))</f>
+        <f>IF(J17="","",IF(J17=H17,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J17" s="5" t="n"/>
@@ -13689,7 +13737,7 @@
         </is>
       </c>
       <c r="I18" s="5">
-        <f>IF(I18="","",IF(I18=G18,"PASS","FAIL"))</f>
+        <f>IF(J18="","",IF(J18=H18,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J18" s="5" t="n"/>
@@ -13746,7 +13794,7 @@
         </is>
       </c>
       <c r="I19" s="5">
-        <f>IF(I19="","",IF(I19=G19,"PASS","FAIL"))</f>
+        <f>IF(J19="","",IF(J19=H19,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J19" s="5" t="n"/>
@@ -13803,7 +13851,7 @@
         </is>
       </c>
       <c r="I20" s="5">
-        <f>IF(I20="","",IF(I20=G20,"PASS","FAIL"))</f>
+        <f>IF(J20="","",IF(J20=H20,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J20" s="5" t="n"/>
@@ -13858,7 +13906,7 @@
         </is>
       </c>
       <c r="I21" s="5">
-        <f>IF(I21="","",IF(I21=G21,"PASS","FAIL"))</f>
+        <f>IF(J21="","",IF(J21=H21,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J21" s="5" t="n"/>
@@ -13915,7 +13963,7 @@
         </is>
       </c>
       <c r="I22" s="5">
-        <f>IF(I22="","",IF(I22=G22,"PASS","FAIL"))</f>
+        <f>IF(J22="","",IF(J22=H22,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J22" s="5" t="n"/>
@@ -13971,7 +14019,7 @@
         </is>
       </c>
       <c r="I23" s="5">
-        <f>IF(I23="","",IF(I23=G23,"PASS","FAIL"))</f>
+        <f>IF(J23="","",IF(J23=H23,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J23" s="5" t="n"/>
@@ -14028,7 +14076,7 @@
         </is>
       </c>
       <c r="I24" s="5">
-        <f>IF(I24="","",IF(I24=G24,"PASS","FAIL"))</f>
+        <f>IF(J24="","",IF(J24=H24,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J24" s="5" t="n"/>
@@ -14084,7 +14132,7 @@
         </is>
       </c>
       <c r="I25" s="5">
-        <f>IF(I25="","",IF(I25=G25,"PASS","FAIL"))</f>
+        <f>IF(J25="","",IF(J25=H25,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J25" s="5" t="n"/>
@@ -14140,7 +14188,7 @@
         </is>
       </c>
       <c r="I26" s="5">
-        <f>IF(I26="","",IF(I26=G26,"PASS","FAIL"))</f>
+        <f>IF(J26="","",IF(J26=H26,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J26" s="5" t="n"/>
@@ -14195,7 +14243,7 @@
         </is>
       </c>
       <c r="I27" s="5">
-        <f>IF(I27="","",IF(I27=G27,"PASS","FAIL"))</f>
+        <f>IF(J27="","",IF(J27=H27,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J27" s="5" t="n"/>
@@ -14250,7 +14298,7 @@
         </is>
       </c>
       <c r="I28" s="5">
-        <f>IF(I28="","",IF(I28=G28,"PASS","FAIL"))</f>
+        <f>IF(J28="","",IF(J28=H28,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J28" s="5" t="n"/>
@@ -14305,7 +14353,7 @@
         </is>
       </c>
       <c r="I29" s="5">
-        <f>IF(I29="","",IF(I29=G29,"PASS","FAIL"))</f>
+        <f>IF(J29="","",IF(J29=H29,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J29" s="5" t="n"/>
@@ -14360,7 +14408,7 @@
         </is>
       </c>
       <c r="I30" s="5">
-        <f>IF(I30="","",IF(I30=G30,"PASS","FAIL"))</f>
+        <f>IF(J30="","",IF(J30=H30,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J30" s="5" t="n"/>
@@ -14416,7 +14464,7 @@
         </is>
       </c>
       <c r="I31" s="5">
-        <f>IF(I31="","",IF(I31=G31,"PASS","FAIL"))</f>
+        <f>IF(J31="","",IF(J31=H31,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J31" s="5" t="n"/>
@@ -14473,7 +14521,7 @@
         </is>
       </c>
       <c r="I32" s="5">
-        <f>IF(I32="","",IF(I32=G32,"PASS","FAIL"))</f>
+        <f>IF(J32="","",IF(J32=H32,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J32" s="5" t="n"/>
@@ -14530,7 +14578,7 @@
         </is>
       </c>
       <c r="I33" s="5">
-        <f>IF(I33="","",IF(I33=G33,"PASS","FAIL"))</f>
+        <f>IF(J33="","",IF(J33=H33,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J33" s="5" t="n"/>
@@ -14587,7 +14635,7 @@
         </is>
       </c>
       <c r="I34" s="5">
-        <f>IF(I34="","",IF(I34=G34,"PASS","FAIL"))</f>
+        <f>IF(J34="","",IF(J34=H34,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J34" s="5" t="n"/>
@@ -14642,7 +14690,7 @@
         </is>
       </c>
       <c r="I35" s="5">
-        <f>IF(I35="","",IF(I35=G35,"PASS","FAIL"))</f>
+        <f>IF(J35="","",IF(J35=H35,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J35" s="5" t="n"/>
@@ -14697,7 +14745,7 @@
         </is>
       </c>
       <c r="I36" s="5">
-        <f>IF(I36="","",IF(I36=G36,"PASS","FAIL"))</f>
+        <f>IF(J36="","",IF(J36=H36,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J36" s="5" t="n"/>
@@ -14753,7 +14801,7 @@
         </is>
       </c>
       <c r="I37" s="5">
-        <f>IF(I37="","",IF(I37=G37,"PASS","FAIL"))</f>
+        <f>IF(J37="","",IF(J37=H37,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J37" s="5" t="n"/>
@@ -14809,7 +14857,7 @@
         </is>
       </c>
       <c r="I38" s="5">
-        <f>IF(I38="","",IF(I38=G38,"PASS","FAIL"))</f>
+        <f>IF(J38="","",IF(J38=H38,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J38" s="5" t="n"/>
@@ -14865,7 +14913,7 @@
         </is>
       </c>
       <c r="I39" s="5">
-        <f>IF(I39="","",IF(I39=G39,"PASS","FAIL"))</f>
+        <f>IF(J39="","",IF(J39=H39,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J39" s="5" t="n"/>
@@ -14921,7 +14969,7 @@
         </is>
       </c>
       <c r="I40" s="5">
-        <f>IF(I40="","",IF(I40=G40,"PASS","FAIL"))</f>
+        <f>IF(J40="","",IF(J40=H40,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J40" s="5" t="n"/>
@@ -14976,7 +15024,7 @@
         </is>
       </c>
       <c r="I41" s="5">
-        <f>IF(I41="","",IF(I41=G41,"PASS","FAIL"))</f>
+        <f>IF(J41="","",IF(J41=H41,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J41" s="5" t="n"/>
@@ -15033,7 +15081,7 @@
         </is>
       </c>
       <c r="I42" s="5">
-        <f>IF(I42="","",IF(I42=G42,"PASS","FAIL"))</f>
+        <f>IF(J42="","",IF(J42=H42,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J42" s="5" t="n"/>
@@ -15089,7 +15137,7 @@
         </is>
       </c>
       <c r="I43" s="5">
-        <f>IF(I43="","",IF(I43=G43,"PASS","FAIL"))</f>
+        <f>IF(J43="","",IF(J43=H43,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J43" s="5" t="n"/>
@@ -15144,7 +15192,7 @@
         </is>
       </c>
       <c r="I44" s="5">
-        <f>IF(I44="","",IF(I44=G44,"PASS","FAIL"))</f>
+        <f>IF(J44="","",IF(J44=H44,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J44" s="5" t="n"/>
@@ -15200,7 +15248,7 @@
         </is>
       </c>
       <c r="I45" s="5">
-        <f>IF(I45="","",IF(I45=G45,"PASS","FAIL"))</f>
+        <f>IF(J45="","",IF(J45=H45,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J45" s="5" t="n"/>
@@ -15255,7 +15303,7 @@
         </is>
       </c>
       <c r="I46" s="5">
-        <f>IF(I46="","",IF(I46=G46,"PASS","FAIL"))</f>
+        <f>IF(J46="","",IF(J46=H46,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J46" s="5" t="n"/>
@@ -15311,7 +15359,7 @@
         </is>
       </c>
       <c r="I47" s="5">
-        <f>IF(I47="","",IF(I47=G47,"PASS","FAIL"))</f>
+        <f>IF(J47="","",IF(J47=H47,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J47" s="5" t="n"/>
@@ -15368,7 +15416,7 @@
         </is>
       </c>
       <c r="I48" s="5">
-        <f>IF(I48="","",IF(I48=G48,"PASS","FAIL"))</f>
+        <f>IF(J48="","",IF(J48=H48,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J48" s="5" t="n"/>
@@ -15423,7 +15471,7 @@
         </is>
       </c>
       <c r="I49" s="5">
-        <f>IF(I49="","",IF(I49=G49,"PASS","FAIL"))</f>
+        <f>IF(J49="","",IF(J49=H49,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J49" s="5" t="n"/>
@@ -15478,7 +15526,7 @@
         </is>
       </c>
       <c r="I50" s="5">
-        <f>IF(I50="","",IF(I50=G50,"PASS","FAIL"))</f>
+        <f>IF(J50="","",IF(J50=H50,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J50" s="5" t="n"/>
@@ -15534,7 +15582,7 @@
         </is>
       </c>
       <c r="I51" s="5">
-        <f>IF(I51="","",IF(I51=G51,"PASS","FAIL"))</f>
+        <f>IF(J51="","",IF(J51=H51,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J51" s="5" t="n"/>
@@ -15589,7 +15637,7 @@
         </is>
       </c>
       <c r="I52" s="5">
-        <f>IF(I52="","",IF(I52=G52,"PASS","FAIL"))</f>
+        <f>IF(J52="","",IF(J52=H52,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J52" s="5" t="n"/>
@@ -15646,7 +15694,7 @@
         </is>
       </c>
       <c r="I53" s="5">
-        <f>IF(I53="","",IF(I53=G53,"PASS","FAIL"))</f>
+        <f>IF(J53="","",IF(J53=H53,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J53" s="5" t="n"/>
@@ -15702,7 +15750,7 @@
         </is>
       </c>
       <c r="I54" s="5">
-        <f>IF(I54="","",IF(I54=G54,"PASS","FAIL"))</f>
+        <f>IF(J54="","",IF(J54=H54,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J54" s="5" t="n"/>
@@ -15758,7 +15806,7 @@
         </is>
       </c>
       <c r="I55" s="5">
-        <f>IF(I55="","",IF(I55=G55,"PASS","FAIL"))</f>
+        <f>IF(J55="","",IF(J55=H55,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J55" s="5" t="n"/>
@@ -15814,7 +15862,7 @@
         </is>
       </c>
       <c r="I56" s="5">
-        <f>IF(I56="","",IF(I56=G56,"PASS","FAIL"))</f>
+        <f>IF(J56="","",IF(J56=H56,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J56" s="5" t="n"/>
@@ -15870,7 +15918,7 @@
         </is>
       </c>
       <c r="I57" s="5">
-        <f>IF(I57="","",IF(I57=G57,"PASS","FAIL"))</f>
+        <f>IF(J57="","",IF(J57=H57,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J57" s="5" t="n"/>
@@ -15928,7 +15976,7 @@
         </is>
       </c>
       <c r="I58" s="5">
-        <f>IF(I58="","",IF(I58=G58,"PASS","FAIL"))</f>
+        <f>IF(J58="","",IF(J58=H58,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J58" s="5" t="n"/>
@@ -15986,7 +16034,7 @@
         </is>
       </c>
       <c r="I59" s="5">
-        <f>IF(I59="","",IF(I59=G59,"PASS","FAIL"))</f>
+        <f>IF(J59="","",IF(J59=H59,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J59" s="5" t="n"/>
@@ -16044,7 +16092,7 @@
         </is>
       </c>
       <c r="I60" s="5">
-        <f>IF(I60="","",IF(I60=G60,"PASS","FAIL"))</f>
+        <f>IF(J60="","",IF(J60=H60,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J60" s="5" t="n"/>
@@ -16102,7 +16150,7 @@
         </is>
       </c>
       <c r="I61" s="5">
-        <f>IF(I61="","",IF(I61=G61,"PASS","FAIL"))</f>
+        <f>IF(J61="","",IF(J61=H61,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J61" s="5" t="n"/>
@@ -16160,7 +16208,7 @@
         </is>
       </c>
       <c r="I62" s="5">
-        <f>IF(I62="","",IF(I62=G62,"PASS","FAIL"))</f>
+        <f>IF(J62="","",IF(J62=H62,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J62" s="5" t="n"/>
@@ -16218,7 +16266,7 @@
         </is>
       </c>
       <c r="I63" s="5">
-        <f>IF(I63="","",IF(I63=G63,"PASS","FAIL"))</f>
+        <f>IF(J63="","",IF(J63=H63,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J63" s="5" t="n"/>
@@ -16276,7 +16324,7 @@
         </is>
       </c>
       <c r="I64" s="5">
-        <f>IF(I64="","",IF(I64=G64,"PASS","FAIL"))</f>
+        <f>IF(J64="","",IF(J64=H64,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J64" s="5" t="n"/>
@@ -16334,7 +16382,7 @@
         </is>
       </c>
       <c r="I65" s="5">
-        <f>IF(I65="","",IF(I65=G65,"PASS","FAIL"))</f>
+        <f>IF(J65="","",IF(J65=H65,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J65" s="5" t="n"/>
@@ -16392,7 +16440,7 @@
         </is>
       </c>
       <c r="I66" s="5">
-        <f>IF(I66="","",IF(I66=G66,"PASS","FAIL"))</f>
+        <f>IF(J66="","",IF(J66=H66,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J66" s="5" t="n"/>
@@ -16450,7 +16498,7 @@
         </is>
       </c>
       <c r="I67" s="5">
-        <f>IF(I67="","",IF(I67=G67,"PASS","FAIL"))</f>
+        <f>IF(J67="","",IF(J67=H67,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J67" s="5" t="n"/>
@@ -16508,7 +16556,7 @@
         </is>
       </c>
       <c r="I68" s="5">
-        <f>IF(I68="","",IF(I68=G68,"PASS","FAIL"))</f>
+        <f>IF(J68="","",IF(J68=H68,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J68" s="5" t="n"/>
@@ -16566,7 +16614,7 @@
         </is>
       </c>
       <c r="I69" s="5">
-        <f>IF(I69="","",IF(I69=G69,"PASS","FAIL"))</f>
+        <f>IF(J69="","",IF(J69=H69,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J69" s="5" t="n"/>
@@ -16624,7 +16672,7 @@
         </is>
       </c>
       <c r="I70" s="5">
-        <f>IF(I70="","",IF(I70=G70,"PASS","FAIL"))</f>
+        <f>IF(J70="","",IF(J70=H70,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J70" s="5" t="n"/>
@@ -16682,7 +16730,7 @@
         </is>
       </c>
       <c r="I71" s="5">
-        <f>IF(I71="","",IF(I71=G71,"PASS","FAIL"))</f>
+        <f>IF(J71="","",IF(J71=H71,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J71" s="5" t="n"/>
@@ -16740,7 +16788,7 @@
         </is>
       </c>
       <c r="I72" s="5">
-        <f>IF(I72="","",IF(I72=G72,"PASS","FAIL"))</f>
+        <f>IF(J72="","",IF(J72=H72,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J72" s="5" t="n"/>
@@ -16799,7 +16847,7 @@
         </is>
       </c>
       <c r="I73" s="5">
-        <f>IF(I73="","",IF(I73=G73,"PASS","FAIL"))</f>
+        <f>IF(J73="","",IF(J73=H73,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J73" s="5" t="n"/>
@@ -16857,7 +16905,7 @@
         </is>
       </c>
       <c r="I74" s="5">
-        <f>IF(I74="","",IF(I74=G74,"PASS","FAIL"))</f>
+        <f>IF(J74="","",IF(J74=H74,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J74" s="5" t="n"/>
@@ -16915,7 +16963,7 @@
         </is>
       </c>
       <c r="I75" s="5">
-        <f>IF(I75="","",IF(I75=G75,"PASS","FAIL"))</f>
+        <f>IF(J75="","",IF(J75=H75,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J75" s="5" t="n"/>
@@ -16973,7 +17021,7 @@
         </is>
       </c>
       <c r="I76" s="5">
-        <f>IF(I76="","",IF(I76=G76,"PASS","FAIL"))</f>
+        <f>IF(J76="","",IF(J76=H76,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J76" s="5" t="n"/>
@@ -17031,7 +17079,7 @@
         </is>
       </c>
       <c r="I77" s="5">
-        <f>IF(I77="","",IF(I77=G77,"PASS","FAIL"))</f>
+        <f>IF(J77="","",IF(J77=H77,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J77" s="5" t="n"/>
@@ -17089,7 +17137,7 @@
         </is>
       </c>
       <c r="I78" s="5">
-        <f>IF(I78="","",IF(I78=G78,"PASS","FAIL"))</f>
+        <f>IF(J78="","",IF(J78=H78,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J78" s="5" t="n"/>
@@ -17147,7 +17195,7 @@
         </is>
       </c>
       <c r="I79" s="5">
-        <f>IF(I79="","",IF(I79=G79,"PASS","FAIL"))</f>
+        <f>IF(J79="","",IF(J79=H79,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J79" s="5" t="n"/>
@@ -17205,7 +17253,7 @@
         </is>
       </c>
       <c r="I80" s="5">
-        <f>IF(I80="","",IF(I80=G80,"PASS","FAIL"))</f>
+        <f>IF(J80="","",IF(J80=H80,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J80" s="5" t="n"/>
@@ -17263,7 +17311,7 @@
         </is>
       </c>
       <c r="I81" s="5">
-        <f>IF(I81="","",IF(I81=G81,"PASS","FAIL"))</f>
+        <f>IF(J81="","",IF(J81=H81,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J81" s="5" t="n"/>
@@ -17321,7 +17369,7 @@
         </is>
       </c>
       <c r="I82" s="5">
-        <f>IF(I82="","",IF(I82=G82,"PASS","FAIL"))</f>
+        <f>IF(J82="","",IF(J82=H82,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J82" s="5" t="n"/>
@@ -17339,6 +17387,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I83">
+        <f>IF(J83="","",IF(J83=H83,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="13" t="inlineStr">
@@ -17351,6 +17403,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I84">
+        <f>IF(J84="","",IF(J84=H84,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -17366,6 +17422,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I85">
+        <f>IF(J85="","",IF(J85=H85,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -17382,6 +17442,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I86">
+        <f>IF(J86="","",IF(J86=H86,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17398,6 +17462,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I87">
+        <f>IF(J87="","",IF(J87=H87,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -17413,6 +17481,10 @@
         <is>
           <t>https://your-domain.com/</t>
         </is>
+      </c>
+      <c r="I88">
+        <f>IF(J88="","",IF(J88=H88,"PASS","FAIL"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -17643,7 +17715,7 @@
         </is>
       </c>
       <c r="I2" s="5">
-        <f>IF(I2="","",IF(I2=G2,"PASS","FAIL"))</f>
+        <f>IF(J2="","",IF(J2=H2,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -17697,7 +17769,7 @@
         </is>
       </c>
       <c r="I3" s="5">
-        <f>IF(I3="","",IF(I3=G3,"PASS","FAIL"))</f>
+        <f>IF(J3="","",IF(J3=H3,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J3" s="5" t="n"/>
@@ -17752,7 +17824,7 @@
         </is>
       </c>
       <c r="I4" s="5">
-        <f>IF(I4="","",IF(I4=G4,"PASS","FAIL"))</f>
+        <f>IF(J4="","",IF(J4=H4,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -17807,7 +17879,7 @@
         </is>
       </c>
       <c r="I5" s="5">
-        <f>IF(I5="","",IF(I5=G5,"PASS","FAIL"))</f>
+        <f>IF(J5="","",IF(J5=H5,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -17862,7 +17934,7 @@
         </is>
       </c>
       <c r="I6" s="5">
-        <f>IF(I6="","",IF(I6=G6,"PASS","FAIL"))</f>
+        <f>IF(J6="","",IF(J6=H6,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -17918,7 +17990,7 @@
         </is>
       </c>
       <c r="I7" s="5">
-        <f>IF(I7="","",IF(I7=G7,"PASS","FAIL"))</f>
+        <f>IF(J7="","",IF(J7=H7,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -17973,7 +18045,7 @@
         </is>
       </c>
       <c r="I8" s="5">
-        <f>IF(I8="","",IF(I8=G8,"PASS","FAIL"))</f>
+        <f>IF(J8="","",IF(J8=H8,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -18029,7 +18101,7 @@
         </is>
       </c>
       <c r="I9" s="5">
-        <f>IF(I9="","",IF(I9=G9,"PASS","FAIL"))</f>
+        <f>IF(J9="","",IF(J9=H9,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J9" s="5" t="n"/>
@@ -18085,7 +18157,7 @@
         </is>
       </c>
       <c r="I10" s="5">
-        <f>IF(I10="","",IF(I10=G10,"PASS","FAIL"))</f>
+        <f>IF(J10="","",IF(J10=H10,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J10" s="5" t="n"/>
@@ -18140,7 +18212,7 @@
         </is>
       </c>
       <c r="I11" s="5">
-        <f>IF(I11="","",IF(I11=G11,"PASS","FAIL"))</f>
+        <f>IF(J11="","",IF(J11=H11,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J11" s="5" t="n"/>
@@ -18197,7 +18269,7 @@
         </is>
       </c>
       <c r="I12" s="5">
-        <f>IF(I12="","",IF(I12=G12,"PASS","FAIL"))</f>
+        <f>IF(J12="","",IF(J12=H12,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J12" s="5" t="n"/>
@@ -18252,7 +18324,7 @@
         </is>
       </c>
       <c r="I13" s="5">
-        <f>IF(I13="","",IF(I13=G13,"PASS","FAIL"))</f>
+        <f>IF(J13="","",IF(J13=H13,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J13" s="5" t="n"/>
@@ -18307,7 +18379,7 @@
         </is>
       </c>
       <c r="I14" s="5">
-        <f>IF(I14="","",IF(I14=G14,"PASS","FAIL"))</f>
+        <f>IF(J14="","",IF(J14=H14,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J14" s="5" t="n"/>
@@ -18362,7 +18434,7 @@
         </is>
       </c>
       <c r="I15" s="5">
-        <f>IF(I15="","",IF(I15=G15,"PASS","FAIL"))</f>
+        <f>IF(J15="","",IF(J15=H15,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J15" s="5" t="n"/>
@@ -18417,7 +18489,7 @@
         </is>
       </c>
       <c r="I16" s="5">
-        <f>IF(I16="","",IF(I16=G16,"PASS","FAIL"))</f>
+        <f>IF(J16="","",IF(J16=H16,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -18472,7 +18544,7 @@
         </is>
       </c>
       <c r="I17" s="5">
-        <f>IF(I17="","",IF(I17=G17,"PASS","FAIL"))</f>
+        <f>IF(J17="","",IF(J17=H17,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J17" s="5" t="n"/>
@@ -18527,7 +18599,7 @@
         </is>
       </c>
       <c r="I18" s="5">
-        <f>IF(I18="","",IF(I18=G18,"PASS","FAIL"))</f>
+        <f>IF(J18="","",IF(J18=H18,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J18" s="5" t="n"/>
@@ -18583,7 +18655,7 @@
         </is>
       </c>
       <c r="I19" s="5">
-        <f>IF(I19="","",IF(I19=G19,"PASS","FAIL"))</f>
+        <f>IF(J19="","",IF(J19=H19,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J19" s="5" t="n"/>
@@ -18638,7 +18710,7 @@
         </is>
       </c>
       <c r="I20" s="5">
-        <f>IF(I20="","",IF(I20=G20,"PASS","FAIL"))</f>
+        <f>IF(J20="","",IF(J20=H20,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J20" s="5" t="n"/>
@@ -18693,7 +18765,7 @@
         </is>
       </c>
       <c r="I21" s="5">
-        <f>IF(I21="","",IF(I21=G21,"PASS","FAIL"))</f>
+        <f>IF(J21="","",IF(J21=H21,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J21" s="5" t="n"/>
@@ -18748,7 +18820,7 @@
         </is>
       </c>
       <c r="I22" s="5">
-        <f>IF(I22="","",IF(I22=G22,"PASS","FAIL"))</f>
+        <f>IF(J22="","",IF(J22=H22,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J22" s="5" t="n"/>
@@ -18805,7 +18877,7 @@
         </is>
       </c>
       <c r="I23" s="5">
-        <f>IF(I23="","",IF(I23=G23,"PASS","FAIL"))</f>
+        <f>IF(J23="","",IF(J23=H23,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J23" s="5" t="n"/>
@@ -18862,7 +18934,7 @@
         </is>
       </c>
       <c r="I24" s="5">
-        <f>IF(I24="","",IF(I24=G24,"PASS","FAIL"))</f>
+        <f>IF(J24="","",IF(J24=H24,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J24" s="5" t="n"/>
@@ -18919,7 +18991,7 @@
         </is>
       </c>
       <c r="I25" s="5">
-        <f>IF(I25="","",IF(I25=G25,"PASS","FAIL"))</f>
+        <f>IF(J25="","",IF(J25=H25,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J25" s="5" t="n"/>
@@ -18976,7 +19048,7 @@
         </is>
       </c>
       <c r="I26" s="5">
-        <f>IF(I26="","",IF(I26=G26,"PASS","FAIL"))</f>
+        <f>IF(J26="","",IF(J26=H26,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J26" s="5" t="n"/>
@@ -19033,7 +19105,7 @@
         </is>
       </c>
       <c r="I27" s="5">
-        <f>IF(I27="","",IF(I27=G27,"PASS","FAIL"))</f>
+        <f>IF(J27="","",IF(J27=H27,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J27" s="5" t="n"/>
@@ -19090,7 +19162,7 @@
         </is>
       </c>
       <c r="I28" s="5">
-        <f>IF(I28="","",IF(I28=G28,"PASS","FAIL"))</f>
+        <f>IF(J28="","",IF(J28=H28,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J28" s="5" t="n"/>
@@ -19147,7 +19219,7 @@
         </is>
       </c>
       <c r="I29" s="5">
-        <f>IF(I29="","",IF(I29=G29,"PASS","FAIL"))</f>
+        <f>IF(J29="","",IF(J29=H29,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J29" s="5" t="n"/>
@@ -19204,7 +19276,7 @@
         </is>
       </c>
       <c r="I30" s="5">
-        <f>IF(I30="","",IF(I30=G30,"PASS","FAIL"))</f>
+        <f>IF(J30="","",IF(J30=H30,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J30" s="5" t="n"/>
@@ -19261,7 +19333,7 @@
         </is>
       </c>
       <c r="I31" s="5">
-        <f>IF(I31="","",IF(I31=G31,"PASS","FAIL"))</f>
+        <f>IF(J31="","",IF(J31=H31,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J31" s="5" t="n"/>
@@ -19318,7 +19390,7 @@
         </is>
       </c>
       <c r="I32" s="5">
-        <f>IF(I32="","",IF(I32=G32,"PASS","FAIL"))</f>
+        <f>IF(J32="","",IF(J32=H32,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J32" s="5" t="n"/>
@@ -19376,7 +19448,7 @@
         </is>
       </c>
       <c r="I33" s="5">
-        <f>IF(I33="","",IF(I33=G33,"PASS","FAIL"))</f>
+        <f>IF(J33="","",IF(J33=H33,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J33" s="5" t="n"/>
@@ -19434,7 +19506,7 @@
         </is>
       </c>
       <c r="I34" s="5">
-        <f>IF(I34="","",IF(I34=G34,"PASS","FAIL"))</f>
+        <f>IF(J34="","",IF(J34=H34,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J34" s="5" t="n"/>
@@ -19492,7 +19564,7 @@
         </is>
       </c>
       <c r="I35" s="5">
-        <f>IF(I35="","",IF(I35=G35,"PASS","FAIL"))</f>
+        <f>IF(J35="","",IF(J35=H35,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J35" s="5" t="n"/>
@@ -19549,7 +19621,7 @@
         </is>
       </c>
       <c r="I36" s="5">
-        <f>IF(I36="","",IF(I36=G36,"PASS","FAIL"))</f>
+        <f>IF(J36="","",IF(J36=H36,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J36" s="5" t="n"/>
@@ -19607,7 +19679,7 @@
         </is>
       </c>
       <c r="I37" s="5">
-        <f>IF(I37="","",IF(I37=G37,"PASS","FAIL"))</f>
+        <f>IF(J37="","",IF(J37=H37,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J37" s="5" t="n"/>
@@ -19664,7 +19736,7 @@
         </is>
       </c>
       <c r="I38" s="5">
-        <f>IF(I38="","",IF(I38=G38,"PASS","FAIL"))</f>
+        <f>IF(J38="","",IF(J38=H38,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J38" s="5" t="n"/>
@@ -19721,7 +19793,7 @@
         </is>
       </c>
       <c r="I39" s="5">
-        <f>IF(I39="","",IF(I39=G39,"PASS","FAIL"))</f>
+        <f>IF(J39="","",IF(J39=H39,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J39" s="5" t="n"/>
@@ -19780,7 +19852,7 @@
         </is>
       </c>
       <c r="I40" s="5">
-        <f>IF(I40="","",IF(I40=G40,"PASS","FAIL"))</f>
+        <f>IF(J40="","",IF(J40=H40,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J40" s="5" t="n"/>
@@ -19838,7 +19910,7 @@
         </is>
       </c>
       <c r="I41" s="5">
-        <f>IF(I41="","",IF(I41=G41,"PASS","FAIL"))</f>
+        <f>IF(J41="","",IF(J41=H41,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J41" s="5" t="n"/>
@@ -19896,7 +19968,7 @@
         </is>
       </c>
       <c r="I42" s="5">
-        <f>IF(I42="","",IF(I42=G42,"PASS","FAIL"))</f>
+        <f>IF(J42="","",IF(J42=H42,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J42" s="5" t="n"/>
@@ -19953,7 +20025,7 @@
         </is>
       </c>
       <c r="I43" s="5">
-        <f>IF(I43="","",IF(I43=G43,"PASS","FAIL"))</f>
+        <f>IF(J43="","",IF(J43=H43,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J43" s="5" t="n"/>
@@ -20011,7 +20083,7 @@
         </is>
       </c>
       <c r="I44" s="5">
-        <f>IF(I44="","",IF(I44=G44,"PASS","FAIL"))</f>
+        <f>IF(J44="","",IF(J44=H44,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J44" s="5" t="n"/>
@@ -20068,7 +20140,7 @@
         </is>
       </c>
       <c r="I45" s="5">
-        <f>IF(I45="","",IF(I45=G45,"PASS","FAIL"))</f>
+        <f>IF(J45="","",IF(J45=H45,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J45" s="5" t="n"/>
@@ -20086,6 +20158,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I46">
+        <f>IF(J46="","",IF(J46=H46,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
@@ -20098,6 +20174,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I47">
+        <f>IF(J47="","",IF(J47=H47,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -20113,6 +20193,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I48">
+        <f>IF(J48="","",IF(J48=H48,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -20129,6 +20213,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I49">
+        <f>IF(J49="","",IF(J49=H49,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -20145,6 +20233,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I50">
+        <f>IF(J50="","",IF(J50=H50,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -20160,6 +20252,10 @@
         <is>
           <t>https://your-domain.com/</t>
         </is>
+      </c>
+      <c r="I51">
+        <f>IF(J51="","",IF(J51=H51,"PASS","FAIL"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -20352,7 +20448,7 @@
         </is>
       </c>
       <c r="I2" s="5">
-        <f>IF(I2="","",IF(I2=G2,"PASS","FAIL"))</f>
+        <f>IF(J2="","",IF(J2=H2,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J2" s="5" t="n"/>
@@ -20407,7 +20503,7 @@
         </is>
       </c>
       <c r="I3" s="5">
-        <f>IF(I3="","",IF(I3=G3,"PASS","FAIL"))</f>
+        <f>IF(J3="","",IF(J3=H3,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J3" s="5" t="n"/>
@@ -20462,7 +20558,7 @@
         </is>
       </c>
       <c r="I4" s="5">
-        <f>IF(I4="","",IF(I4=G4,"PASS","FAIL"))</f>
+        <f>IF(J4="","",IF(J4=H4,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -20518,7 +20614,7 @@
         </is>
       </c>
       <c r="I5" s="5">
-        <f>IF(I5="","",IF(I5=G5,"PASS","FAIL"))</f>
+        <f>IF(J5="","",IF(J5=H5,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -20573,7 +20669,7 @@
         </is>
       </c>
       <c r="I6" s="5">
-        <f>IF(I6="","",IF(I6=G6,"PASS","FAIL"))</f>
+        <f>IF(J6="","",IF(J6=H6,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -20628,7 +20724,7 @@
         </is>
       </c>
       <c r="I7" s="5">
-        <f>IF(I7="","",IF(I7=G7,"PASS","FAIL"))</f>
+        <f>IF(J7="","",IF(J7=H7,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -20683,7 +20779,7 @@
         </is>
       </c>
       <c r="I8" s="5">
-        <f>IF(I8="","",IF(I8=G8,"PASS","FAIL"))</f>
+        <f>IF(J8="","",IF(J8=H8,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -20738,7 +20834,7 @@
         </is>
       </c>
       <c r="I9" s="5">
-        <f>IF(I9="","",IF(I9=G9,"PASS","FAIL"))</f>
+        <f>IF(J9="","",IF(J9=H9,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J9" s="5" t="n"/>
@@ -20793,7 +20889,7 @@
         </is>
       </c>
       <c r="I10" s="5">
-        <f>IF(I10="","",IF(I10=G10,"PASS","FAIL"))</f>
+        <f>IF(J10="","",IF(J10=H10,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J10" s="5" t="n"/>
@@ -20848,7 +20944,7 @@
         </is>
       </c>
       <c r="I11" s="5">
-        <f>IF(I11="","",IF(I11=G11,"PASS","FAIL"))</f>
+        <f>IF(J11="","",IF(J11=H11,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J11" s="5" t="n"/>
@@ -20906,7 +21002,7 @@
         </is>
       </c>
       <c r="I12" s="5">
-        <f>IF(I12="","",IF(I12=G12,"PASS","FAIL"))</f>
+        <f>IF(J12="","",IF(J12=H12,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J12" s="5" t="n"/>
@@ -20963,7 +21059,7 @@
         </is>
       </c>
       <c r="I13" s="5">
-        <f>IF(I13="","",IF(I13=G13,"PASS","FAIL"))</f>
+        <f>IF(J13="","",IF(J13=H13,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J13" s="5" t="n"/>
@@ -21020,7 +21116,7 @@
         </is>
       </c>
       <c r="I14" s="5">
-        <f>IF(I14="","",IF(I14=G14,"PASS","FAIL"))</f>
+        <f>IF(J14="","",IF(J14=H14,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J14" s="5" t="n"/>
@@ -21078,7 +21174,7 @@
         </is>
       </c>
       <c r="I15" s="5">
-        <f>IF(I15="","",IF(I15=G15,"PASS","FAIL"))</f>
+        <f>IF(J15="","",IF(J15=H15,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J15" s="5" t="n"/>
@@ -21136,7 +21232,7 @@
         </is>
       </c>
       <c r="I16" s="5">
-        <f>IF(I16="","",IF(I16=G16,"PASS","FAIL"))</f>
+        <f>IF(J16="","",IF(J16=H16,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J16" s="5" t="n"/>
@@ -21194,7 +21290,7 @@
         </is>
       </c>
       <c r="I17" s="5">
-        <f>IF(I17="","",IF(I17=G17,"PASS","FAIL"))</f>
+        <f>IF(J17="","",IF(J17=H17,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J17" s="5" t="n"/>
@@ -21252,7 +21348,7 @@
         </is>
       </c>
       <c r="I18" s="5">
-        <f>IF(I18="","",IF(I18=G18,"PASS","FAIL"))</f>
+        <f>IF(J18="","",IF(J18=H18,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J18" s="5" t="n"/>
@@ -21310,7 +21406,7 @@
         </is>
       </c>
       <c r="I19" s="5">
-        <f>IF(I19="","",IF(I19=G19,"PASS","FAIL"))</f>
+        <f>IF(J19="","",IF(J19=H19,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J19" s="5" t="n"/>
@@ -21368,7 +21464,7 @@
         </is>
       </c>
       <c r="I20" s="5">
-        <f>IF(I20="","",IF(I20=G20,"PASS","FAIL"))</f>
+        <f>IF(J20="","",IF(J20=H20,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J20" s="5" t="n"/>
@@ -21426,7 +21522,7 @@
         </is>
       </c>
       <c r="I21" s="5">
-        <f>IF(I21="","",IF(I21=G21,"PASS","FAIL"))</f>
+        <f>IF(J21="","",IF(J21=H21,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J21" s="5" t="n"/>
@@ -21484,7 +21580,7 @@
         </is>
       </c>
       <c r="I22" s="5">
-        <f>IF(I22="","",IF(I22=G22,"PASS","FAIL"))</f>
+        <f>IF(J22="","",IF(J22=H22,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J22" s="5" t="n"/>
@@ -21542,7 +21638,7 @@
         </is>
       </c>
       <c r="I23" s="5">
-        <f>IF(I23="","",IF(I23=G23,"PASS","FAIL"))</f>
+        <f>IF(J23="","",IF(J23=H23,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J23" s="5" t="n"/>
@@ -21600,7 +21696,7 @@
         </is>
       </c>
       <c r="I24" s="5">
-        <f>IF(I24="","",IF(I24=G24,"PASS","FAIL"))</f>
+        <f>IF(J24="","",IF(J24=H24,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J24" s="5" t="n"/>
@@ -21658,7 +21754,7 @@
         </is>
       </c>
       <c r="I25" s="5">
-        <f>IF(I25="","",IF(I25=G25,"PASS","FAIL"))</f>
+        <f>IF(J25="","",IF(J25=H25,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J25" s="5" t="n"/>
@@ -21716,7 +21812,7 @@
         </is>
       </c>
       <c r="I26" s="5">
-        <f>IF(I26="","",IF(I26=G26,"PASS","FAIL"))</f>
+        <f>IF(J26="","",IF(J26=H26,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J26" s="5" t="n"/>
@@ -21774,7 +21870,7 @@
         </is>
       </c>
       <c r="I27" s="5">
-        <f>IF(I27="","",IF(I27=G27,"PASS","FAIL"))</f>
+        <f>IF(J27="","",IF(J27=H27,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J27" s="5" t="n"/>
@@ -21832,7 +21928,7 @@
         </is>
       </c>
       <c r="I28" s="5">
-        <f>IF(I28="","",IF(I28=G28,"PASS","FAIL"))</f>
+        <f>IF(J28="","",IF(J28=H28,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J28" s="5" t="n"/>
@@ -21890,7 +21986,7 @@
         </is>
       </c>
       <c r="I29" s="5">
-        <f>IF(I29="","",IF(I29=G29,"PASS","FAIL"))</f>
+        <f>IF(J29="","",IF(J29=H29,"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="J29" s="5" t="n"/>
@@ -21908,6 +22004,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I30">
+        <f>IF(J30="","",IF(J30=H30,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
@@ -21920,6 +22020,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I31">
+        <f>IF(J31="","",IF(J31=H31,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -21935,6 +22039,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I32">
+        <f>IF(J32="","",IF(J32=H32,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -21951,6 +22059,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I33">
+        <f>IF(J33="","",IF(J33=H33,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -21967,6 +22079,10 @@
           <t>https://your-domain.com/</t>
         </is>
       </c>
+      <c r="I34">
+        <f>IF(J34="","",IF(J34=H34,"PASS","FAIL"))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -21982,6 +22098,10 @@
         <is>
           <t>https://your-domain.com/</t>
         </is>
+      </c>
+      <c r="I35">
+        <f>IF(J35="","",IF(J35=H35,"PASS","FAIL"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>